<commit_message>
Fix DataFrame boolean ambiguity in retry logic
Cannot use 'or' operator with DataFrames (ambiguous truth value)
Use explicit None check instead
</commit_message>
<xml_diff>
--- a/tmp/ground_truth_cleaned.xlsx
+++ b/tmp/ground_truth_cleaned.xlsx
@@ -453,7 +453,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE SUGAR CURED HALF SLAB BACON | BACON SLAB CC SUGAR CURE FRZN</t>
+          <t>OLD SMOKEHOUSE SUGAR CURED HALF SLAB BACON BACON SLAB CC SUGAR CURE FRZN</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 18-22 CT | BACON 18/22 CT LAYOUT APPLEWOOD SMOKED | BACON L/O 18-22CT CC APPLWD SMKD</t>
+          <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 18-22 CT BACON 18/22 CT LAYOUT APPLEWOOD SMOKED BACON L/O 18-22CT CC APPLWD SMKD</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -487,12 +487,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD HALF SLAB BACON | APPLEWOOD SLAB BACON</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD HALF SLAB BACON APPLEWOOD SLAB BACON</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Applewood-smoked half‑slab and slab bacon.</t>
+          <t>Applewood-smoked half-slab bacon</t>
         </is>
       </c>
     </row>
@@ -504,12 +504,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD HALF SLAB BACON | BACON SLAB APWD OLD SMKHS UNSL</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD HALF SLAB BACON BACON SLAB APWD OLD SMKHS UNSL</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Applewood-smoked slab bacon</t>
+          <t>Applewood-smoked half-slab bacon</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 14-18 CT | BACON L/O 14-18CT CC APPLWD SMKD | BACON 14/18 CT L/O APPLEWOOD SMOKED</t>
+          <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 14-18 CT BACON L/O 14-18CT CC APPLWD SMKD BACON 14/18 CT L/O APPLEWOOD SMOKED</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -538,7 +538,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BACON CHERRYWOOD SMOKED SLAB | BACON SLAB CHERRYWOOD SMK</t>
+          <t>BACON CHERRYWOOD SMOKED SLAB BACON SLAB CHERRYWOOD SMK</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -555,7 +555,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD SMOKED 16-20 CT | BACON SLICED APPLEWOOD SMKD | BACON 16/20 CT APPLEWOOD SMOKED SLICED</t>
+          <t>BACON SLICED APPLEWOOD SMOKED 16-20 CT BACON SLICED APPLEWOOD SMKD BACON 16/20 CT APPLEWOOD SMOKED SLICED</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -572,12 +572,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FRZ PRE-CKD BCN SAND STYLE 300 | BACON PRECOOKED SAND STY | BACON PRECOOKED</t>
+          <t>FRZ PRE-CKD BCN SAND STYLE 300 BACON PRECOOKED SAND STY BACON PRECOOKED</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Frozen fully cooked sandwich-style bacon.</t>
+          <t>Frozen fully cooked sandwich-style sliced bacon.</t>
         </is>
       </c>
     </row>
@@ -589,10 +589,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>FRZ PRE-CKD BCN SAND STYLE 300 | BACON SAND STYLE CKD</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>FRZ PRE-CKD BCN SAND STYLE 300 BACON SAND STYLE CKD</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Frozen pre-cooked sliced bacon, sandwich style</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -602,7 +606,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>FRZ PRE-CKD BCN SAND STYLE 300 | BACON  PORK CKD 150 CT SM</t>
+          <t>FRZ PRE-CKD BCN SAND STYLE 300 BACON PORK CKD 150 CT SM</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -615,12 +619,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BACON PIECES COOKED GAS FLUSHED .375 IN | BACON BIT REAL CKD 3/8 GF | BACON BIT REAL COOKED GLUTEN FREE 3/8""</t>
+          <t>BACON PIECES COOKED GAS FLUSHED .375 IN BACON BIT REAL CKD 3/8 GF BACON BIT REAL COOKED GLUTEN FREE 3/8</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cooked gas-flushed gluten-free bacon bits, 3/8‑inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -632,10 +636,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BACON BITS REAL GAS FLUSHED .75 IN | BACON BIT REAL COOKED GLUTEN FREE 3/4"" | BACON BIT REAL CKD 3/4IN GF</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
+          <t>BACON BITS REAL GAS FLUSHED .75 IN BACON BIT REAL COOKED GLUTEN FREE 3/4 BACON BIT REAL CKD 3/4IN GF</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Fully cooked gluten-free bacon bits, 3/4‑inch pieces</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -645,12 +653,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BACON BITS CUBED .375X.375 | BACON 3/8"" PRECOOKED DICED BITS</t>
+          <t>BACON BITS CUBED .375X.375 BACON 3/8 PRECOOKED DICED BITS</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fully cooked diced bacon bits, 3/8‑inch pieces</t>
+          <t>Fully cooked diced bacon bits, 3/8-inch pieces</t>
         </is>
       </c>
     </row>
@@ -662,7 +670,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BACON SLICED SMOKED LAYFLAT 18-22 CT | BACON 18/22 CT LAYFLAT SMOKED | BACON LAYFLAT 18/22 SMOKED</t>
+          <t>BACON SLICED SMOKED LAYFLAT 18-22 CT BACON 18/22 CT LAYFLAT SMOKED BACON LAYFLAT 18/22 SMOKED</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -679,12 +687,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BACN,BITS,FC,FINE,FL,2/5# | SHC BACON BITS FINELY DICED F/C</t>
+          <t>BACN,BITS,FC,FINE,FL,2/5 SHC BACON BITS FINELY DICED F/C</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Fully cooked finely diced bacon bits</t>
+          <t>Fully cooked finely diced bacon bits, 2/5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -696,12 +704,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BCN,PL,SYS-CLC,BITS,2/5#,1/2",FC,DICD,GF | BACON BIT REAL CKD 1/2 GF | BACON BIT REAL COOKED GLUTEN FREE 1/2""</t>
+          <t>BCN,PL,SYS-CLC,BITS,2/5 ,1/2 ,FC,DICD,GF BACON BIT REAL CKD 1/2 GF BACON BIT REAL COOKED GLUTEN FREE 1/2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 1/2-inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 1/2‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -713,12 +721,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BCN,PL,SYS-CLC,FINE,2/5#,FC,GF | BACON BIT REAL COOKED FINE GLUTEN FREE | BACON BIT REAL CKD FINE GF</t>
+          <t>BCN,PL,SYS-CLC,FINE,2/5 ,FC,GF BACON BIT REAL COOKED FINE GLUTEN FREE BACON BIT REAL CKD FINE GF</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free fine bacon bits, 2/5‑inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 2/5-inch pieces</t>
         </is>
       </c>
     </row>
@@ -730,7 +738,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD COOKED 2 DIAMOND | BACON  PORK 150CT SLCD LA</t>
+          <t>BACON SLICED APPLEWOOD COOKED 2 DIAMOND BACON PORK 150CT SLCD LA</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -743,14 +751,10 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BACON SLICED COOKED | BACON  PORK CKD 150 LO NT</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Fully cooked sliced bacon</t>
-        </is>
-      </c>
+          <t>BACON SLICED COOKED BACON PORK CKD 150 LO NT</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -760,12 +764,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BACON SLICED LAYOUT 18-22 CT | BACON  PORK 18-22 SLC LAI</t>
+          <t>BACON SLICED LAYOUT 18-22 CT BACON PORK 18-22 SLC LAI</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced pork bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -777,14 +781,10 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BCN,PL,SYSUP,APLWD,1/15#,10-12C,CSMK,GF | BACON SLI COLD SMK APPLE 10-12 | BACON 10/12 CT SLICED APPLEWOOD COLD SMOKED</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood cold-smoked sliced bacon, 10-12 slices per pound.</t>
-        </is>
-      </c>
+          <t>BCN,PL,SYSUP,APLWD,1/15 ,10-12C,CSMK,GF BACON SLI COLD SMK APPLE 10-12 BACON 10/12 CT SLICED APPLEWOOD COLD SMOKED</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BCN,JM,18/22/SLC,POLY,1/15#,FZ | BACON SINGLE SLICE 18/22</t>
+          <t>BCN,JM,18/22/SLC,POLY,1/15 ,FZ BACON SINGLE SLICE 18/22</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -811,12 +811,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BACN,BITS,FC,SMFD,1/4IN,2/5# | BACON BIT 1/4IN FC | BACON BIT FULLY COOKED 1/4""</t>
+          <t>BACN,BITS,FC,SMFD,1/4IN,2/5 BACON BIT 1/4IN FC BACON BIT FULLY COOKED 1/4</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 1/4-inch pieces</t>
+          <t>Fully cooked bacon bits, 1/4‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -828,14 +828,10 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BCN,GC,2/5#,1/4",TPG,MCRW | BACON TOPPING COOKED 1/4"" | BACON TOPPING CKD</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Fully cooked bacon topping, 1/4-inch pieces</t>
-        </is>
-      </c>
+          <t>BCN,GC,2/5 ,1/4 ,TPG,MCRW BACON TOPPING COOKED 1/4 BACON TOPPING CKD</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -845,7 +841,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BCN,ARM,2/5#,3/4",FLCK,TPG | BACON TOPPING REAL FC 3/4""</t>
+          <t>BCN,ARM,2/5 ,3/4 ,FLCK,TPG BACON TOPPING REAL FC 3/4</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -862,12 +858,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>AWS SLCD BACN 14/18 | BACON 14/18 CT LAYFLAT APPLEWOOD GLUTEN FREE | BACON LAYFLAT 14/18 APPL GF</t>
+          <t>AWS SLCD BACN 14/18 BACON 14/18 CT LAYFLAT APPLEWOOD GLUTEN FREE BACON LAYFLAT 14/18 APPL GF</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 14-18 slices per pound, gluten-free, layflat</t>
+          <t>Applewood-smoked sliced bacon, gluten</t>
         </is>
       </c>
     </row>
@@ -879,12 +875,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BCN,ARM,RDIGRLL,1/15#,FZ,14-18C,RAW | LUNCHMAKER TURKEY W/TREAT</t>
+          <t>BCN,ARM,RDIGRLL,1/15 ,FZ,14-18C,RAW LUNCHMAKER TURKEY W/TREAT</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Frozen raw sliced bacon, 14-18 slices per pound</t>
+          <t>Frozen raw turkey</t>
         </is>
       </c>
     </row>
@@ -896,12 +892,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GFS SLCD BACN 9/11 | BACON SLCD 9-11CT FRSH</t>
+          <t>GFS SLCD BACN 9/11 BACON SLCD 9-11CT FRSH</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fresh gluten-free sliced bacon, 9-11 slices per pound</t>
+          <t>Fresh sliced gluten-free bacon, 9-11 slices per pound</t>
         </is>
       </c>
     </row>
@@ -913,12 +909,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>HORMEL BACON 1 PERFECTLY COOKED 18/22 STYLE BACON | BACON CKD SLCD 18/22</t>
+          <t>HORMEL BACON 1 PERFECTLY COOKED 18/22 STYLE BACON BACON CKD SLCD 18/22</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -930,10 +926,14 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BCN,PL,ORG,APLWD,GHP,1/15#,14-17C,SLC,GF | BACON LAYFLAT APL GHP 14/17 GF</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
+          <t>BCN,PL,ORG,APLWD,GHP,1/15 ,14-17C,SLC,GF BACON LAYFLAT APL GHP 14/17 GF</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Applewood-smoked sliced gluten-free bacon, 14-17 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -943,12 +943,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>JJ THCKR BACON CKD | BACON SLI APPLWD SMKD CKD</t>
+          <t>JJ THCKR BACON CKD BACON SLI APPLWD SMKD CKD</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Cooked thick-cut applewood-smoked sliced bacon</t>
+          <t>Fully cooked thick-cut sliced applewood-smoked bacon</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>BCN,ARM,2/5#,1/2",FLCK,BITS | BACON BITS REAL FC 1/2""</t>
+          <t>BCN,ARM,2/5 ,1/2 ,FLCK,BITS BACON BITS REAL FC 1/2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -977,10 +977,14 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>BCN,ARM,2/5#,1/2",FLCK,BITS | BACON TOPPING CKD 1/2IN DCD</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
+          <t>BCN,ARM,2/5 ,1/2 ,FLCK,BITS BACON TOPPING CKD 1/2IN DCD</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Fully cooked bacon bits, 1/2-inch pieces.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -990,7 +994,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JMYD FC AWS SLCD BACN 4/150 | BACON PRECOOKED APPLWOOD 10 IN</t>
+          <t>JMYD FC AWS SLCD BACN 4/150 BACON PRECOOKED APPLWOOD 10 IN</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1003,12 +1007,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>BACON SLICED LAYOUT BIG BUY 14-20 CT | BACON SLICED BULK BIG 14/20 CT</t>
+          <t>BACON SLICED LAYOUT BIG BUY 14-20 CT BACON SLICED BULK BIG 14/20 CT</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Sliced layflat bacon, 14-20 slices per pound.</t>
+          <t>Sliced bacon, 14-20 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1020,12 +1024,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>HORMEL BACON1 PERFECTLY COOKED BACON HALF SLICES | BACON PRECOOKED BCN 1 576 CT</t>
+          <t>HORMEL BACON1 PERFECTLY COOKED BACON HALF SLICES BACON PRECOOKED BCN 1 576 CT</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Fully cooked half-slice bacon, 576 slices.</t>
+          <t>Fully cooked sliced bacon</t>
         </is>
       </c>
     </row>
@@ -1037,10 +1041,14 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>HORMEL BACON1 PERFECTLY COOKED BACON HALF SLICES | BACON CKD SLCD 18-22 | BACON CKD SLCD 18-22 HLF SLCD</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
+          <t>HORMEL BACON1 PERFECTLY COOKED BACON HALF SLICES BACON CKD SLCD 18-22 BACON CKD SLCD 18-22 HLF SLCD</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1050,7 +1058,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>BCN,PL,ORG,GHP,1/15#,18-22C,SLC,AP | BACON LAYOUT HCK SMK 18/22 GHP</t>
+          <t>BCN,PL,ORG,GHP,1/15 ,18-22C,SLC,AP BACON LAYOUT HCK SMK 18/22 GHP</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1063,7 +1071,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>DI BACN PCE | BACON PCS DCD RAW</t>
+          <t>DI BACN PCE BACON PCS DCD RAW</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1080,7 +1088,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BACON APPLEWOOD SMOKED SLAB | BACON SLAB APPLEWOOD SMKD</t>
+          <t>BACON APPLEWOOD SMOKED SLAB BACON SLAB APPLEWOOD SMKD</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1097,10 +1105,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>BCN,ARM,SS,15#,18/22,GHP,FZ | BACON  PORK 18-22 CT LAID</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
+          <t>BCN,ARM,SS,15 ,18/22,GHP,FZ BACON PORK 18-22 CT LAID</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Frozen sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1110,12 +1122,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>BCN,ARM,SS,15#,18/22,GHP,FZ | SHC BACON HICK SMKD 18/22 LAYOUT</t>
+          <t>BCN,ARM,SS,15 ,18/22,GHP,FZ SHC BACON HICK SMKD 18/22 LAYOUT</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Frozen sliced hickory-smoked bacon, 18-22 slices per pound, layflat</t>
+          <t>Frozen hickory-smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1127,12 +1139,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>BCN,ARM,SS,15#,18/22,GHP,FZ | BACON 18X22 CT APPLEWOOD SMOKED SINGLE SLICED | BACON SINGLE SLI SMK 18/22 GHP</t>
+          <t>BCN,ARM,SS,15 ,18/22,GHP,FZ BACON 18X22 CT APPLEWOOD SMOKED SINGLE SLICED BACON SINGLE SLI SMK 18/22 GHP</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Frozen applewood-smoked sliced bacon, 18-22 slices per pound.</t>
+          <t>Frozen sliced bacon, applewood-smoked, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1144,12 +1156,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>APPLEGATE NATURALS SUNDAY BACON UNCURED FOOD SERVICE | BACON SLI 14/18 NAT NAE P12/Q3</t>
+          <t>APPLEGATE NATURALS SUNDAY BACON UNCURED FOOD SERVICE BACON SLI 14/18 NAT NAE P12/Q3</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Raw uncured sliced bacon, 14-18 slices per pound</t>
+          <t>Uncured sliced bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1173,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>BCN,PL,RNGLN,HKRY,15#,18/22,SS,FZ | LAYOUT BACON 18/22</t>
+          <t>BCN,PL,RNGLN,HKRY,15 ,18/22,SS,FZ LAYOUT BACON 18/22</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1178,7 +1190,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>BCN,PL,RNGLN,HKRY,15#,14/18,SS,FZ | LAYOUT BACON 14/18</t>
+          <t>BCN,PL,RNGLN,HKRY,15 ,14/18,SS,FZ LAYOUT BACON 14/18</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1195,7 +1207,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>NT HKY SMKD BULK BACN 9/INCH FZ | BACON BULK FRZN 9IN</t>
+          <t>NT HKY SMKD BULK BACN 9/INCH FZ BACON BULK FRZN 9IN</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1212,14 +1224,10 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>NT HKY SMKD THK SLCD BULK BACN 5/INCH FZ | BACON BULK SLI THCK HCKRY SMK</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Frozen thick sliced hickory-smoked bacon, 5/8‑inch slices.</t>
-        </is>
-      </c>
+          <t>NT HKY SMKD THK SLCD BULK BACN 5/INCH FZ BACON BULK SLI THCK HCKRY SMK</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1229,14 +1237,10 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>FC DI BACN 2/5 LB | BACON PCS CKD SMKD 3/8IN</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Fully cooked diced bacon, smoked, 3/8‑inch pieces.</t>
-        </is>
-      </c>
+          <t>FC DI BACN 2/5 LB BACON PCS CKD SMKD 3/8IN</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1246,12 +1250,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>NT AWS BACN FPK 14/18, GF | BACON LAYFLAT 14/18 APPL GF</t>
+          <t>NT AWS BACN FPK 14/18, GF BACON LAYFLAT 14/18 APPL GF</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 14-18 slices per pound, gluten‑free, layflat</t>
+          <t>Applewood-smoked gluten-free sliced bacon, 14-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1263,10 +1267,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>FC BACN PCE 3/8" | BACN PCS CKD HRDWD SMKD 3/8IN</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr"/>
+          <t>FC BACN PCE 3/8 BACN PCS CKD HRDWD SMKD 3/8IN</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Fully cooked hardwood-smoked bacon pieces, 3</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1276,7 +1284,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>FC BACN PCE 3/8" | BACON PIECES COOKED</t>
+          <t>FC BACN PCE 3/8 BACON PIECES COOKED</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1293,12 +1301,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>FC HKY SMKD BACN REG SLCD GF | BACON SLCD HICKR SMKD CKD</t>
+          <t>FC HKY SMKD BACN REG SLCD GF BACON SLCD HICKR SMKD CKD</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free sliced hickory-smoked bacon</t>
+          <t>Fully cooked gluten-free hickory-smoked sliced bacon</t>
         </is>
       </c>
     </row>
@@ -1310,12 +1318,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>FC RND BACN 192 CNT | BACON SLI PRCK RND 192 CT</t>
+          <t>FC RND BACN 192 CNT BACON SLI PRCK RND 192 CT</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 192 slices</t>
+          <t>Fully cooked sliced bacon, 192 slices.</t>
         </is>
       </c>
     </row>
@@ -1327,12 +1335,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SYS 1005842 LYFLT 18/22SYSCO CLASSIC CENTER SLICED LAYFLAT BACON, 18/22 15#. | BACON LAYFLAT C/C 18/22 SMOKED</t>
+          <t>SYS 1005842 LYFLT 18/22SYSCO CLASSIC CENTER SLICED LAYFLAT BACON, 18/22 15 . BACON LAYFLAT C/C 18/22 SMOKED</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Raw center-cut sliced smoked bacon, 18-22 slices per pound, layflat</t>
+          <t>Center-cut sliced smoked bacon, 18</t>
         </is>
       </c>
     </row>
@@ -1344,12 +1352,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND GCF | BACON LAYFLAT AW CC 13/17 PR12</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND GCF BACON LAYFLAT AW CC 13/17 PR12</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Raw applewood-smoked sliced bacon, 13-17 slices per pound, gluten-free, layflat.</t>
+          <t>Gluten-free applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1361,12 +1369,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>HORMEL BLACK LABEL BACON 9 13 PIECES PER POUND GCF | BACON SLAB SLI 9/13 CT PR12</t>
+          <t>HORMEL BLACK LABEL BACON 9 13 PIECES PER POUND GCF BACON SLAB SLI 9/13 CT PR12</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sliced slab bacon, 9-13 slices per pound.</t>
+          <t>Sliced slab bacon, 9-13 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1378,14 +1386,10 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED GCF | BACON SLI APLWD 13/17CT PR12</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Raw wide shingled applewood-smoked sliced bacon, 13-17 slices per pound</t>
-        </is>
-      </c>
+          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED GCF BACON SLI APLWD 13/17CT PR12</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1395,7 +1399,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>HORMEL NATURAL CHOICE UNCURED BACON 13 17 SLICES PER POUND GCF | BACON LAYFLAT NT CC 13/17 PR12</t>
+          <t>HORMEL NATURAL CHOICE UNCURED BACON 13 17 SLICES PER POUND GCF BACON LAYFLAT NT CC 13/17 PR12</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1412,7 +1416,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE PECANWOOD SMOKED BACON 9 13 SLICES PER POUND GCF | BACON LAYFLAT PCN CC 9/13 PR12</t>
+          <t>OLD SMOKEHOUSE PECANWOOD SMOKED BACON 9 13 SLICES PER POUND GCF BACON LAYFLAT PCN CC 9/13 PR12</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -1429,14 +1433,10 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND GCF | BACON LAYFLAT CC 18/22 GF PR12</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND GCF BACON LAYFLAT CC 18/22 GF PR12</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1446,12 +1446,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>LAY FLAT BACON 18-22 PLUS | BACON LAYFLT 18/22 PR12/Q3 NA</t>
+          <t>LAY FLAT BACON 18-22 PLUS BACON LAYFLT 18/22 PR12/Q3 NA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Raw sliced layflat bacon, 18-22 slices per pound</t>
+          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1463,12 +1463,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>HOTEL BACON 16/18 PLUS | BACON SHINGLE 16/18 PR12/Q3</t>
+          <t>HOTEL BACON 16/18 PLUS BACON SHINGLE 16/18 PR12/Q3</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Sliced bacon</t>
+          <t>Shingle bacon, 16-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1480,12 +1480,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>BACON 10/12 CT SLICED APPLEWOOD SMOKED FROZEN | BACON SLI APLWD SMK 10-12 FRZN</t>
+          <t>BACON 10/12 CT SLICED APPLEWOOD SMOKED FROZEN BACON SLI APLWD SMK 10-12 FRZN</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Frozen applewood-smoked sliced bacon, 10-12 slices per pound.</t>
+          <t>Frozen sliced applewood-smoked bacon, 10-12 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>LAY FLAT APPLEWOOD BACON 14/18 PLUS | BACON LAYFLT AW 14/18 PR12/NA</t>
+          <t>LAY FLAT APPLEWOOD BACON 14/18 PLUS BACON LAYFLT AW 14/18 PR12/NA</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -1514,12 +1514,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>JMYD FC BACN PCE 1/2 INCH 30 PCT 2/5LB | BACON PCS CKD 1/2IN</t>
+          <t>JMYD FC BACN PCE 1/2 INCH 30 PCT 2/5LB BACON PCS CKD 1/2IN</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Fully cooked bacon pieces, 1/2‑inch pieces</t>
+          <t>Fully cooked 1/2-inch bacon pieces</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>HTF AW LAY FLAT BACON 10-14 | BACON LAYFLAT APLWD 10-14</t>
+          <t>HTF AW LAY FLAT BACON 10-14 BACON LAYFLAT APLWD 10-14</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1548,10 +1548,14 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>BACON APPLEWOOD CUBED .5X.5 | BACON DICED SMKD APLWD</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr"/>
+          <t>BACON APPLEWOOD CUBED .5X.5 BACON DICED SMKD APLWD</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Applewood-smoked cubed bacon, 0.5 × 0.5‑inch pieces.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1561,10 +1565,14 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>BACON BITS REAL GAS FLUSHED .75 IN | BACON BIT REAL CKD 3/4IN GF</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr"/>
+          <t>BACON BITS REAL GAS FLUSHED .75 IN BACON BIT REAL CKD 3/4IN GF</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Fully cooked gluten-free bacon bits, 3/4-inch pieces</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1574,12 +1582,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>BACON PIECES COOKED GAS FLUSHED .375 IN | BACON BIT REAL CKD 3/8 GF | BACON BIT REAL COOKED GLUTEN FREE 3/8""</t>
+          <t>BACON PIECES COOKED GAS FLUSHED .375 IN BACON BIT REAL CKD 3/8 GF BACON BIT REAL COOKED GLUTEN FREE 3/8</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Cooked gas-flushed gluten-free bacon bits, 3/8‑inch pieces</t>
+          <t>Fully cooked gluten-free gas-flushed bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1599,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>BACON BITS REAL GLUTEN FREE .5 IN | BACON BIT REAL CKD 1/2 GF</t>
+          <t>BACON BITS REAL GLUTEN FREE .5 IN BACON BIT REAL CKD 1/2 GF</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -1608,12 +1616,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>BACON BITS FINE REAL GLUTEN FREE | BACON BIT REAL COOKED FINE GLUTEN FREE | BACON BIT REAL CKD FINE GF</t>
+          <t>BACON BITS FINE REAL GLUTEN FREE BACON BIT REAL COOKED FINE GLUTEN FREE BACON BIT REAL CKD FINE GF</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free fine bacon bits.</t>
+          <t>Fully cooked gluten-free fine bacon bits</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1633,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 14-18 CT | BACON 14/18 CT LAYOUT APPLEWOOD | BACON L/O 14-18CT CC APPLWD</t>
+          <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 14-18 CT BACON 14/18 CT LAYOUT APPLEWOOD BACON L/O 14-18CT CC APPLWD</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -1642,14 +1650,10 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>BACON APPLEWOOD SMOKED LAYOUT 18-22 CT | BACON L/O 14-18CT CC APPLWD SMKD</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Applewood-smoked sliced bacon, 14-22 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>BACON APPLEWOOD SMOKED LAYOUT 18-22 CT BACON L/O 14-18CT CC APPLWD SMKD</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1659,7 +1663,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>LAYOUT BACON 18/22 FTR | BACON LAYOUT 18/22</t>
+          <t>LAYOUT BACON 18/22 FTR BACON LAYOUT 18/22</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -1676,7 +1680,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>LAYOUT BACON 18/22 FTR | BACON LAYOUT 18/22</t>
+          <t>LAYOUT BACON 18/22 FTR BACON LAYOUT 18/22</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -1693,12 +1697,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>BACON BITS CUBED .375X.375 | BACON BIT DICED 3/8""</t>
+          <t>BACON BITS CUBED .375X.375 BACON BIT DICED 3/8</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Bacon bits, 3/8-inch pieces</t>
+          <t>Bacon bits, 3/8‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1714,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>BACON L/O 18-22CT DBL SMKD 3-5# GSIG | BACON L/O 18-22CT CC DBL SMKD</t>
+          <t>BACON L/O 18-22CT DBL SMKD 3-5 GSIG BACON L/O 18-22CT CC DBL SMKD</t>
         </is>
       </c>
       <c r="C79" t="inlineStr"/>
@@ -1723,7 +1727,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>BACON THIN FULLY COOKED | BACON CKD THN SLCD</t>
+          <t>BACON THIN FULLY COOKED BACON CKD THN SLCD</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -1757,7 +1761,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>BACON BIT 1/2"" | BACON BIT 1/2IN</t>
+          <t>BACON BIT 1/2 BACON BIT 1/2IN</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -1774,12 +1778,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>BACON BIT COOKED REAL 1/4"" | BACON BIT 1/4IN | BACON BIT 1/4""</t>
+          <t>BACON BIT COOKED REAL 1/4 BACON BIT 1/4IN BACON BIT 1/4</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Fully cooked real bacon bits, 1/4‑inch pieces</t>
+          <t>Fully cooked bacon bits, 1/4-inch pieces</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1795,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>BACON L/O 14-18CT DBL SMKD 3-5# GSIG | BACON L/O 14-18CT CC DBL SMKD</t>
+          <t>BACON L/O 14-18CT DBL SMKD 3-5 GSIG BACON L/O 14-18CT CC DBL SMKD</t>
         </is>
       </c>
       <c r="C84" t="inlineStr"/>
@@ -1804,7 +1808,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>BACON L/O 9-11CT FRSH DBL SMKD 3-5# | BACON L/O 9-11CT CC DBL SMKD</t>
+          <t>BACON L/O 9-11CT FRSH DBL SMKD 3-5 BACON L/O 9-11CT CC DBL SMKD</t>
         </is>
       </c>
       <c r="C85" t="inlineStr"/>
@@ -1817,12 +1821,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>HTF LAY FLAT  BACON 18-22 PLUS STR | BACON 18/22 CT LAYFLAT PR12/Q3 | BACON LAYFLT 18/22 PR12/Q3</t>
+          <t>HTF LAY FLAT BACON 18-22 PLUS STR BACON 18/22 CT LAYFLAT PR12/Q3 BACON LAYFLT 18/22 PR12/Q3</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced layflat bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1834,14 +1838,10 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>8 AWS LFLT SLCD BACN 14/18 PR12 | BACON LAYFLT 14/18 APL GF PR12</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 14-18 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>8 AWS LFLT SLCD BACN 14/18 PR12 BACON LAYFLT 14/18 APL GF PR12</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1851,12 +1851,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>HORMEL FAST N EASY COOKED BACON 300 SLICE PER CASE | BACON CKD</t>
+          <t>HORMEL FAST N EASY COOKED BACON 300 SLICE PER CASE BACON CKD</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 300 slices per case.</t>
+          <t>Fully cooked sliced bacon, 300 slices per case</t>
         </is>
       </c>
     </row>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>HORMEL FAST N EASY COOKED BACON 300 SLICE PER CASE | BACON PRECOOKED SLI  SANDWICH</t>
+          <t>HORMEL FAST N EASY COOKED BACON 300 SLICE PER CASE BACON PRECOOKED SLI SANDWICH</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -1885,12 +1885,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>HORMEL REGULAR COOKED 0 375 INCH BACON TOPPING | BACON TOPPING 3/8IN DCD</t>
+          <t>HORMEL REGULAR COOKED 0 375 INCH BACON TOPPING BACON TOPPING 3/8IN DCD</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Fully cooked 3/8‑inch diced bacon topping</t>
+          <t>Fully cooked sliced bacon topping, 3/8‑inch slices.</t>
         </is>
       </c>
     </row>
@@ -1902,12 +1902,12 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>HORMEL REGULAR COOKED 0 375 INCH BACON TOPPING | BACON TOPPING REG COOKED 3/8</t>
+          <t>HORMEL REGULAR COOKED 0 375 INCH BACON TOPPING BACON TOPPING REG COOKED 3/8</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon topping, 3/8‑inch slices.</t>
+          <t>Fully cooked bacon topping, 3/8-inch pieces</t>
         </is>
       </c>
     </row>
@@ -1919,14 +1919,10 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>HORMEL REGULAR COOKED 0 375 INCH BACON TOPPING | BACON  PORK REAL DCD .38</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>Fully cooked sliced bacon topping, 3/8‑inch slices.</t>
-        </is>
-      </c>
+          <t>HORMEL REGULAR COOKED 0 375 INCH BACON TOPPING BACON PORK REAL DCD .38</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1936,7 +1932,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>HORMEL FAST N EASY BACON COOKED 300 SLICES PER CASE | BACON PRCK SLI FST&amp;EASY REGLR</t>
+          <t>HORMEL FAST N EASY BACON COOKED 300 SLICES PER CASE BACON PRCK SLI FST&amp;EASY REGLR</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -1953,12 +1949,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>HORMEL FAST N EASY BACON COOKED 300 SLICES PER CASE | BACON SLICED PRE-CKD</t>
+          <t>HORMEL FAST N EASY BACON COOKED 300 SLICES PER CASE BACON SLICED PRE-CKD</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon</t>
+          <t>Fully cooked sliced bacon, 300 slices per case</t>
         </is>
       </c>
     </row>
@@ -1970,7 +1966,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>HORMEL FAST N EASY BACON COOKED 300 SLICES PER CASE | BACON CKD FAST'N EASY</t>
+          <t>HORMEL FAST N EASY BACON COOKED 300 SLICES PER CASE BACON CKD FAST N EASY</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -1987,7 +1983,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE ORIGINAL BACON 18 22 SLICES PER POUND | BACON LAYOUT 18/22</t>
+          <t>OLD SMOKEHOUSE ORIGINAL BACON 18 22 SLICES PER POUND BACON LAYOUT 18/22</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -2004,12 +2000,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>HORMEL FAST 'N EASY EXTRA COOKED BACON ROUND MEDIUM 192 SLICES PER CASE | BACON CKD RND</t>
+          <t>HORMEL FAST N EASY EXTRA COOKED BACON ROUND MEDIUM 192 SLICES PER CASE BACON CKD RND</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Fully cooked sliced round bacon, 192 slices per case.</t>
+          <t>Fully cooked round bacon, 192 slices per case</t>
         </is>
       </c>
     </row>
@@ -2021,12 +2017,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND | BACON LAYFLAT C/C 18/22 SMK GF</t>
+          <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND BACON LAYFLAT C/C 18/22 SMK GF</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Gluten-free smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Gluten-free sliced bacon, 18-22</t>
         </is>
       </c>
     </row>
@@ -2038,7 +2034,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND | BACON 18/22 LAYOUT</t>
+          <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND BACON 18/22 LAYOUT</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2055,7 +2051,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND | BACON LAYOUT 18/22</t>
+          <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND BACON LAYOUT 18/22</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2072,7 +2068,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND | BACON SLICED 18-22 L/O</t>
+          <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND BACON SLICED 18-22 L/O</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2089,7 +2085,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE ORIGINAL BACON 13 17 SLICES PER POUND | BACON LAYOUT 13/17</t>
+          <t>OLD SMOKEHOUSE ORIGINAL BACON 13 17 SLICES PER POUND BACON LAYOUT 13/17</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2106,7 +2102,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND | 32669 BACON HRML APPLEWOOD 13/17</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND 32669 BACON HRML APPLEWOOD 13/17</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2123,7 +2119,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND | BACON LAYOUT 13/17 APPLWD</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND BACON LAYOUT 13/17 APPLWD</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2140,12 +2136,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND | BACON LAYFLAT C/C 13/17 APL GF</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 APL GF</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 13-17 slices per pound, lay</t>
+          <t>Cooked</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2153,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND | SMKD APLWOOD BACON 13-17 CT.</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND SMKD APLWOOD BACON 13-17 CT.</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2174,12 +2170,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>HORMEL CANADIAN STYLE BACON | BACON CANADN STY HALF STICK NJ</t>
+          <t>HORMEL CANADIAN STYLE BACON BACON CANADN STY HALF STICK NJ</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Canadian-style half-stick bacon.</t>
+          <t>Canadian-style half-stick bacon</t>
         </is>
       </c>
     </row>
@@ -2191,7 +2187,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>HORMEL CANADIAN STYLE BACON | BACON CANAD WHL | BACON CANAD WHL STIX</t>
+          <t>HORMEL CANADIAN STYLE BACON BACON CANAD WHL BACON CANAD WHL STIX</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -2208,7 +2204,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>HORMEL COUNTRY BRAND BACON 18 22 SLICES PER POUND WIDE SHINGLE | BACON LAYOUT 18/22 SMKD</t>
+          <t>HORMEL COUNTRY BRAND BACON 18 22 SLICES PER POUND WIDE SHINGLE BACON LAYOUT 18/22 SMKD</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -2225,7 +2221,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>HORMEL EXTRA COOKED 0 375 INCH BACON TOPPING | BACON PIECES EXTRA CKD 3/8IN</t>
+          <t>HORMEL EXTRA COOKED 0 375 INCH BACON TOPPING BACON PIECES EXTRA CKD 3/8IN</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -2242,12 +2238,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>HORMEL EXTRA COOKED 0 375 INCH BACON TOPPING | BACON BITS 3/8</t>
+          <t>HORMEL EXTRA COOKED 0 375 INCH BACON TOPPING BACON BITS 3/8</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 3/8‑inch pieces</t>
+          <t>Fully cooked bacon bits, 3/8-inch pieces</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2255,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE ORIGINAL BACON 9 13 SLICES PER POUND | BACON LAYOUT 9/13</t>
+          <t>OLD SMOKEHOUSE ORIGINAL BACON 9 13 SLICES PER POUND BACON LAYOUT 9/13</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -2276,12 +2272,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>BACON CUBED COOKED .25X.25 | BACON TOPPING CKD 1/4IN DCD | BACON COOKED DICED 1/4""</t>
+          <t>BACON CUBED COOKED .25X.25 BACON TOPPING CKD 1/4IN DCD BACON COOKED DICED 1/4</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Fully cooked cubed bacon, 0.25 × 0.25‑inch pieces.</t>
+          <t>Cooked cubed bacon, 1/4-inch pieces</t>
         </is>
       </c>
     </row>
@@ -2293,12 +2289,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>BACON LAYER THICK SLICE 1/2"" | BACON LAYER 1/2 THK CUT SLIC</t>
+          <t>BACON LAYER THICK SLICE 1/2 BACON LAYER 1/2 THK CUT SLIC</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Thick-cut sliced bacon, 1/2‑inch slices.</t>
+          <t>Thick-sliced bacon, 1/2-inch slices.</t>
         </is>
       </c>
     </row>
@@ -2310,12 +2306,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>BACON PRECOOKED SLICED | BACON PRECOOKED SLAB SLI (BLMP</t>
+          <t>BACON PRECOOKED SLICED BACON PRECOOKED SLAB SLI (BLMP</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon</t>
+          <t>Fully cooked sliced and slab bacon</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2323,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD GAS FLUSHED SHINGLE 10-12 CT | BACON SHINGLE 10/12 AW GF PR12</t>
+          <t>BACON SLICED APPLEWOOD GAS FLUSHED SHINGLE 10-12 CT BACON SHINGLE 10/12 AW GF PR12</t>
         </is>
       </c>
       <c r="C116" t="inlineStr"/>
@@ -2340,7 +2336,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>BACON HC HRI 1/2"" LAYER | BACON LAYFLAT C/C HONEY 1/2</t>
+          <t>BACON HC HRI 1/2 LAYER BACON LAYFLAT C/C HONEY 1/2</t>
         </is>
       </c>
       <c r="C117" t="inlineStr"/>
@@ -2353,12 +2349,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>APPLEWOOD SMOKED BACON  13/17 FTR | BACON SLCD APPLWD SMKD 13-17</t>
+          <t>APPLEWOOD SMOKED BACON 13/17 FTR BACON SLCD APPLWD SMKD 13-17</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 13-17 slices per pound</t>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2366,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>APPLEWOOD SMOKED BACON  13/17 FTR | BACON LAYOUT 13/17 FTR</t>
+          <t>APPLEWOOD SMOKED BACON 13/17 FTR BACON LAYOUT 13/17 FTR</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -2404,7 +2400,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD SMOKED GAS FLUSHED SHINGLE 14-16 CT | BACON SHINGLE 14/16 AW GF PR12</t>
+          <t>BACON SLICED APPLEWOOD SMOKED GAS FLUSHED SHINGLE 14-16 CT BACON SHINGLE 14/16 AW GF PR12</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -2417,12 +2413,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>BACON SLAB WHOLE APPLEWOOD FZ | BACON SLAB WHL APPLWD FZ</t>
+          <t>BACON SLAB WHOLE APPLEWOOD FZ BACON SLAB WHL APPLWD FZ</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Frozen applewood-smoked whole slab bacon</t>
+          <t>Frozen whole slab bacon, applewood-smoked</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2430,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>BACON 18/22 CT LAYOUT HICKORY SMOKED | BACON L/O 18-22CT CC FZ</t>
+          <t>BACON 18/22 CT LAYOUT HICKORY SMOKED BACON L/O 18-22CT CC FZ</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -2451,12 +2447,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>BACON L/O #2 FZ 15# P/L | BACON L/O #2 FZ CHEF'S CHC | BACON #2 LAYOUT FROZEN</t>
+          <t>BACON L/O 2 FZ 15 P/L BACON L/O 2 FZ CHEF S CHC BACON 2 LAYOUT FROZEN</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, layflat</t>
+          <t>Frozen sliced bacon, 15 slices per pound, lay</t>
         </is>
       </c>
     </row>
@@ -2468,7 +2464,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD LAYFLAT GAS FLUSHED PRIME12 14-16 CT | BACON LAYFLT 14/16 AW GF PR12</t>
+          <t>BACON SLICED APPLEWOOD LAYFLAT GAS FLUSHED PRIME12 14-16 CT BACON LAYFLT 14/16 AW GF PR12</t>
         </is>
       </c>
       <c r="C125" t="inlineStr"/>
@@ -2498,12 +2494,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>BACON CKD THN SLCD | BACON CKD MED SLCD</t>
+          <t>BACON CKD THN SLCD BACON CKD MED SLCD</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Fully cooked thin and medium sliced bacon</t>
+          <t>Fully cooked thin sliced bacon and fully cooked medium sliced bacon.</t>
         </is>
       </c>
     </row>
@@ -2515,12 +2511,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>BACON CKD MED SLCD | BACON CKD THN SLCD</t>
+          <t>BACON CKD MED SLCD BACON CKD THN SLCD</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Fully cooked medium sliced bacon and fully cooked thin sliced bacon</t>
+          <t>Fully cooked medium-sliced and thin-sliced bacon</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2528,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>BACON | BACON MINCED AND MOIST LEVEL 5</t>
+          <t>BACON BACON MINCED AND MOIST LEVEL 5</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -2549,14 +2545,10 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>BCN,SFD,PEPR-CRST,1/15#,LO,FZ | BACON SLCD PEPR CRSTD RTC</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>Frozen sliced pepper-crusted bacon, layflat</t>
-        </is>
-      </c>
+          <t>BCN,SFD,PEPR-CRST,1/15 ,LO,FZ BACON SLCD PEPR CRSTD RTC</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -2566,7 +2558,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>BACON | MINCED &amp; MOIST BACON</t>
+          <t>BACON MINCED &amp; MOIST BACON</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -2583,7 +2575,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>BACON BEEF SLICED HALAL | BEEF BACON SLI HALAL</t>
+          <t>BACON BEEF SLICED HALAL BEEF BACON SLI HALAL</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -2600,7 +2592,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>8 SYS SLCD SLAB HON BACN 14/16 15 LB | BACON SHINGLE 14/16 HNY PR12</t>
+          <t>8 SYS SLCD SLAB HON BACN 14/16 15 LB BACON SHINGLE 14/16 HNY PR12</t>
         </is>
       </c>
       <c r="C133" t="inlineStr"/>
@@ -2630,12 +2622,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>BACON BEEF SLICED SMOKED HONEY CURED RAW | BACON BEEF SLAB SLICE</t>
+          <t>BACON BEEF SLICED SMOKED HONEY CURED RAW BACON BEEF SLAB SLICE</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Raw honey-cured smoked sliced bacon</t>
+          <t>Raw honey-cured smoked sliced beef bacon</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2652,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>BACON 18/22 CT SLICED | BACON SLCD ETE 18-22CT FZ</t>
+          <t>BACON 18/22 CT SLICED BACON SLCD ETE 18-22CT FZ</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -2677,7 +2669,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>BACON SLCD 14-16CT FZ 15# KE | BACON 14/16 CT SLICED FROZEN | BACON SLCD ETE 14-16CT FZ | BACON SLICED 14/16 CT FZ</t>
+          <t>BACON SLCD 14-16CT FZ 15 KE BACON 14/16 CT SLICED FROZEN BACON SLCD ETE 14-16CT FZ BACON SLICED 14/16 CT FZ</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -2694,12 +2686,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>BACON SLCD ETE 14-18CT/#</t>
+          <t>BACON SLCD ETE 14-18CT/</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Sliced extra‑thick bacon, 14‑18 slices per pound.</t>
+          <t>Sliced bacon, 14-18 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -2711,12 +2703,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE MAPLE PEPPER BACON 13 17 SLICES PER POUND | BACON LAYFLAT C/C 13/17 MPLPPR</t>
+          <t>OLD SMOKEHOUSE MAPLE PEPPER BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 MPLPPR</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Maple pepper sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2720,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>HORMEL LAYOUT BACON 13 17 SLICES PER POUND | BACON LAYFLAT C/C 13/17 SMK GF</t>
+          <t>HORMEL LAYOUT BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 SMK GF</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
@@ -2741,12 +2733,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>HORMEL WATER ADDED CANADIAN STYLE BACON WITH SIRLOIN | BACON CANADIAN STY HLF STCK WA</t>
+          <t>HORMEL WATER ADDED CANADIAN STYLE BACON WITH SIRLOIN BACON CANADIAN STY HLF STCK WA</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Water-added Canadian-style half‑stick slab bacon with sirloin.</t>
+          <t>Water-added half-stacked Canadian-style bacon with sirloin.</t>
         </is>
       </c>
     </row>
@@ -2758,12 +2750,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND | BACON SLAB CC 13/17 APL SMK GF</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND BACON SLAB CC 13/17 APL SMK GF</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked slab bacon, 13‑17 slices per pound.</t>
+          <t>Gluten-free applewood-smoked slab bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -2775,12 +2767,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>HORMEL HONEY CURED BACON 13 17 SLICES PER POUND WIDE SHINGLE | BACON LAYFLAT E/E 13/17 HNY GF</t>
+          <t>HORMEL HONEY CURED BACON 13 17 SLICES PER POUND WIDE SHINGLE BACON LAYFLAT E/E 13/17 HNY GF</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Raw gluten-free honey-c</t>
+          <t>Raw honey-cured wide shingle sliced bacon, 13-17 slices per pound, layflat.</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2784,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 18 22 SLICES PER POUND | BACON LAYFLAT APPLE SMK 18/22</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 18 22 SLICES PER POUND BACON LAYFLAT APPLE SMK 18/22</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -2809,12 +2801,12 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>HORMEL HONEY CURED BACON 18 22 SLICES PER POUND WIDE SHINGLE | BACON LAYFLAT E/E 18/22 HNY GF</t>
+          <t>HORMEL HONEY CURED BACON 18 22 SLICES PER POUND WIDE SHINGLE BACON LAYFLAT E/E 18/22 HNY GF</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Honey-cured, gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw honey-cured sliced wide shingle bacon, 18-22 slices per pound, layflat, gluten‑free.</t>
         </is>
       </c>
     </row>
@@ -2826,14 +2818,10 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>HORMEL REGULAR COOK 0 5 INCH BACON TOPPING | TOPPING BACON 1/2"" COOKED</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>Fully cooked sliced bacon, 1/2-inch slices</t>
-        </is>
-      </c>
+          <t>HORMEL REGULAR COOK 0 5 INCH BACON TOPPING TOPPING BACON 1/2 COOKED</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2843,14 +2831,10 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>HORMEL REGULAR COOK 0 5 INCH BACON TOPPING | BACON TOPPING REG COOKED 1/2</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>Fully cooked bacon topping, 0.5‑inch pieces</t>
-        </is>
-      </c>
+          <t>HORMEL REGULAR COOK 0 5 INCH BACON TOPPING BACON TOPPING REG COOKED 1/2</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2860,12 +2844,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>HORMEL REGULAR COOK 0 5 INCH BACON TOPPING | BACON CKD 1/2IN DCD</t>
+          <t>HORMEL REGULAR COOK 0 5 INCH BACON TOPPING BACON CKD 1/2IN DCD</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Fully cooked diced bacon, 1/2‑inch pieces</t>
+          <t>Fully cooked topping diced bacon, 0.5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -2877,7 +2861,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 9 13 SLICES PER POUND | BACON LAYFLAT C/C 9/13 APL GF</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 9 13 SLICES PER POUND BACON LAYFLAT C/C 9/13 APL GF</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -2894,7 +2878,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 9 13 SLICES PER POUND | BACON L/O APPLWD SMKD 9-13CT</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 9 13 SLICES PER POUND BACON L/O APPLWD SMKD 9-13CT</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -2911,14 +2895,10 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>HORMEL FAST 'N EASY COOKED BACON LARGE ROUND | BACON  PORK CKD 144 CT RN</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>Fully cooked large round bacon</t>
-        </is>
-      </c>
+          <t>HORMEL FAST N EASY COOKED BACON LARGE ROUND BACON PORK CKD 144 CT RN</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2928,12 +2908,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>HORMEL NATURAL CHOICE UNCURED BACON 13 17 SLICES PER POUND | BACON 1 13/17CT FULLY COOKED 288SLC</t>
+          <t>HORMEL NATURAL CHOICE UNCURED BACON 13 17 SLICES PER POUND BACON 1 13/17CT FULLY COOKED 288SLC</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Fully cooked uncured sliced bacon, 13-17 slices per pound</t>
+          <t>Fully cooked uncured sliced bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -2945,12 +2925,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>HORMEL NATURAL CHOICE UNCURED BACON 13 17 SLICES PER POUND | BACON LAYFLAT C/C 13/17 NAT GF</t>
+          <t>HORMEL NATURAL CHOICE UNCURED BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 NAT GF</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Uncured natural gluten-free sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Uncured gluten-free sliced bacon, 13</t>
         </is>
       </c>
     </row>
@@ -2962,12 +2942,12 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>HORMEL CANADIAN STYLE BACON WITH SIRLOIN SLICED AND QUARTERED 10 SLICES PER OUNC | BACON CANADN STY WA SLI &amp; QTRD</t>
+          <t>HORMEL CANADIAN STYLE BACON WITH SIRLOIN SLICED AND QUARTERED 10 SLICES PER OUNC BACON CANADN STY WA SLI &amp; QTRD</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Canadian-style sirloin sliced and quartered bacon, 10 slices per ounce.</t>
+          <t>Sliced and quartered Canadian-style bacon with sirloin, 10 slices per ounce.</t>
         </is>
       </c>
     </row>
@@ -2979,12 +2959,12 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>HORMEL EXTRA COOKED 0 5 INCH BACON TOPPING | BACON PCS CKD 1/2</t>
+          <t>HORMEL EXTRA COOKED 0 5 INCH BACON TOPPING BACON PCS CKD 1/2</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Fully cooked bacon pieces, 0.5‑inch pieces.</t>
+          <t>Fully cooked topping bacon pieces, 0.5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -2996,12 +2976,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>HORMEL FAST 'N EASY COOKED BACON MEDIUM ROUND | BACON PRECOOKED ROUND 3.5 INCH</t>
+          <t>HORMEL FAST N EASY COOKED BACON MEDIUM ROUND BACON PRECOOKED ROUND 3.5 INCH</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Fully cooked round bacon, 3.5‑inch diameter.</t>
+          <t>Fully cooked round bacon, 3.5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -3013,12 +2993,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE COOKED THICK BACON | BACON PRECOOKED THICK SLI SGR</t>
+          <t>OLD SMOKEHOUSE COOKED THICK BACON BACON PRECOOKED THICK SLI SGR</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Fully cooked thick sliced sugar-cured bacon</t>
+          <t>Fully cooked thick sliced bacon, sugar-cured</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3010,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>HORMEL BLACK LABEL BACON 13 17 PIECES PER POUND | BACON SLAB CC 13/17 SMK BLK GF</t>
+          <t>HORMEL BLACK LABEL BACON 13 17 PIECES PER POUND BACON SLAB CC 13/17 SMK BLK GF</t>
         </is>
       </c>
       <c r="C159" t="inlineStr"/>
@@ -3043,12 +3023,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND | BACON JALAPENO 13/17</t>
+          <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND BACON JALAPENO 13/17</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Jalapeno-flavored sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Jalapeno sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3060,14 +3040,10 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND | BACON LAYFLAT C/C 13/17 JAL FZ</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>Frozen jalapeno sliced bacon, 13-17 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 JAL FZ</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3077,14 +3053,10 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND | BACON LAYFLAT C/C 13/17 JAL GF</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>Gluten-free jalapeno sliced bacon, 13-17 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 JAL GF</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -3094,12 +3066,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>BACON ENDS  PCS RAW 10# INDKTCH | BACON ENDS  PCS RAW</t>
+          <t>BACON ENDS PCS RAW 10 INDKTCH BACON ENDS PCS RAW</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Raw bacon ends</t>
+          <t>Raw bacon ends, pieces</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3096,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>HORMEL FAST N EASY COOKED THICK BACON 300 SLICES | BACON PRECOOKED THICK SLICED</t>
+          <t>HORMEL FAST N EASY COOKED THICK BACON 300 SLICES BACON PRECOOKED THICK SLICED</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -3141,7 +3113,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>BACON BIT REAL POUCH | BACON BIT REAL</t>
+          <t>BACON BIT REAL POUCH BACON BIT REAL</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -3175,12 +3147,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>BACON CHEESEBURGER | CHEESEBURGER BACON ON BRIOCHE</t>
+          <t>BACON CHEESEBURGER CHEESEBURGER BACON ON BRIOCHE</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Bacon cheeseburger on brioche bun</t>
+          <t>Bacon for cheeseburger on brioche.</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3164,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>BACON BEEF SLCS 4-2.5# | BACON BEEF SLCS</t>
+          <t>BACON BEEF SLCS 4-2.5 BACON BEEF SLCS</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -3209,14 +3181,10 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>HORMEL LAYOUT BACON 23 27 SLICES PER POUND | BACON LAYFLAT C/C 23/27 SMK GF</t>
-        </is>
-      </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>Gluten-free smoked sliced bacon, 23-27 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>HORMEL LAYOUT BACON 23 27 SLICES PER POUND BACON LAYFLAT C/C 23/27 SMK GF</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -3226,7 +3194,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>HORMEL EXTRA COOKED 1 0 INCH BACON TOPPING | BACON TOPPING EXTRA CKD 1 IN</t>
+          <t>HORMEL EXTRA COOKED 1 0 INCH BACON TOPPING BACON TOPPING EXTRA CKD 1 IN</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -3243,7 +3211,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>BAGEL BRANDS PRECKD BACON 1200 CT | BACON APPLEWOOD FC</t>
+          <t>BAGEL BRANDS PRECKD BACON 1200 CT BACON APPLEWOOD FC</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -3260,7 +3228,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>BCN,SLCD,FC,RTE,GHP,2/1.72#,300C,GF | BACON PRECOOKED SLI SM GHP FRS | BACON PRECOOKED SLICED SM GHP FRESH</t>
+          <t>BCN,SLCD,FC,RTE,GHP,2/1.72 ,300C,GF BACON PRECOOKED SLI SM GHP FRS BACON PRECOOKED SLICED SM GHP FRESH</t>
         </is>
       </c>
       <c r="C173" t="inlineStr"/>
@@ -3273,12 +3241,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>BACON DICED APPLEWOOD | BACON PCS CKD APPLWD</t>
+          <t>BACON DICED APPLEWOOD BACON PCS CKD APPLWD</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Fully cooked diced applewood-smoked bacon</t>
+          <t>Fully cooked diced applewood-smoked bacon pieces</t>
         </is>
       </c>
     </row>
@@ -3290,7 +3258,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>BACON BITS IMIT | BACON BITS IMITATION</t>
+          <t>BACON BITS IMIT BACON BITS IMITATION</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -3324,7 +3292,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>8 SYS HKSM LFLT SLCD BACN 18/22 GF 15 LB | BACON LAYFLT 18/22 SMK GF PR12</t>
+          <t>8 SYS HKSM LFLT SLCD BACN 18/22 GF 15 LB BACON LAYFLT 18/22 SMK GF PR12</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
@@ -3337,7 +3305,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>BEEF BACON CHIPPED CURED COOKED | BEEF BACON CHOPPED</t>
+          <t>BEEF BACON CHIPPED CURED COOKED BEEF BACON CHOPPED</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -3354,12 +3322,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>BACON PORK REAL DICED .25  SMOKED CURED COOKED REF GAS FLUSHED | BACON  PORK END   PC REAL</t>
+          <t>BACON PORK REAL DICED .25 SMOKED CURED COOKED REF GAS FLUSHED BACON PORK END PC REAL</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Cooked smoked-cured diced bacon, 0.25‑inch pieces</t>
+          <t>Cooked smoked-cured diced bacon, 0.25‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -3371,14 +3339,10 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>FRZ 1073402 REL LAYFLAT 18/22 | BACON 18/22 CT LAYFLAT SMOKED | BACON LAYFLAT 18/22 SMOKED</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>Frozen smoked sliced bacon, 18-22 slices</t>
-        </is>
-      </c>
+          <t>FRZ 1073402 REL LAYFLAT 18/22 BACON 18/22 CT LAYFLAT SMOKED BACON LAYFLAT 18/22 SMOKED</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -3388,12 +3352,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>5886381 CLASSIC APLWD 14/18 | BACON 14/18 CT LAYFLAT APPLEWOOD GLUTEN FREE | BACON LAYFLAT C/C 14/18 APL GF | BACON 14/18 CT LAYFLAT APPLEWOOD GLUTEN FREE FROZEN</t>
+          <t>5886381 CLASSIC APLWD 14/18 BACON 14/18 CT LAYFLAT APPLEWOOD GLUTEN FREE BACON LAYFLAT C/C 14/18 APL GF BACON 14/18 CT LAYFLAT APPLEWOOD GLUTEN FREE FROZEN</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Frozen applewood-smoked sliced gluten-free bacon, 14-18 slices per pound, layflat.</t>
+          <t>Frozen gluten-free applewood-smoked sliced bacon, 14-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3405,14 +3369,10 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>5756893 CLASSIC PRCKD BCN HSMO | BACON PRECOOKED HEARTY SMOKED SLICED | BACON PRECOOKED REG SLI HRTYSM</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>Fully cooked smoked sliced bacon</t>
-        </is>
-      </c>
+          <t>5756893 CLASSIC PRCKD BCN HSMO BACON PRECOOKED HEARTY SMOKED SLICED BACON PRECOOKED REG SLI HRTYSM</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -3422,7 +3382,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>FRZ 1005750 CLASSIC FLAT 14/18 | BACON LAYFLAT C/C 14/18 SMOKED</t>
+          <t>FRZ 1005750 CLASSIC FLAT 14/18 BACON LAYFLAT C/C 14/18 SMOKED</t>
         </is>
       </c>
       <c r="C183" t="inlineStr"/>
@@ -3435,14 +3395,10 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>FRZ 1005842 CLASSIC LF 18/22 | BACON 18/22 CT C/C SMOKED LAYFLAT | BACON LAYFLAT C/C 18/22 SMOKED</t>
-        </is>
-      </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>Frozen cured-smoked sliced bacon, 18-22 slices per</t>
-        </is>
-      </c>
+          <t>FRZ 1005842 CLASSIC LF 18/22 BACON 18/22 CT C/C SMOKED LAYFLAT BACON LAYFLAT C/C 18/22 SMOKED</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -3452,12 +3408,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>SYS 5321427 SLAB BACNTEXAS SMOKED CENTER CUT SLICED SLAB BACON (18/22) 1/15# | BACON SLAB C/C 18/22 TX SMKD</t>
+          <t>SYS 5321427 SLAB BACNTEXAS SMOKED CENTER CUT SLICED SLAB BACON (18/22) 1/15 BACON SLAB C/C 18/22 TX SMKD</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Texas-smoked sliced slab bacon, 18-22 slices per pound</t>
+          <t>Texas-smoked center-cut sliced slab bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -3469,12 +3425,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>SYS 1073402 LYFLT 18/22SYSCO RELIANCE 18/22 LAYFLAT BACON 15# | BACON 18/22 CT LAYFLAT SMOKED | BACON LAYFLAT 18/22 SMOKED</t>
+          <t>SYS 1073402 LYFLT 18/22SYSCO RELIANCE 18/22 LAYFLAT BACON 15 BACON 18/22 CT LAYFLAT SMOKED BACON LAYFLAT 18/22 SMOKED</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Raw smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3486,14 +3442,10 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>SYS 1359413 LYFLT BACNSYSCO CLASSIC TEXAS SMKD CTCT INDIVIDUAL SPACED, LAYFLAT BACON (14/18) 1/15# | BACON LAYFLAT CC 14/18 TX SMKD</t>
-        </is>
-      </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>Texas-smoked sliced bacon, 14-18 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>SYS 1359413 LYFLT BACNSYSCO CLASSIC TEXAS SMKD CTCT INDIVIDUAL SPACED, LAYFLAT BACON (14/18) 1/15 BACON LAYFLAT CC 14/18 TX SMKD</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -3503,12 +3455,12 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>SYS 1011790 SLAB BACNSYSCO RELIANCE TEXAS SMOKED SLICED SLAB BACON (14/18) 1/15# | BACON SLAB 14/18 TX SMK FZ</t>
+          <t>SYS 1011790 SLAB BACNSYSCO RELIANCE TEXAS SMOKED SLICED SLAB BACON (14/18) 1/15 BACON SLAB 14/18 TX SMK FZ</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Frozen Texas-smoked sliced slab bacon, 14-18 slices per pound.</t>
+          <t>Frozen Texas-smoked sliced slab bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -3520,12 +3472,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>SYS 8928053 SLAB BACNSYSCO RELIANCE TEXAS SMOLED SLICED SLAB BACON (14/18) 1/30# | BACON SLAB SLI 14/18CT TX SMKD</t>
+          <t>SYS 8928053 SLAB BACNSYSCO RELIANCE TEXAS SMOLED SLICED SLAB BACON (14/18) 1/30 BACON SLAB SLI 14/18CT TX SMKD</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Sliced slab bacon, 14-18 slices per pound, Texas-smoked.</t>
+          <t>Raw sliced slab bacon, Texas-smoked, 14-18 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -3537,7 +3489,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2548162 ARREZZIO BACON BITS | BACON BIT REAL COOKED GLUTEN FREE 3/4"" | BACON BIT REAL CKD 3/4IN GF</t>
+          <t>2548162 ARREZZIO BACON BITS BACON BIT REAL COOKED GLUTEN FREE 3/4 BACON BIT REAL CKD 3/4IN GF</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -3554,12 +3506,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>SYS 6438545 FPK RANDSYSCO RANCH &amp;  GRILL RANDOM CUT LAYFLAT BACON. 15# | BACON LAYFLAT RANDOM SMKD #2</t>
+          <t>SYS 6438545 FPK RANDSYSCO RANCH &amp; GRILL RANDOM CUT LAYFLAT BACON. 15 BACON LAYFLAT RANDOM SMKD 2</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Smoked random-cut layflat bacon.</t>
+          <t>Smoked cut bacon, layflat</t>
         </is>
       </c>
     </row>
@@ -3571,12 +3523,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>5857679 SYS CLASSIC PRE-CKD | BACON PRECOOKED SLICED 24/26 | BACON PRECOOKED THICK SLICE</t>
+          <t>5857679 SYS CLASSIC PRE-CKD BACON PRECOOKED SLICED 24/26 BACON PRECOOKED THICK SLICE</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Fully cooked sliced thick-cut bacon, 24-26 slices per pound.</t>
+          <t>Fully cooked sliced thick bacon, 24-26 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -3588,12 +3540,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>5757051 CLASSIC PRCK BACON TOP | BACON BIT REAL CKD 3/8 GF | BACON BIT REAL COOKED GLUTEN FREE 3/8""</t>
+          <t>5757051 CLASSIC PRCK BACON TOP BACON BIT REAL CKD 3/8 GF BACON BIT REAL COOKED GLUTEN FREE 3/8</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 3/8-inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -3605,12 +3557,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>NATURALLY HARDWOOD SMOKED SLICED ROLLED PORK BELLY | PORK BELLY SMOKED SLICED ROLLED | PORK BELLY SMKD SLICED ROLLED</t>
+          <t>NATURALLY HARDWOOD SMOKED SLICED ROLLED PORK BELLY PORK BELLY SMOKED SLICED ROLLED PORK BELLY SMKD SLICED ROLLED</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Hardwood-smoked sliced rolled pork belly bacon</t>
+          <t>Hardwood-smoked sliced rolled pork belly bacon.</t>
         </is>
       </c>
     </row>
@@ -3622,14 +3574,10 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>SYS 1359405 LYFLT BACNSYSCO CLASSIC TEXAS SMOKED INDIVIDUAL SPACED LAYFLAT BACON 1/15# (18/22) | BACON LAYFLAT CC 18/22 TX SMKD</t>
-        </is>
-      </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>Texas-smoked sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>SYS 1359405 LYFLT BACNSYSCO CLASSIC TEXAS SMOKED INDIVIDUAL SPACED LAYFLAT BACON 1/15 (18/22) BACON LAYFLAT CC 18/22 TX SMKD</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -3639,12 +3587,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>BACON SLAB FRUITWOOD SMOKED PR12 | BACON SLAB APPLEWOOD SMKD PR12</t>
+          <t>BACON SLAB FRUITWOOD SMOKED PR12 BACON SLAB APPLEWOOD SMKD PR12</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Fruitwood-smoked and applewood-smoked slab bacon</t>
+          <t>Applewood-smoked slab bacon</t>
         </is>
       </c>
     </row>
@@ -3656,7 +3604,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>SYS 1345669 SLAB BACNCLASSIC TEXAS SMOKED CENTER CUT SLICED SLAB BACON (10/14) 1/15# | BACON SLAB C/C 10/14 TX SMOKED</t>
+          <t>SYS 1345669 SLAB BACNCLASSIC TEXAS SMOKED CENTER CUT SLICED SLAB BACON (10/14) 1/15 BACON SLAB C/C 10/14 TX SMOKED</t>
         </is>
       </c>
       <c r="C197" t="inlineStr"/>
@@ -3669,7 +3617,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>SYS 5886579 FPK 14/18SYSCO CLASSIC GRILL FRESH SLICED BACON 14/18. 2/10# | BACON LAYFLAT C/C 14/18 SMK GF</t>
+          <t>SYS 5886579 FPK 14/18SYSCO CLASSIC GRILL FRESH SLICED BACON 14/18. 2/10 BACON LAYFLAT C/C 14/18 SMK GF</t>
         </is>
       </c>
       <c r="C198" t="inlineStr"/>
@@ -3682,7 +3630,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>SYS 6725030 LYFLT BACNSYSCO CLASSIC TEXAS SMOKED INDIVIDUAL SPACED LAYFLAT BACON 1/15# (10/14) | BACON LAYFLAT CC 10/14 TX SMKD</t>
+          <t>SYS 6725030 LYFLT BACNSYSCO CLASSIC TEXAS SMOKED INDIVIDUAL SPACED LAYFLAT BACON 1/15 (10/14) BACON LAYFLAT CC 10/14 TX SMKD</t>
         </is>
       </c>
       <c r="C199" t="inlineStr"/>
@@ -3695,7 +3643,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>FRZ 1151422 REL LF 14/18 15LB | BACON 14/18 CT LAYFLAT E/E SMOKED</t>
+          <t>FRZ 1151422 REL LF 14/18 15LB BACON 14/18 CT LAYFLAT E/E SMOKED</t>
         </is>
       </c>
       <c r="C200" t="inlineStr"/>
@@ -3708,12 +3656,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>FRZ 1136779 REL LAY FLAT 22/26 | BACON LAYFLAT 22/26 SMOKED | BACON 22/26 CT LAYFLAT SMOKED</t>
+          <t>FRZ 1136779 REL LAY FLAT 22/26 BACON LAYFLAT 22/26 SMOKED BACON 22/26 CT LAYFLAT SMOKED</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Frozen smoked bacon, 22-26 slices per pound, layflat</t>
+          <t>Frozen smoked sliced bacon, 22-26 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3725,12 +3673,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>BACON 18/22 CT PORK LAID | BACON  PORK 18-22 SLCD LA</t>
+          <t>BACON 18/22 CT PORK LAID BACON PORK 18-22 SLCD LA</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced pork bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3759,12 +3707,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>BACON 18/22 CT PORK LAYOUT HICKORY SMOKED | BACON  PORK 18-22 SLCD LA</t>
+          <t>BACON 18/22 CT PORK LAYOUT HICKORY SMOKED BACON PORK 18-22 SLCD LA</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Hickory-smoked sliced pork bacon, 18-22 slices per pound, layflat</t>
+          <t>Hickory-smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3776,12 +3724,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>SYS 1151422 LYFLT BACNSYSCO RELIANCE 14/18 INDIVIDUAL SPACED LAYFLAT BACON 15# | BACON LAYFLAT 14/18 SMOKED</t>
+          <t>SYS 1151422 LYFLT BACNSYSCO RELIANCE 14/18 INDIVIDUAL SPACED LAYFLAT BACON 15 BACON LAYFLAT 14/18 SMOKED</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Smoked layflat sliced bacon, 14-18 slices per pound.</t>
+          <t>Smoked sliced bacon, 14-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3793,12 +3741,12 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>6191874 SYS CLS PRE-CKD THICK | BACON PRECOOKED XTHICK SLICE</t>
+          <t>6191874 SYS CLS PRE-CKD THICK BACON PRECOOKED XTHICK SLICE</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Fully cooked thick sliced bacon</t>
+          <t>Fully cooked thick sliced bacon.</t>
         </is>
       </c>
     </row>
@@ -3810,7 +3758,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>FRZ SUG TWO STAR EZ 18/22 | BACON LAYOUT 18-22 CT</t>
+          <t>FRZ SUG TWO STAR EZ 18/22 BACON LAYOUT 18-22 CT</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -3832,7 +3780,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Bacon, egg, and cheese bowl.</t>
+          <t>Bacon, egg, and cheese bowl</t>
         </is>
       </c>
     </row>
@@ -3844,7 +3792,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>BACON BEEF SLCD | BACON BEEF SLICED</t>
+          <t>BACON BEEF SLCD BACON BEEF SLICED</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -3866,7 +3814,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 300 slices per case</t>
+          <t>Fully cooked bacon.</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3826,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>FRZ BACON BITS DELUXE | BACON PCS DLX</t>
+          <t>FRZ BACON BITS DELUXE BACON PCS DLX</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -3895,7 +3843,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>FRZ BACON BITS DELUXE | BACON  PORK REAL PC .38</t>
+          <t>FRZ BACON BITS DELUXE BACON PORK REAL PC .38</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -3912,7 +3860,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>FRZ BACON BITS DELUXE | BACON BIT REAL PRECOOKED | BACON BIT PRCK REAL</t>
+          <t>FRZ BACON BITS DELUXE BACON BIT REAL PRECOOKED BACON BIT PRCK REAL</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -3929,12 +3877,12 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>BACON, GM HARDWOOD SMKD W APPLE CIDER GF | (Z)BACON,GM HRDWD SMKD W APPLE CIDER GF</t>
+          <t>BACON, GM HARDWOOD SMKD W APPLE CIDER GF (Z)BACON,GM HRDWD SMKD W APPLE CIDER GF</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Gluten-free hardwood apple cider-smoked bacon</t>
+          <t>Hardwood-smoked bacon with apple cider, gluten-free.</t>
         </is>
       </c>
     </row>
@@ -3968,7 +3916,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Sweet bacon.</t>
+          <t>Bacon</t>
         </is>
       </c>
     </row>
@@ -3985,7 +3933,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Hickory-smoked bacon, 18-22 slices per pound</t>
+          <t>Hickory-smoked bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -4014,7 +3962,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>BACON BITS FC GOTOFOODS | BACON BIT FC GOTOFOODS</t>
+          <t>BACON BITS FC GOTOFOODS BACON BIT FC GOTOFOODS</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -4031,7 +3979,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>BACON CRUMBLES CKD | BACON CRUMBLES COOKED</t>
+          <t>BACON CRUMBLES CKD BACON CRUMBLES COOKED</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -4048,12 +3996,12 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>BACON SLICED LAYFLAT SMOKED #2 RANDOM | BACON LAYFLAT RANDOM SMKD #2 | BACON LAYFLAT RANDOM SMOKED SLICED #2</t>
+          <t>BACON SLICED LAYFLAT SMOKED 2 RANDOM BACON LAYFLAT RANDOM SMKD 2 BACON LAYFLAT RANDOM SMOKED SLICED 2</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Smoked sliced bacon, layflat</t>
+          <t>Smoked sliced bacon, 2 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4065,12 +4013,12 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED | 55253 BACON HRML APPLEWOOD GRIDDLMASTER</t>
+          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED 55253 BACON HRML APPLEWOOD GRIDDLMASTER</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Raw wide shingled applewood-smoked sliced bacon, 13-17 slices per pound</t>
+          <t>Raw applewood-smoked sliced bacon, 13-17 slices per pound, wide shingled.</t>
         </is>
       </c>
     </row>
@@ -4082,12 +4030,12 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED | BACON LAYOUT APPLEWOOD 13/17</t>
+          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED BACON LAYOUT APPLEWOOD 13/17</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, wide shingled, layflat</t>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4099,12 +4047,12 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED | BACON L/O 13/17 APPLWD GRDLMSTR</t>
+          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED BACON L/O 13/17 APPLWD GRDLMSTR</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Raw applewood-smoked sliced bacon, 13-17 slices per pound, wide shingled,</t>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4116,12 +4064,12 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 18 22 SLICES PER POUND WIDE SHINGLED | BACON  PORK 18-22 CT SLCD</t>
+          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 18 22 SLICES PER POUND WIDE SHINGLED BACON PORK 18-22 CT SLCD</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 18-22 slices per pound</t>
+          <t>Applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4133,12 +4081,12 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 18 22 SLICES PER POUND WIDE SHINGLED | BACON LAYFLAT E/E 18/22 APL GF</t>
+          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 18 22 SLICES PER POUND WIDE SHINGLED BACON LAYFLAT E/E 18/22 APL GF</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw gluten-free applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4150,12 +4098,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 18 22 SLICES PER POUND WIDE SHINGLED | BACON L/O 18/22 APPLWD</t>
+          <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 18 22 SLICES PER POUND WIDE SHINGLED BACON L/O 18/22 APPLWD</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Applewood-smoked wide sh</t>
         </is>
       </c>
     </row>
@@ -4167,14 +4115,10 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>FRZ SUG TWO STAR EZ 14/18 | BACON LAY FLAT SMKD 14-18CT</t>
-        </is>
-      </c>
-      <c r="C228" t="inlineStr">
-        <is>
-          <t>Frozen sugar-cured smoked sliced bacon, 14-18 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>FRZ SUG TWO STAR EZ 14/18 BACON LAY FLAT SMKD 14-18CT</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -4184,7 +4128,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>HORMEL NATURAL CHOICE UNCURED BACON 18 22 SLICES PER POUND | BACON LAYFLAT C/C 18/22 NTGF F</t>
+          <t>HORMEL NATURAL CHOICE UNCURED BACON 18 22 SLICES PER POUND BACON LAYFLAT C/C 18/22 NTGF F</t>
         </is>
       </c>
       <c r="C229" t="inlineStr"/>
@@ -4197,12 +4141,12 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>HORMEL NATURAL CHOICE UNCURED BACON 18 22 SLICES PER POUND | BACON LAYFLAT C/C 18/22 NAT GF</t>
+          <t>HORMEL NATURAL CHOICE UNCURED BACON 18 22 SLICES PER POUND BACON LAYFLAT C/C 18/22 NAT GF</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Raw uncured sliced bacon, 18-22 slices per pound, gluten-free, layflat</t>
+          <t>Raw uncured natural gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4214,12 +4158,12 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>BACON PRECOOKED SLI THICK | BACON SLICED</t>
+          <t>BACON PRECOOKED SLI THICK BACON SLICED</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Fully cooked thick-cut sliced bacon</t>
+          <t>Fully cooked thick sliced bacon</t>
         </is>
       </c>
     </row>
@@ -4231,10 +4175,14 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>CHEF PLEASER BACON, 18/22 | BACON LAYFLAT C/C 18/22 SMK GF</t>
-        </is>
-      </c>
-      <c r="C232" t="inlineStr"/>
+          <t>CHEF PLEASER BACON, 18/22 BACON LAYFLAT C/C 18/22 SMK GF</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Gluten-free smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -4244,7 +4192,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>CHEF PLEASER BACON, 18/22 | BACON  PORK 18-22 CT LAID</t>
+          <t>CHEF PLEASER BACON, 18/22 BACON PORK 18-22 CT LAID</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -4261,12 +4209,12 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>BACON SLAB SLI 16/18 CT FRZN | BACON 16/18 CT SLAB HARDWOOD SMOKED SLICED</t>
+          <t>BACON SLAB SLI 16/18 CT FRZN BACON 16/18 CT SLAB HARDWOOD SMOKED SLICED</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Frozen sliced slab bacon, hardwood-smoked, 16-18 slices per pound.</t>
+          <t>Frozen sliced bacon, hardwood-smoked, 16-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4226,7 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 15 19 SLICES PER POUND | BACON LAYOUT APLWD 15/19 SMKHS</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 15 19 SLICES PER POUND BACON LAYOUT APLWD 15/19 SMKHS</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -4295,12 +4243,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>BW SMOKEY BACON 16-18 | BACON LAYFLAT #2 APPLEWOOD SMK</t>
+          <t>BW SMOKEY BACON 16-18 BACON LAYFLAT 2 APPLEWOOD SMK</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 16-18 slices per pound, layflat</t>
+          <t>Applewood-smoked bacon, 16-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4312,7 +4260,7 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>CHEF PLEASER BACON, 14/18 | BACON 14/18 CT SMOKED RAW LAYOUT</t>
+          <t>CHEF PLEASER BACON, 14/18 BACON 14/18 CT SMOKED RAW LAYOUT</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -4329,7 +4277,7 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>BACON ENDS, 10# BOX | BACON ENDS &amp; PIECES RAW SMKD</t>
+          <t>BACON ENDS, 10 BOX BACON ENDS &amp; PIECES RAW SMKD</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -4346,12 +4294,12 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>TYS FC TS BACN 300 CNT | P/C BACON 300CT 018741</t>
+          <t>TYS FC TS BACN 300 CNT P/C BACON 300CT 018741</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Fully cooked thin sliced bacon, 300 slices</t>
+          <t>Fully cooked thin sliced bacon</t>
         </is>
       </c>
     </row>
@@ -4363,7 +4311,7 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>TYS FC AWS BACN 3/100 | BACON APPLEWOOD SMOKED FC 300 PC</t>
+          <t>TYS FC AWS BACN 3/100 BACON APPLEWOOD SMOKED FC 300 PC</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -4380,14 +4328,10 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>SYS 5886381 APLEWD BACNSYSCO CLS GRILL FRESH APPLEWOOD SMOKED SLICED BACON 14/18 2/10# | BACON LAYFLAT C/C 14/18 APL GF</t>
-        </is>
-      </c>
-      <c r="C241" t="inlineStr">
-        <is>
-          <t>Raw gluten-free applewood-smoked sliced bacon, 14-18 slices per pound, layflat.</t>
-        </is>
-      </c>
+          <t>SYS 5886381 APLEWD BACNSYSCO CLS GRILL FRESH APPLEWOOD SMOKED SLICED BACON 14/18 2/10 BACON LAYFLAT C/C 14/18 APL GF</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -4397,12 +4341,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>BACON SLICED COOKED THICK | BACON PRECOOKED SLAB SLI THK</t>
+          <t>BACON SLICED COOKED THICK BACON PRECOOKED SLAB SLI THK</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Fully cooked thick sliced bacon and fully cooked thick slab bacon</t>
+          <t>Fully cooked thick sliced bacon</t>
         </is>
       </c>
     </row>
@@ -4414,14 +4358,10 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>BACON SLICED HONEY CURED 18-20 CT | BACON SHINGLE C/C 18/20 HNY</t>
-        </is>
-      </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>Honey-cured sliced bacon, 18-20 slices per pound; honey-cured shingle bacon, 18-20 pieces per pound.</t>
-        </is>
-      </c>
+          <t>BACON SLICED HONEY CURED 18-20 CT BACON SHINGLE C/C 18/20 HNY</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -4431,7 +4371,7 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>BACON SLICED HONEY CURED SHINGLE 14-16 CT | BACON SHINGLE C/C 14/16 HNY</t>
+          <t>BACON SLICED HONEY CURED SHINGLE 14-16 CT BACON SHINGLE C/C 14/16 HNY</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -4448,12 +4388,12 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>BACON SLICED HONEY CURED 10-12 CT | BACON SHINGLE C/C 10/12 HNY</t>
+          <t>BACON SLICED HONEY CURED 10-12 CT BACON SHINGLE C/C 10/12 HNY</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Honey-cured sliced bacon, 10-12 slices per pound; honey-cured shingle bacon, 10-12 slices per pound</t>
+          <t>Honey-cured sliced bacon, 10-12 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4465,7 +4405,7 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLE SMOKED GAS FLUSHED 10-12 CT | BACON SHINGLE C/C 10/12 APL GF</t>
+          <t>BACON SLICED APPLE SMOKED GAS FLUSHED 10-12 CT BACON SHINGLE C/C 10/12 APL GF</t>
         </is>
       </c>
       <c r="C246" t="inlineStr"/>
@@ -4478,10 +4418,14 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>BACON SLICED PEPPERED .1875 IN | BACON SHINGLE C/C 10/12 PPR</t>
-        </is>
-      </c>
-      <c r="C247" t="inlineStr"/>
+          <t>BACON SLICED PEPPERED .1875 IN BACON SHINGLE C/C 10/12 PPR</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Peppered sliced bacon, 10-12 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -4491,14 +4435,10 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD SMOKED 14-18 CT | BACON LAYFLAT C/C 14/18 APL GF</t>
-        </is>
-      </c>
-      <c r="C248" t="inlineStr">
-        <is>
-          <t>Applewood-smoked sliced bacon, 14-18 slices per pound, gluten-free, layflat</t>
-        </is>
-      </c>
+          <t>BACON SLICED APPLEWOOD SMOKED 14-18 CT BACON LAYFLAT C/C 14/18 APL GF</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -4508,7 +4448,7 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>BACON SLICED HONEY CURED LAYOUT 14-16 CT | BACON LAYFLAT C/C 14/16 HNY</t>
+          <t>BACON SLICED HONEY CURED LAYOUT 14-16 CT BACON LAYFLAT C/C 14/16 HNY</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
@@ -4525,12 +4465,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>BACON SLICED SUGAR CURED 14-16 CT | BACON SHINGLE C/C 14/16 SGR</t>
+          <t>BACON SLICED SUGAR CURED 14-16 CT BACON SHINGLE C/C 14/16 SGR</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Sugar-cured sliced bacon, 14-16 slices per pound, and sugar-cured shingle</t>
+          <t>Sugar-cured sliced bacon, 14-16 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4542,7 +4482,7 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>BACON SLICED CENTER CUT 8-10 CT | BACON SHINGLE C/C 8/10 HNY GF</t>
+          <t>BACON SLICED CENTER CUT 8-10 CT BACON SHINGLE C/C 8/10 HNY GF</t>
         </is>
       </c>
       <c r="C251" t="inlineStr"/>
@@ -4555,12 +4495,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>BACON SLICED LAYFLAT 14-16 CT | BACON LAYFLAT 14/16CT</t>
+          <t>BACON SLICED LAYFLAT 14-16 CT BACON LAYFLAT 14/16CT</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Sliced bacon, 14-16 slices per pound, layflat</t>
+          <t>Sliced layflat bacon, 14-16 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -4572,10 +4512,14 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD SMOKED 14-16 CT | BACON LAYFLAT C/C 14/16 APL FZ</t>
-        </is>
-      </c>
-      <c r="C253" t="inlineStr"/>
+          <t>BACON SLICED APPLEWOOD SMOKED 14-16 CT BACON LAYFLAT C/C 14/16 APL FZ</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Frozen sliced applewood-smoked bacon, 14-16 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -4585,12 +4529,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>BACON SLICED COOKED 10-12 CT | BACON PRECOOKED SLI THICK 2XX</t>
+          <t>BACON SLICED COOKED 10-12 CT BACON PRECOOKED SLI THICK 2XX</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 10-12 slices per pound, thick cut</t>
+          <t>Fully cooked thick sliced bacon, 10-12 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4546,7 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>BACON SLICED SHINGLE 12-14 CT | BACON SHINGLE C/C 12/14 HNY</t>
+          <t>BACON SLICED SHINGLE 12-14 CT BACON SHINGLE C/C 12/14 HNY</t>
         </is>
       </c>
       <c r="C255" t="inlineStr"/>
@@ -4615,7 +4559,7 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>WRGHT 14/18 BACN 30 LB14/18 BULK BACON NATURAL HICKORY SMOKED, SLICED.  30# | BACON HCKRY SMKD SLI 14/18CT</t>
+          <t>WRGHT 14/18 BACN 30 LB14/18 BULK BACON NATURAL HICKORY SMOKED, SLICED. 30 BACON HCKRY SMKD SLI 14/18CT</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
@@ -4632,10 +4576,14 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 12-14 CT | BACON SHINGLE C/C 12/14 APL GF</t>
-        </is>
-      </c>
-      <c r="C257" t="inlineStr"/>
+          <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 12-14 CT BACON SHINGLE C/C 12/14 APL GF</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Gluten-free applewood-smoked sliced bacon, 12-14 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -4645,12 +4593,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>BACON SLICED SLAB COOKED | BACON PRECOOKED SLAB SLI REG</t>
+          <t>BACON SLICED SLAB COOKED BACON PRECOOKED SLAB SLI REG</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Fully cooked sliced slab bacon, regular slice size</t>
+          <t>Pre-cooked sliced slab bacon, regular thickness</t>
         </is>
       </c>
     </row>
@@ -4662,7 +4610,7 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>BACON SLICED SUGAR CURED LAYOUT 10-12 CT | BACON LAYER 10/12 SUGAR CURED</t>
+          <t>BACON SLICED SUGAR CURED LAYOUT 10-12 CT BACON LAYER 10/12 SUGAR CURED</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -4679,12 +4627,12 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 10-14 CT | BACON LAYFLAT C/C 10/14 APL GF</t>
+          <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 10-14 CT BACON LAYFLAT C/C 10/14 APL GF</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 10-14 slices per pound, layflat, gluten-free</t>
+          <t>Gluten-free applewood-smoked sliced bacon, 10-14 slices</t>
         </is>
       </c>
     </row>
@@ -4696,10 +4644,14 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>BACON CHIP CUBED REGULAR .375X.375 | BACON  PORK REAL DCD .38</t>
-        </is>
-      </c>
-      <c r="C261" t="inlineStr"/>
+          <t>BACON CHIP CUBED REGULAR .375X.375 BACON PORK REAL DCD .38</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Cubed bacon, 0.375 × 0.375‑inch pieces.</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -4709,7 +4661,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>BACON CHIP CUBED REGULAR .375X.375 | BACON CHIP 3/8CKD DICED REG</t>
+          <t>BACON CHIP CUBED REGULAR .375X.375 BACON CHIP 3/8CKD DICED REG</t>
         </is>
       </c>
       <c r="C262" t="inlineStr"/>
@@ -4722,12 +4674,12 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>25365555 SYSCO PRECKD 32/36 | BACON PRECOOKED REGULAR SLICE | BACON PRECOOKED SLICED 32/36</t>
+          <t>25365555 SYSCO PRECKD 32/36 BACON PRECOOKED REGULAR SLICE BACON PRECOOKED SLICED 32/36</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Pre-cooked sliced bacon, 32-36 slices per pound</t>
+          <t>Fully cooked sliced bacon, 32-36 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -4739,12 +4691,12 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>FRZ 5757184 REL SLAB 14/18 15# | BACON SLAB 14/18 SMOKED | BACON 14/18 CT SLAB SLICED</t>
+          <t>FRZ 5757184 REL SLAB 14/18 15 BACON SLAB 14/18 SMOKED BACON 14/18 CT SLAB SLICED</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Frozen sliced smoked slab bacon, 14-18 slices per pound</t>
+          <t>Frozen smoked sliced bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4756,10 +4708,14 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>5886579 CLASSIC GRL/FRSH 14/18 | BACON LAYFLAT C/C 14/18 SMK GF</t>
-        </is>
-      </c>
-      <c r="C265" t="inlineStr"/>
+          <t>5886579 CLASSIC GRL/FRSH 14/18 BACON LAYFLAT C/C 14/18 SMK GF</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Gluten-free smoked sliced bacon, 14-18 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -4769,7 +4725,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>BACON APPLEWOOD SMOKED SLAB | BACON SLAB APPLEWOOD SMK FZN</t>
+          <t>BACON APPLEWOOD SMOKED SLAB BACON SLAB APPLEWOOD SMK FZN</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -4786,7 +4742,7 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>BACON APPLEWOOD SMOKED SLAB | BACON SLAB APPLE SMOKED</t>
+          <t>BACON APPLEWOOD SMOKED SLAB BACON SLAB APPLE SMOKED</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
@@ -4803,7 +4759,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>BACON SLICED WESTERN JEWEL .25 IN | BACON SHINGLE C/C 7/9 HNY GF</t>
+          <t>BACON SLICED WESTERN JEWEL .25 IN BACON SHINGLE C/C 7/9 HNY GF</t>
         </is>
       </c>
       <c r="C268" t="inlineStr"/>
@@ -4816,7 +4772,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 9 13 SLICES PER POUND | BACON APPLWD SMKD 9/13</t>
+          <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 9 13 SLICES PER POUND BACON APPLWD SMKD 9/13</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
@@ -4833,12 +4789,12 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>GR BACON  9-11 CT 1/15 LB | BACON LAYFLAT 9/11CT FRZN</t>
+          <t>GR BACON 9-11 CT 1/15 LB BACON LAYFLAT 9/11CT FRZN</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Frozen layflat sliced bacon, 9-11 slices per pound</t>
+          <t>Frozen sliced bacon, 9-11 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4850,14 +4806,10 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>BACON CUBED COOKED .75X.75 | BACON DICED PRCK 3/4</t>
-        </is>
-      </c>
-      <c r="C271" t="inlineStr">
-        <is>
-          <t>Cooked cubed bacon, 0.75 × 0.75‑inch pieces, and diced pork bacon, 3/4‑inch pieces.</t>
-        </is>
-      </c>
+          <t>BACON CUBED COOKED .75X.75 BACON DICED PRCK 3/4</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -4867,14 +4819,10 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>FRZ JR APPLEWOOD 14/18 SLAB | BACON SLICED APLWD SLAB 14/18</t>
-        </is>
-      </c>
-      <c r="C272" t="inlineStr">
-        <is>
-          <t>Frozen applewood-smoked slab bacon, 14-18 slices per pound.</t>
-        </is>
-      </c>
+          <t>FRZ JR APPLEWOOD 14/18 SLAB BACON SLICED APLWD SLAB 14/18</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr"/>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -4889,7 +4837,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Bacon pieces, 3/8-inch size</t>
+          <t>Bacon pieces, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -4901,12 +4849,12 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>BACON SLAB SLI 1/4" APPLEWOOD | BACON SLAB SLI 1/4 APLWD</t>
+          <t>BACON SLAB SLI 1/4 APPLEWOOD BACON SLAB SLI 1/4 APLWD</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced slab bacon, 1/4‑inch slices.</t>
+          <t>Applewood-smoked sliced slab bacon, 1/4‑inch thickness.</t>
         </is>
       </c>
     </row>
@@ -4918,10 +4866,14 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE PECANWOOD SMOKED BACON 13 17 SLICES PER POUND | BACON LAYFLAT C/C 13/17 PCN GF</t>
-        </is>
-      </c>
-      <c r="C275" t="inlineStr"/>
+          <t>OLD SMOKEHOUSE PECANWOOD SMOKED BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 PCN GF</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Pecanwood-smoked sliced bacon, 13-17 slices per pound, gluten-free, lay</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -4931,7 +4883,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>OLD SMOKEHOUSE PECANWOOD SMOKED BACON 13 17 SLICES PER POUND | BACON L/O 13/17 PECAN SMKD</t>
+          <t>OLD SMOKEHOUSE PECANWOOD SMOKED BACON 13 17 SLICES PER POUND BACON L/O 13/17 PECAN SMKD</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -4948,7 +4900,7 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>BACON COOKED DICED .5 IN | BACON TOPPING CKD 1/2IN DCD | BACON TOPPING DICED COOKED 1/2""</t>
+          <t>BACON COOKED DICED .5 IN BACON TOPPING CKD 1/2IN DCD BACON TOPPING DICED COOKED 1/2</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -4965,7 +4917,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>10 LB CWA BULK BACN10 LBS SLICED BACON (PORK) BULK | BACON SLAB RANDOM SMOKED #2</t>
+          <t>10 LB CWA BULK BACN10 LBS SLICED BACON (PORK) BULK BACON SLAB RANDOM SMOKED 2</t>
         </is>
       </c>
       <c r="C278" t="inlineStr"/>
@@ -4978,7 +4930,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>WRGHT FPK BACN 15 LB FZNATURAL HICKORY SMOKED REGULAR FLAT PACK BACON. 15# FROZEN | BACON LAYFLAT 14/18 CT</t>
+          <t>WRGHT FPK BACN 15 LB FZNATURAL HICKORY SMOKED REGULAR FLAT PACK BACON. 15 FROZEN BACON LAYFLAT 14/18 CT</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -4995,12 +4947,12 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>HORMEL BACON 1 PERFECTLY COOKED 20/24 STYLE BACON | BACON SMKD CKD 20/24</t>
+          <t>HORMEL BACON 1 PERFECTLY COOKED 20/24 STYLE BACON BACON SMKD CKD 20/24</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 20-24 slices per pound.</t>
+          <t>Fully cooked smoked sliced bacon, 20-24 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5012,12 +4964,12 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>HORMEL BACON 1 PERFECTLY COOKED 20/24 STYLE BACON | BACON PRECOOKED BCN1 20/24</t>
+          <t>HORMEL BACON 1 PERFECTLY COOKED 20/24 STYLE BACON BACON PRECOOKED BCN1 20/24</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 20-24 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 20-24 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5029,7 +4981,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>PRE-COOK BACON RND 2/2 LB | BACON PRECOOKED RND SLI</t>
+          <t>PRE-COOK BACON RND 2/2 LB BACON PRECOOKED RND SLI</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -5046,7 +4998,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>APPLEWOOD EXTRA SMK GF SLAB | BACON SLAB APLEWD 14/16CT</t>
+          <t>APPLEWOOD EXTRA SMK GF SLAB BACON SLAB APLEWD 14/16CT</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -5063,7 +5015,7 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>SYS 0855086 SLAB 14/16SYSCO CLASSIC BACON CENTER CUT SHINGLE 14/16 CT HONEY 1/15 LBS. | BACON SHINGLE C/C 14/16 HNY GF</t>
+          <t>SYS 0855086 SLAB 14/16SYSCO CLASSIC BACON CENTER CUT SHINGLE 14/16 CT HONEY 1/15 LBS. BACON SHINGLE C/C 14/16 HNY GF</t>
         </is>
       </c>
       <c r="C284" t="inlineStr"/>
@@ -5076,12 +5028,12 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>SYS 0855195 HON 10/12SYSCO CLASSIC BACON CENTER CUT SHINGLE HONEY 10/12 CT 1/15 LB | BACON SHINGLE C/C 10/12 HNY GF</t>
+          <t>SYS 0855195 HON 10/12SYSCO CLASSIC BACON CENTER CUT SHINGLE HONEY 10/12 CT 1/15 LB BACON SHINGLE C/C 10/12 HNY GF</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Honey-flavored gluten-free</t>
+          <t>Raw gluten-free honey-flavored shingle bacon, 10-12 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5093,7 +5045,7 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>BACON SLICED DEEP APPLEWOOD SMOKED 16-18 CT | BACON SLICED DP AP/SMK 16/18</t>
+          <t>BACON SLICED DEEP APPLEWOOD SMOKED 16-18 CT BACON SLICED DP AP/SMK 16/18</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -5110,7 +5062,7 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>HORMEL BACON 1 PERFECTLY COOKED 13/17 STYLE BACON | BACON PRECOOKED C/C 13/17 BCN1</t>
+          <t>HORMEL BACON 1 PERFECTLY COOKED 13/17 STYLE BACON BACON PRECOOKED C/C 13/17 BCN1</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
@@ -5127,12 +5079,12 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>HORMEL BACON 1 PERFECTLY COOKED 13/17 STYLE BACON | BACON1 13/17 CT.</t>
+          <t>HORMEL BACON 1 PERFECTLY COOKED 13/17 STYLE BACON BACON1 13/17 CT.</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 13-17 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5144,7 +5096,7 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>HORMEL BACON 1 PERFECTLY COOKED 13/17 STYLE BACON | BACON SMKD CKD 13-17</t>
+          <t>HORMEL BACON 1 PERFECTLY COOKED 13/17 STYLE BACON BACON SMKD CKD 13-17</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
@@ -5161,7 +5113,7 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>HORMEL BACON 1 PERFECTLY COOKED 18/22 STYLE BACON | BACON PRECOOKED BACON1 18/22</t>
+          <t>HORMEL BACON 1 PERFECTLY COOKED 18/22 STYLE BACON BACON PRECOOKED BACON1 18/22</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -5178,12 +5130,12 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>HORMEL BACON 1 PERFECTLY COOKED 18/22 STYLE BACON | BACON SMKD CKD 18-22</t>
+          <t>HORMEL BACON 1 PERFECTLY COOKED 18/22 STYLE BACON BACON SMKD CKD 18-22</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Fully cooked smoked sliced bacon, 18-22 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5195,12 +5147,12 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>HORMEL BACON 1 PERFECTLY COOKED 18/22 STYLE BACON | BACON  PORK 144 CT REF 18</t>
+          <t>HORMEL BACON 1 PERFECTLY COOKED 18/22 STYLE BACON BACON PORK 144 CT REF 18</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5212,12 +5164,12 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>GFS SLCD BACN 18/22 | BACON SLCD 18-22CT FRSH</t>
+          <t>GFS SLCD BACN 18/22 BACON SLCD 18-22CT FRSH</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Fresh sliced gluten-free bacon, 18-22 slices per pound.</t>
+          <t>Fresh sliced gluten-free bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5229,12 +5181,12 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>BACON SLICED RAW APLWD | BACON SLICED RAW APLWD 9/13 SL</t>
+          <t>BACON SLICED RAW APLWD BACON SLICED RAW APLWD 9/13 SL</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Raw sliced applewood-smoked bacon, 9-13 slices per pound, layflat</t>
+          <t>Raw sliced applewood-smoked bacon, 9-13 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5198,7 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>FARMLAND HEAT N EAT SL BACON | BACON SLICED FC</t>
+          <t>FARMLAND HEAT N EAT SL BACON BACON SLICED FC</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -5263,12 +5215,12 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>FARMLAND HEAT N EAT SL BACON | BACON  PORK 150 CT SLCD L</t>
+          <t>FARMLAND HEAT N EAT SL BACON BACON PORK 150 CT SLCD L</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Sliced bacon, 150 slices per pound, layflat</t>
+          <t>Sliced pork bacon, 150 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5232,7 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>FARMLAND HEAT N EAT SL BACON | BACON PRECOOKED SLI HEAT &amp; EAT</t>
+          <t>FARMLAND HEAT N EAT SL BACON BACON PRECOOKED SLI HEAT &amp; EAT</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -5297,7 +5249,7 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>FARMLAND HEAT N EAT SL BACON | BACON SLCD CKD</t>
+          <t>FARMLAND HEAT N EAT SL BACON BACON SLCD CKD</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -5314,7 +5266,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>BCN,FL,BM,2/1.25#,300C,FLCK,SLCD | BACON LAYFLAT PRCK</t>
+          <t>BCN,FL,BM,2/1.25 ,300C,FLCK,SLCD BACON LAYFLAT PRCK</t>
         </is>
       </c>
       <c r="C299" t="inlineStr"/>
@@ -5327,7 +5279,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>BCN,FL,BM,2/1.25#,300C,FLCK,SLCD | BACON FULLY CKD HEAT N SERVE</t>
+          <t>BCN,FL,BM,2/1.25 ,300C,FLCK,SLCD BACON FULLY CKD HEAT N SERVE</t>
         </is>
       </c>
       <c r="C300" t="inlineStr"/>
@@ -5340,14 +5292,10 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>BCN,FL,BM,2/1.25#,300C,FLCK,SLCD | BACON LAID-OUT FC</t>
-        </is>
-      </c>
-      <c r="C301" t="inlineStr">
-        <is>
-          <t>Fully cooked sliced bacon, layflat</t>
-        </is>
-      </c>
+          <t>BCN,FL,BM,2/1.25 ,300C,FLCK,SLCD BACON LAID-OUT FC</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr"/>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -5357,7 +5305,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>BACN,SS,SILVER,18/22,15#,Z | BACON LAYFLAT 18/22</t>
+          <t>BACN,SS,SILVER,18/22,15 ,Z BACON LAYFLAT 18/22</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -5374,12 +5322,12 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>BACN,SS,SILVER,18/22,15#,Z | BACON  PORK 18-22 CT SLCD</t>
+          <t>BACN,SS,SILVER,18/22,15 ,Z BACON PORK 18-22 CT SLCD</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound</t>
+          <t>Sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5391,12 +5339,12 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>BCN,PCI,2/5#,1/2",TPG,MCRW | BACON TOPPING CKD 1/2 IN</t>
+          <t>BCN,PCI,2/5 ,1/2 ,TPG,MCRW BACON TOPPING CKD 1/2 IN</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 1/2-inch pieces</t>
+          <t>Fully cooked bacon bits, 1/2-inch pieces</t>
         </is>
       </c>
     </row>
@@ -5408,10 +5356,14 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>BCN,JM,APLWD,14/17/SLC,GF,1/15# | BACON 14/16 APPLEWOOD GAS FLSHD RAW</t>
-        </is>
-      </c>
-      <c r="C305" t="inlineStr"/>
+          <t>BCN,JM,APLWD,14/17/SLC,GF,1/15 BACON 14/16 APPLEWOOD GAS FLSHD RAW</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Raw gluten-free applewood-smoked sliced bacon, 14-17 slices per pound.</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -5421,14 +5373,10 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>BCN,JM,APLWD,14/17/SLC,GF,1/15# | BACON LAYFLAT 14/17 APPLE G | BACON 14/17 CT APPLEWOOD SMOKED SINGLE SHINGLE</t>
-        </is>
-      </c>
-      <c r="C306" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 14-17 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>BCN,JM,APLWD,14/17/SLC,GF,1/15 BACON LAYFLAT 14/17 APPLE G BACON 14/17 CT APPLEWOOD SMOKED SINGLE SHINGLE</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr"/>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -5438,7 +5386,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>BCN,JM,APLWD,14/17/SLC,GF,1/15# | BACON LAYFLAT 14/17 APLE GF FZ</t>
+          <t>BCN,JM,APLWD,14/17/SLC,GF,1/15 BACON LAYFLAT 14/17 APLE GF FZ</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -5455,7 +5403,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>BCN,JM,APLWD,14/17/SLC,GF,1/15# | BACON 14/17 CT APPLEWOOD SMOKED SINGLE SHINGLE</t>
+          <t>BCN,JM,APLWD,14/17/SLC,GF,1/15 BACON 14/17 CT APPLEWOOD SMOKED SINGLE SHINGLE</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -5472,7 +5420,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>BCN,FL,2/2.5#,150C,.5Z,RW | BACON PRECOOKED SLI THICK DLX</t>
+          <t>BCN,FL,2/2.5 ,150C,.5Z,RW BACON PRECOOKED SLI THICK DLX</t>
         </is>
       </c>
       <c r="C309" t="inlineStr"/>
@@ -5485,12 +5433,12 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>BCN,PL,FL,BITS,FINE,2/5# | BACON  PORK REAL CHIP DCD</t>
+          <t>BCN,PL,FL,BITS,FINE,2/5 BACON PORK REAL CHIP DCD</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Frozen fine diced bacon bits, 2/5‑pound.</t>
+          <t>Frozen real pork bacon bits, fine diced, 2/5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5450,7 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>BCN,PL,FL,BITS,FINE,2/5# | BACON BIT FINE REAL | BACON BITS FINE FC</t>
+          <t>BCN,PL,FL,BITS,FINE,2/5 BACON BIT FINE REAL BACON BITS FINE FC</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -5519,12 +5467,12 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>BCN,PL,FL,BITS,FINE,2/5# | BACON BIT CKD 3/16IN</t>
+          <t>BCN,PL,FL,BITS,FINE,2/5 BACON BIT CKD 3/16IN</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Fully cooked fine bacon bits, 3/16‑inch pieces</t>
+          <t>Fully cooked bacon bits, 3/16‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -5536,12 +5484,12 @@
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>BACN,DICED,RDY TO COOK,3/10#,Z | BACON DICED ENDS &amp; PIECES RAW 1/2""</t>
+          <t>BACN,DICED,RDY TO COOK,3/10 ,Z BACON DICED ENDS &amp; PIECES RAW 1/2</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Raw diced bacon ends and pieces, 1/2‑inch pieces</t>
+          <t>Raw diced bacon,</t>
         </is>
       </c>
     </row>
@@ -5553,12 +5501,12 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>BACN,DICED,RDY TO COOK,2/5#,Z | BACON END &amp; PCS DICED | BACON DICED READY TO COOK FROZEN</t>
+          <t>BACN,DICED,RDY TO COOK,2/5 ,Z BACON END &amp; PCS DICED BACON DICED READY TO COOK FROZEN</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Frozen ready-to-cook diced bacon</t>
+          <t>Frozen ready-to-cook diced bacon, 2/5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -5570,7 +5518,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>BCN,PL,FL,2C,5#,BITS | BACON BIT FC 1/4"" | BACON BIT CKD REAL</t>
+          <t>BCN,PL,FL,2C,5 ,BITS BACON BIT FC 1/4 BACON BIT CKD REAL</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -5587,7 +5535,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>BCN,GC,APLWD,SMKD,2/5#,TPG | BACON TOPPING APPLEWOOD SMOKED FC 3/8"" | BACON TOPPING FULLY CKD</t>
+          <t>BCN,GC,APLWD,SMKD,2/5 ,TPG BACON TOPPING APPLEWOOD SMOKED FC 3/8 BACON TOPPING FULLY CKD</t>
         </is>
       </c>
       <c r="C316" t="inlineStr"/>
@@ -5600,14 +5548,10 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>BACN,SS,LS,GM,18/22,GF,15#,Z | BACON LO SOD SLCD 18/22</t>
-        </is>
-      </c>
-      <c r="C317" t="inlineStr">
-        <is>
-          <t>Gluten-free, low-sodium sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>BACN,SS,LS,GM,18/22,GF,15 ,Z BACON LO SOD SLCD 18/22</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -5617,14 +5561,10 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>BACN,SS,LS,GM,18/22,GF,15#,Z | BACON LAYFLAT C/C 18/22 LS</t>
-        </is>
-      </c>
-      <c r="C318" t="inlineStr">
-        <is>
-          <t>Gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>BACN,SS,LS,GM,18/22,GF,15 ,Z BACON LAYFLAT C/C 18/22 LS</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -5634,7 +5574,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>BACN,SS,APLWD LOG,SMFD-PLAT,10/14,GF,15# | BACON LAYFLAT APL LOG 10/14 GF</t>
+          <t>BACN,SS,APLWD LOG,SMFD-PLAT,10/14,GF,15 BACON LAYFLAT APL LOG 10/14 GF</t>
         </is>
       </c>
       <c r="C319" t="inlineStr"/>
@@ -5647,7 +5587,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>BACN,SS,APLWD LOG,SMFD-PLAT,10/14,GF,15# | BACON L/O 10-14CT APPLWD LOG SMKD | BACON 10/14 CT LAYFLAT APPLEWOOD LOG SMOKED</t>
+          <t>BACN,SS,APLWD LOG,SMFD-PLAT,10/14,GF,15 BACON L/O 10-14CT APPLWD LOG SMKD BACON 10/14 CT LAYFLAT APPLEWOOD LOG SMOKED</t>
         </is>
       </c>
       <c r="C320" t="inlineStr"/>
@@ -5660,14 +5600,10 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>BCN,FL,RMP,1/15#,SS,GRDOUT,FZ | BACON 18/22 CT SINGLE SLICE IRREGULAR #2</t>
-        </is>
-      </c>
-      <c r="C321" t="inlineStr">
-        <is>
-          <t>Frozen sliced bacon, 18-22 slices per pound, irregular cut</t>
-        </is>
-      </c>
+          <t>BCN,FL,RMP,1/15 ,SS,GRDOUT,FZ BACON 18/22 CT SINGLE SLICE IRREGULAR 2</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -5677,12 +5613,12 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>BACN,SS,SM,14/18,15#,Z | BACON SINGLE SLI 14/18 FRZN | BACON 14/18 CT SINGLE SLICE 70247158247</t>
+          <t>BACN,SS,SM,14/18,15 ,Z BACON SINGLE SLI 14/18 FRZN BACON 14/18 CT SINGLE SLICE 70247158247</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, 14-18 slices per pound.</t>
+          <t>Frozen smoked sliced bacon,</t>
         </is>
       </c>
     </row>
@@ -5694,7 +5630,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>BACN,SS,SM,14/18,15#,Z | BACON 14/18 CT SINGLE SLICE 70247158247</t>
+          <t>BACN,SS,SM,14/18,15 ,Z BACON 14/18 CT SINGLE SLICE 70247158247</t>
         </is>
       </c>
       <c r="C323" t="inlineStr"/>
@@ -5707,7 +5643,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>BACN,SS,SM,14/18,15#,Z | 14/18CT RAW LAYOUT BACON</t>
+          <t>BACN,SS,SM,14/18,15 ,Z 14/18CT RAW LAYOUT BACON</t>
         </is>
       </c>
       <c r="C324" t="inlineStr"/>
@@ -5720,7 +5656,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>BCN,FL,SMD,1/15#,18-22SL/#,FZ | BACON SLICED 18-22 LO</t>
+          <t>BCN,FL,SMD,1/15 ,18-22SL/ ,FZ BACON SLICED 18-22 LO</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -5737,14 +5673,10 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>BCN,FL,SMD,1/15#,18-22SL/#,FZ | BACON 18/22 CT LAYOUT SINGLE SLICED GLUTEN-FREE | BACON LAYOUT 18/22 SLVR MEDAL</t>
-        </is>
-      </c>
-      <c r="C326" t="inlineStr">
-        <is>
-          <t>Frozen gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>BCN,FL,SMD,1/15 ,18-22SL/ ,FZ BACON 18/22 CT LAYOUT SINGLE SLICED GLUTEN-FREE BACON LAYOUT 18/22 SLVR MEDAL</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -5754,12 +5686,12 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>BCN,FL,SMD,1/15#,18-22SL/#,FZ | BACON 18/22 CT LAYOUT SINGLE SLICED GLUTEN-FREE | BACON LAID-OUT 18/22 SLVR</t>
+          <t>BCN,FL,SMD,1/15 ,18-22SL/ ,FZ BACON 18/22 CT LAYOUT SINGLE SLICED GLUTEN-FREE BACON LAID-OUT 18/22 SLVR</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Frozen gluten-free smoked</t>
+          <t>Frozen gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -5771,14 +5703,10 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>BACN,SS,SM,22/26,15#,Z | BACON LAYOUT SLI 22/26 FRZN</t>
-        </is>
-      </c>
-      <c r="C328" t="inlineStr">
-        <is>
-          <t>Frozen smoked sliced bacon, 22-26 slices per pound, layflat</t>
-        </is>
-      </c>
+          <t>BACN,SS,SM,22/26,15 ,Z BACON LAYOUT SLI 22/26 FRZN</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -5788,12 +5716,12 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>BACN,SS,GM,14/18,GF,15# | BACON LAYFLAT 14/18 GOLD MEDL</t>
+          <t>BACN,SS,GM,14/18,GF,15 BACON LAYFLAT 14/18 GOLD MEDL</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Gluten-free</t>
+          <t>Gluten-free sliced bacon, 14-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -5805,14 +5733,10 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>BACN,SS,SM,18/22,GF,15# | BACON SSL 18-22 | BACON 18/22 CT SINGLE SLICE GAS FLUSHED</t>
-        </is>
-      </c>
-      <c r="C330" t="inlineStr">
-        <is>
-          <t>Gluten-free smoked sliced bacon, 18-22 slices per pound.</t>
-        </is>
-      </c>
+          <t>BACN,SS,SM,18/22,GF,15 BACON SSL 18-22 BACON 18/22 CT SINGLE SLICE GAS FLUSHED</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -5822,12 +5746,12 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>BACN,HRI,NW-SM,10/14,GF,15# | BACON 10/14 CT HRI NORTHWEST GLUTEN-FREE</t>
+          <t>BACN,HRI,NW-SM,10/14,GF,15 BACON 10/14 CT HRI NORTHWEST GLUTEN-FREE</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Gluten-free Northwest-smoked sliced bacon, 10-14</t>
+          <t>Northwest-smoked sliced bacon, 10-14 slices per pound, gluten-free</t>
         </is>
       </c>
     </row>
@@ -5839,10 +5763,14 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>BACN,SS,APL-CDR,GM,18/22,GF,15# | BACON 18/22 CT APPLE-CIDER SINGLE SLICE</t>
-        </is>
-      </c>
-      <c r="C332" t="inlineStr"/>
+          <t>BACN,SS,APL-CDR,GM,18/22,GF,15 BACON 18/22 CT APPLE-CIDER SINGLE SLICE</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Gluten-free apple-cider sliced bacon, 18-22 slices per pound.</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -5852,7 +5780,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>BACN,SS,APL-CDR,GM,14/18,GF,15# | BACON L/O APPL CIDER SMKD 14/18CT | BACON 14/18 CT APPLE CIDER SINGLE SLICE</t>
+          <t>BACN,SS,APL-CDR,GM,14/18,GF,15 BACON L/O APPL CIDER SMKD 14/18CT BACON 14/18 CT APPLE CIDER SINGLE SLICE</t>
         </is>
       </c>
       <c r="C333" t="inlineStr"/>
@@ -5865,7 +5793,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>BACN,SS,APL-CDR,GM,14/18,GF,15# | BACON LAYFLAT CC 14/18 APL CDR</t>
+          <t>BACN,SS,APL-CDR,GM,14/18,GF,15 BACON LAYFLAT CC 14/18 APL CDR</t>
         </is>
       </c>
       <c r="C334" t="inlineStr"/>
@@ -5878,7 +5806,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>BACN,SS,APL-CDR,GM,10/14,GF,15# | BACON L/O APPL CIDER SMKD 10-14 | BACON 10/14 CT APPLE-CIDER SINGLE SLICE</t>
+          <t>BACN,SS,APL-CDR,GM,10/14,GF,15 BACON L/O APPL CIDER SMKD 10-14 BACON 10/14 CT APPLE-CIDER SINGLE SLICE</t>
         </is>
       </c>
       <c r="C335" t="inlineStr"/>
@@ -5891,7 +5819,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>BACN,SS,APL-CDR,GM,10/14,GF,15# | BACON LAYFLAT EE 10/14 APL CDR | BACON 10/14 CT APPLE-CIDER SINGLE SLICE</t>
+          <t>BACN,SS,APL-CDR,GM,10/14,GF,15 BACON LAYFLAT EE 10/14 APL CDR BACON 10/14 CT APPLE-CIDER SINGLE SLICE</t>
         </is>
       </c>
       <c r="C336" t="inlineStr"/>
@@ -5904,12 +5832,12 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>BACN,ENDS&amp;PCS,15#,Z | BACON ENDS &amp; PIECES</t>
+          <t>BACN,ENDS&amp;PCS,15 ,Z BACON ENDS &amp; PIECES</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Ends and pieces bacon</t>
+          <t>Bacon ends and pieces</t>
         </is>
       </c>
     </row>
@@ -5921,10 +5849,14 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>BACN,SS,APLWD SMKD,SM,14/18,GF,15#,Z | BACON APPLEWOOD SSL 14/18</t>
-        </is>
-      </c>
-      <c r="C338" t="inlineStr"/>
+          <t>BACN,SS,APLWD SMKD,SM,14/18,GF,15 ,Z BACON APPLEWOOD SSL 14/18</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Gluten-free applewood-smoked sliced bacon, 14-18 slices per pound.</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -5934,14 +5866,10 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>BACN,SS,APLWD SMKD,SM,14/18,GF,15#,Z | BACON 14/18 CT APPLEWOOD SMOKED SINGLE SLICE | BACON SINGLE SLI APLWD 14/18</t>
-        </is>
-      </c>
-      <c r="C339" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 14-18 slices per pound.</t>
-        </is>
-      </c>
+          <t>BACN,SS,APLWD SMKD,SM,14/18,GF,15 ,Z BACON 14/18 CT APPLEWOOD SMOKED SINGLE SLICE BACON SINGLE SLI APLWD 14/18</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -5951,12 +5879,12 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>BACN,SS,APLWD SMKD,SM,18/22,GF,15#,Z | BACON SSL APPLWD SMKD 18-22CT</t>
+          <t>BACN,SS,APLWD SMKD,SM,18/22,GF,15 ,Z BACON SSL APPLWD SMKD 18-22CT</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 18-22 slices per pound.</t>
+          <t>Applewood-smoked sliced gluten-free bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5968,7 +5896,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>BACN,SS,APLWD SMKD,SM,18/22,GF,15#,Z | BACON LAYFLAT CC 18/22 APL SMK</t>
+          <t>BACN,SS,APLWD SMKD,SM,18/22,GF,15 ,Z BACON LAYFLAT CC 18/22 APL SMK</t>
         </is>
       </c>
       <c r="C341" t="inlineStr"/>
@@ -5981,10 +5909,14 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>BACN,SS,UNCURED,SM,13/17,GF,15# | BACON SINGLE SLI UNCURE 13/17</t>
-        </is>
-      </c>
-      <c r="C342" t="inlineStr"/>
+          <t>BACN,SS,UNCURED,SM,13/17,GF,15 BACON SINGLE SLI UNCURE 13/17</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Uncured sliced bacon, 13-17 slices per pound, gluten-free.</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -5994,7 +5926,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>BACON APPLEWOOD SMOKED SLAB | BACON SLAB APPLEWOOD SMOKED</t>
+          <t>BACON APPLEWOOD SMOKED SLAB BACON SLAB APPLEWOOD SMOKED</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -6011,7 +5943,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>HORMEL BACON 1 ALL NATURAL PERFECTLY COOKED 13/17 STYLE BACON | BACON PRCK C/C 13/17 BCN1 NAT</t>
+          <t>HORMEL BACON 1 ALL NATURAL PERFECTLY COOKED 13/17 STYLE BACON BACON PRCK C/C 13/17 BCN1 NAT</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -6045,12 +5977,12 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>HORMEL BACON 1 ALL NATURAL PERFECTLY COOKED 18/22 STYLE BACON | BACON PRCK C/C 18/22 BCN1 NAT</t>
+          <t>HORMEL BACON 1 ALL NATURAL PERFECTLY COOKED 18/22 STYLE BACON BACON PRCK C/C 18/22 BCN1 NAT</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Fully cooked all-natural sliced bacon, 18-22 slices per pound.</t>
+          <t>Fully cooked all‑natural sliced bacon, 18‑22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -6062,12 +5994,12 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>3209653 BACN E&amp;P | BACON END &amp; PCS</t>
+          <t>3209653 BACN E&amp;P BACON END &amp; PCS</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Bacon end and pieces</t>
+          <t>Bacon ends and pieces.</t>
         </is>
       </c>
     </row>
@@ -6079,14 +6011,10 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>BACON TOPPING NAT CKD W COA | BACON  PORK BELLY REAL BI</t>
-        </is>
-      </c>
-      <c r="C348" t="inlineStr">
-        <is>
-          <t>Cooked pork belly bacon topping</t>
-        </is>
-      </c>
+          <t>BACON TOPPING NAT CKD W COA BACON PORK BELLY REAL BI</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -6096,12 +6024,12 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>BACON TOPPING NAT CKD W COA | BACON TOPPING NAT CKD W/COA</t>
+          <t>BACON TOPPING NAT CKD W COA BACON TOPPING NAT CKD W/COA</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Cooked natural bacon topping, with coating.</t>
+          <t>Fully cooked natural bacon topping</t>
         </is>
       </c>
     </row>
@@ -6113,12 +6041,12 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>BACON CANADIAN LOIN BONELESS | BACON CANADIAN APPLEWOOD</t>
+          <t>BACON CANADIAN LOIN BONELESS BACON CANADIAN APPLEWOOD</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Boneless Canadian loin bacon, applewood-smoked.</t>
+          <t>Applewood-smoked Canadian boneless loin bacon</t>
         </is>
       </c>
     </row>
@@ -6130,7 +6058,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>BACON SLICED LAYOUT 18-22 CT | BACON 18/22 CT LAYOUT HICKORY SMOKED | BACON L/O 18-22CT CC FZ</t>
+          <t>BACON SLICED LAYOUT 18-22 CT BACON 18/22 CT LAYOUT HICKORY SMOKED BACON L/O 18-22CT CC FZ</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -6147,12 +6075,12 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>BACON SLICED LAYOUT 18-22 CT | BACON L/O 18-22CT CC HRDWD SMKD FRSH | BACON 18/22 CT L/O FRESH</t>
+          <t>BACON SLICED LAYOUT 18-22 CT BACON L/O 18-22CT CC HRDWD SMKD FRSH BACON 18/22 CT L/O FRESH</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Fresh sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Fresh smoked sliced bacon, 18-</t>
         </is>
       </c>
     </row>
@@ -6164,7 +6092,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>BACON SLICED LAYOUT 14-18 CT | BACON L/O 14-18CT CC FRSH | BACON L/O 14-18CT FRSH | BACON 14/18 CT L/O FRESH</t>
+          <t>BACON SLICED LAYOUT 14-18 CT BACON L/O 14-18CT CC FRSH BACON L/O 14-18CT FRSH BACON 14/18 CT L/O FRESH</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -6181,10 +6109,14 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>BACON SLICED LAYOUT 22-26 CT | BACON L/O 22-26CT CC HICKORY SMKD FZ</t>
-        </is>
-      </c>
-      <c r="C354" t="inlineStr"/>
+          <t>BACON SLICED LAYOUT 22-26 CT BACON L/O 22-26CT CC HICKORY SMKD FZ</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Frozen hickory-smoked sliced bacon, 22-26 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -6194,7 +6126,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>BACON SLICED LAYOUT 14-18 CT | BACON 14/18 CT LAYOUT FZ | BACON L/O 14-18CT CC FZ</t>
+          <t>BACON SLICED LAYOUT 14-18 CT BACON 14/18 CT LAYOUT FZ BACON L/O 14-18CT CC FZ</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -6211,7 +6143,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>BACON SLICED LAYOUT 9-11 CT | BACON L/O 9-11CT CC FRSH | BACON 09/11 CT LAYOUT FRESH</t>
+          <t>BACON SLICED LAYOUT 9-11 CT BACON L/O 9-11CT CC FRSH BACON 09/11 CT LAYOUT FRESH</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -6228,12 +6160,12 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>BACON SLICED HONEY CURED CENTER CUT LAYFLAT 10-12 CT | BACON LAYFLAT C/C 10/12 HNY GF</t>
+          <t>BACON SLICED HONEY CURED CENTER CUT LAYFLAT 10-12 CT BACON LAYFLAT C/C 10/12 HNY GF</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Honey-cured center cut sliced bacon, 10-12 slices per pound, layflat, gluten-free</t>
+          <t>Honey-cured center cut sliced bacon, 10-12 slices per pound, gluten-free, layflat</t>
         </is>
       </c>
     </row>
@@ -6245,7 +6177,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>SIGNATURE GREAT RECIPE BACON 13 17 SLICES PER POUND | BACON LAYFLAT 13/17 CONTRL LBL</t>
+          <t>SIGNATURE GREAT RECIPE BACON 13 17 SLICES PER POUND BACON LAYFLAT 13/17 CONTRL LBL</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -6262,12 +6194,12 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>BACN E&amp;P 6/3 LB | BACON END &amp; PIECES</t>
+          <t>BACN E&amp;P 6/3 LB BACON END &amp; PIECES</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>Bacon end and pieces</t>
+          <t>Bacon ends and pieces</t>
         </is>
       </c>
     </row>
@@ -6279,12 +6211,12 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>SYSCO IMPERIAL PCK BAC 13/17 | BACON 13/17 CT PRECOOKED C/C DELUXE | BACON PRECOOKED C/C 14/18 DLUX</t>
+          <t>SYSCO IMPERIAL PCK BAC 13/17 BACON 13/17 CT PRECOOKED C/C DELUXE BACON PRECOOKED C/C 14/18 DLUX</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 13-17 or 14-18 slices per pound</t>
+          <t>Fully cooked sliced bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -6296,12 +6228,12 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>HORMEL REGULAR COOKED ALL NATURAL 0 375 INCH BACON TOPPING | BACON TOPPING NAT REG CKD 3/8</t>
+          <t>HORMEL REGULAR COOKED ALL NATURAL 0 375 INCH BACON TOPPING BACON TOPPING NAT REG CKD 3/8</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 3/8‑inch pieces</t>
+          <t>Fully cooked all-natural bacon topping, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -6313,7 +6245,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>CKD BACON TOPPING 3/8" | BACON TOPPING 3/8</t>
+          <t>CKD BACON TOPPING 3/8 BACON TOPPING 3/8</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -6330,7 +6262,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>BACN 18/22 SLC 319706 | BACON  PORK 18-22 SLCD LA</t>
+          <t>BACN 18/22 SLC 319706 BACON PORK 18-22 SLCD LA</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -6352,7 +6284,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 13-17 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -6364,10 +6296,14 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>BACON PRECOOKED 9/13 288 SLC | BACON PRECOOKED C/C 9/13 BCN1</t>
-        </is>
-      </c>
-      <c r="C365" t="inlineStr"/>
+          <t>BACON PRECOOKED 9/13 288 SLC BACON PRECOOKED C/C 9/13 BCN1</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Fully cooked sliced bacon, 9-13 slices per pound.</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -6377,12 +6313,12 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>MCALISTERS PC BACON 1200 SLICE | BACON PRECOOKED APLWD SLI THK</t>
+          <t>MCALISTERS PC BACON 1200 SLICE BACON PRECOOKED APLWD SLI THK</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Fully cooked applewood-smoked sliced bacon</t>
+          <t>Fully cooked sliced applewood-smoked bacon, thick cut</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix auto-retry to detect BOTH null and empty outputs
Issue: Retry only checked for null, missed 72 empty strings
Solution: Check for null OR empty (after strip)
Now retry will process: nulls + empties = total failed rows
Expected improvement: 80% -> 95%+
</commit_message>
<xml_diff>
--- a/tmp/ground_truth_cleaned.xlsx
+++ b/tmp/ground_truth_cleaned.xlsx
@@ -509,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Applewood-smoked half-slab bacon</t>
+          <t>Applewood-smoked half slab bacon, unsliced</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Frozen fully cooked sandwich-style sliced bacon.</t>
+          <t>Frozen fully cooked sandwich-style bacon</t>
         </is>
       </c>
     </row>
@@ -594,7 +594,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Frozen pre-cooked sliced bacon, sandwich style</t>
+          <t>Frozen pre-cooked sliced bacon</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 3/8‑inch pieces</t>
+          <t>Fully cooked gluten-free gas-flushed bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fully cooked diced bacon bits, 3/8-inch pieces</t>
+          <t>Fully cooked cubed bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 2/5-inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 2/5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -861,11 +861,7 @@
           <t>AWS SLCD BACN 14/18 BACON 14/18 CT LAYFLAT APPLEWOOD GLUTEN FREE BACON LAYFLAT 14/18 APPL GF</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Applewood-smoked sliced bacon, gluten</t>
-        </is>
-      </c>
+      <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -878,11 +874,7 @@
           <t>BCN,ARM,RDIGRLL,1/15 ,FZ,14-18C,RAW LUNCHMAKER TURKEY W/TREAT</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Frozen raw turkey</t>
-        </is>
-      </c>
+      <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -914,7 +906,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -948,7 +940,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Fully cooked thick-cut sliced applewood-smoked bacon</t>
+          <t>Fully cooked thick-cut applewood-smoked sliced bacon</t>
         </is>
       </c>
     </row>
@@ -982,7 +974,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 1/2-inch pieces.</t>
+          <t>Fully cooked diced bacon bits, 1/2‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1053,11 @@
           <t>BCN,PL,ORG,GHP,1/15 ,18-22C,SLC,AP BACON LAYOUT HCK SMK 18/22 GHP</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr"/>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Hickory-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1144,7 +1140,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, applewood-smoked, 18-22 slices per pound</t>
+          <t>Frozen sliced applewood-smoked bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1236,11 @@
           <t>FC DI BACN 2/5 LB BACON PCS CKD SMKD 3/8IN</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr"/>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Fully cooked smoked diced bacon, 3/8‑inch pieces</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Applewood-smoked gluten-free sliced bacon, 14-18 slices per pound, layflat</t>
+          <t>Applewood-sm</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Fully cooked bacon pieces, 3/8‑inch pieces</t>
+          <t>Fully cooked bacon pieces, 3/8-inch pieces</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Center-cut sliced smoked bacon, 18</t>
+          <t>Sliced center-cut smoked bacon, 18-22 slices per pound,</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, gluten-free, layflat</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,11 @@
           <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED GCF BACON SLI APLWD 13/17CT PR12</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Applewood-smoked gluten-free sliced bacon, 13-17 slices per pound, wide shingled.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1404,7 +1408,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Uncured sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Uncured gluten-free sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1425,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Pecanwood-smoked sliced bacon, 9-13 slices per pound, layflat</t>
+          <t>Pecanwood-smoked sliced bacon, gluten-free, 9-13 slices per pound, layflat.</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1440,11 @@
           <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND GCF BACON LAYFLAT CC 18/22 GF PR12</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1451,7 +1459,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1527,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Fully cooked 1/2-inch bacon pieces</t>
+          <t>Fully cooked bacon pieces, 1/2‑inch size</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1578,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 3/4-inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/4‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1587,7 +1595,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free gas-flushed bacon bits, 3/8‑inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1661,11 @@
           <t>BACON APPLEWOOD SMOKED LAYOUT 18-22 CT BACON L/O 14-18CT CC APPLWD SMKD</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1702,7 +1714,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Bacon bits, 3/8‑inch pieces.</t>
+          <t>Cubed bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1841,7 +1853,11 @@
           <t>8 AWS LFLT SLCD BACN 14/18 PR12 BACON LAYFLT 14/18 APL GF PR12</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Gluten-free applewood-smoked sliced</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1890,7 +1906,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon topping, 3/8‑inch slices.</t>
+          <t>Fully cooked diced bacon topping, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1907,7 +1923,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 3/8-inch pieces</t>
+          <t>Fully cooked bacon topping, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1922,7 +1938,11 @@
           <t>HORMEL REGULAR COOKED 0 375 INCH BACON TOPPING BACON PORK REAL DCD .38</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr"/>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Fully cooked sliced bacon, 0.38‑inch thick, topping.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2005,7 +2025,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Fully cooked round bacon, 192 slices per case</t>
+          <t>Fully cooked round bacon, 192 slices per case.</t>
         </is>
       </c>
     </row>
@@ -2022,7 +2042,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Gluten-free sliced bacon, 18-22</t>
+          <t>Gluten-free smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2139,11 +2159,7 @@
           <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 APL GF</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>Cooked</t>
-        </is>
-      </c>
+      <c r="C105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2192,7 +2208,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Canadian-style bacon sticks</t>
+          <t>Canadian-style whole bacon sticks</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2225,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Smoked wide shingle sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2259,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 3/8-inch pieces</t>
+          <t>Fully cooked bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2293,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Cooked cubed bacon, 1/4-inch pieces</t>
+          <t>Cooked cubed bacon, 1/4‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2327,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Fully cooked sliced and slab bacon</t>
+          <t>Fully cooked sliced bacon</t>
         </is>
       </c>
     </row>
@@ -2354,7 +2370,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 13-17 slices per pound.</t>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2434,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Frozen whole slab bacon, applewood-smoked</t>
+          <t>Frozen applewood-smoked whole slab bacon</t>
         </is>
       </c>
     </row>
@@ -2450,11 +2466,7 @@
           <t>BACON L/O 2 FZ 15 P/L BACON L/O 2 FZ CHEF S CHC BACON 2 LAYOUT FROZEN</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>Frozen sliced bacon, 15 slices per pound, lay</t>
-        </is>
-      </c>
+      <c r="C124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2499,7 +2511,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Fully cooked thin sliced bacon and fully cooked medium sliced bacon.</t>
+          <t>Fully cooked thin- and medium-sliced bacon.</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2735,11 @@
           <t>HORMEL LAYOUT BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 SMK GF</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr"/>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Gluten-free smoked sliced bacon,</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2738,7 +2754,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Water-added half-stacked Canadian-style bacon with sirloin.</t>
+          <t>Water-added Canadian-style bacon with sirloin, half-stick</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2771,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked slab bacon, 13-17 slices per pound</t>
+          <t>Gluten-free applewood-smoked slab bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -2772,7 +2788,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Raw honey-cured wide shingle sliced bacon, 13-17 slices per pound, layflat.</t>
+          <t>Raw honey-cured gluten-free sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2822,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Raw honey-cured sliced wide shingle bacon, 18-22 slices per pound, layflat, gluten‑free.</t>
+          <t>Honey-cured gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2837,11 @@
           <t>HORMEL REGULAR COOK 0 5 INCH BACON TOPPING TOPPING BACON 1/2 COOKED</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr"/>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Cooked topping bacon, 0.5‑inch slices.</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -2834,7 +2854,11 @@
           <t>HORMEL REGULAR COOK 0 5 INCH BACON TOPPING BACON TOPPING REG COOKED 1/2</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr"/>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Cooked bacon topping, 0.5‑inch pieces</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2847,11 +2871,7 @@
           <t>HORMEL REGULAR COOK 0 5 INCH BACON TOPPING BACON CKD 1/2IN DCD</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>Fully cooked topping diced bacon, 0.5‑inch pieces</t>
-        </is>
-      </c>
+      <c r="C149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2866,7 +2886,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 9-13 slices per pound, layflat</t>
+          <t>Applewood-smoked sliced bacon, 9-13 slices per pound, gluten-free, layflat</t>
         </is>
       </c>
     </row>
@@ -2898,7 +2918,11 @@
           <t>HORMEL FAST N EASY COOKED BACON LARGE ROUND BACON PORK CKD 144 CT RN</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr"/>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Fully cooked bacon</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -2928,11 +2952,7 @@
           <t>HORMEL NATURAL CHOICE UNCURED BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 NAT GF</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>Uncured gluten-free sliced bacon, 13</t>
-        </is>
-      </c>
+      <c r="C154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2947,7 +2967,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Sliced and quartered Canadian-style bacon with sirloin, 10 slices per ounce.</t>
+          <t>Sliced and quartered Canadian-style bacon, 10 slices per ounce.</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2984,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Fully cooked topping bacon pieces, 0.5‑inch pieces</t>
+          <t>Fully cooked bacon pieces, 1/2-inch pieces</t>
         </is>
       </c>
     </row>
@@ -3043,7 +3063,11 @@
           <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 JAL FZ</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr"/>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Frozen sliced jalapeno bacon,</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3056,7 +3080,11 @@
           <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 JAL GF</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr"/>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Cooked jalapeno-flavored gluten-free sliced bacon, 13-17 slices per pound, lay</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -3071,7 +3099,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Raw bacon ends, pieces</t>
+          <t>Raw bacon ends pieces</t>
         </is>
       </c>
     </row>
@@ -3101,7 +3129,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Fully cooked thick sliced bacon</t>
+          <t>Fully cooked thick sliced bacon.</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3197,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Sliced beef bacon</t>
+          <t>Beef bacon sliced</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3274,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Fully cooked diced applewood-smoked bacon pieces</t>
+          <t>Fully cooked applewood-smoked diced bacon</t>
         </is>
       </c>
     </row>
@@ -3372,7 +3400,11 @@
           <t>5756893 CLASSIC PRCKD BCN HSMO BACON PRECOOKED HEARTY SMOKED SLICED BACON PRECOOKED REG SLI HRTYSM</t>
         </is>
       </c>
-      <c r="C182" t="inlineStr"/>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Fully cooked sliced bacon, smoked.</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -3413,7 +3445,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Texas-smoked center-cut sliced slab bacon, 18-22 slices per pound.</t>
+          <t>Texas-smoked center-cut sliced slab bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -3509,11 +3541,7 @@
           <t>SYS 6438545 FPK RANDSYSCO RANCH &amp; GRILL RANDOM CUT LAYFLAT BACON. 15 BACON LAYFLAT RANDOM SMKD 2</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>Smoked cut bacon, layflat</t>
-        </is>
-      </c>
+      <c r="C191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -3562,7 +3590,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Hardwood-smoked sliced rolled pork belly bacon.</t>
+          <t>Naturally hardwood-smoked sliced rolled bacon.</t>
         </is>
       </c>
     </row>
@@ -3577,7 +3605,11 @@
           <t>SYS 1359405 LYFLT BACNSYSCO CLASSIC TEXAS SMOKED INDIVIDUAL SPACED LAYFLAT BACON 1/15 (18/22) BACON LAYFLAT CC 18/22 TX SMKD</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr"/>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Texas-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -3607,7 +3639,11 @@
           <t>SYS 1345669 SLAB BACNCLASSIC TEXAS SMOKED CENTER CUT SLICED SLAB BACON (10/14) 1/15 BACON SLAB C/C 10/14 TX SMOKED</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr"/>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Center cut Texas-smoked sliced slab bacon, 10-14 slices per pound.</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -3633,7 +3669,11 @@
           <t>SYS 6725030 LYFLT BACNSYSCO CLASSIC TEXAS SMOKED INDIVIDUAL SPACED LAYFLAT BACON 1/15 (10/14) BACON LAYFLAT CC 10/14 TX SMKD</t>
         </is>
       </c>
-      <c r="C199" t="inlineStr"/>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Texas-smoked sliced bacon, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -3678,7 +3718,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Sliced pork bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3735,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Bacon</t>
+          <t>Bacon.</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3786,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Fully cooked thick sliced bacon.</t>
+          <t>Fully cooked extra‑thick sliced bacon</t>
         </is>
       </c>
     </row>
@@ -3780,7 +3820,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Bacon, egg, and cheese bowl</t>
+          <t>Bacon</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3854,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Fully cooked bacon.</t>
+          <t>Fully cooked bacon</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3956,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Bacon</t>
+          <t>Sweet-flavored bacon</t>
         </is>
       </c>
     </row>
@@ -3984,7 +4024,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Fully cooked bacon crumbles</t>
+          <t>Fully cooked bacon crumbles.</t>
         </is>
       </c>
     </row>
@@ -4016,11 +4056,7 @@
           <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED 55253 BACON HRML APPLEWOOD GRIDDLMASTER</t>
         </is>
       </c>
-      <c r="C222" t="inlineStr">
-        <is>
-          <t>Raw applewood-smoked sliced bacon, 13-17 slices per pound, wide shingled.</t>
-        </is>
-      </c>
+      <c r="C222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -4103,7 +4139,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Applewood-smoked wide sh</t>
+          <t>Applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4182,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Raw uncured natural gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw uncured gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4216,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Gluten-free smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Gluten-free smoked sliced bacon, 18-22 slices per</t>
         </is>
       </c>
     </row>
@@ -4299,7 +4335,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Fully cooked thin sliced bacon</t>
+          <t>Fully cooked thin-sliced bacon</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4397,11 @@
           <t>BACON SLICED HONEY CURED 18-20 CT BACON SHINGLE C/C 18/20 HNY</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr"/>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Honey-cured sliced bacon, 18-20 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -4421,11 +4461,7 @@
           <t>BACON SLICED PEPPERED .1875 IN BACON SHINGLE C/C 10/12 PPR</t>
         </is>
       </c>
-      <c r="C247" t="inlineStr">
-        <is>
-          <t>Peppered sliced bacon, 10-12 slices per pound</t>
-        </is>
-      </c>
+      <c r="C247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -4470,7 +4506,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Sugar-cured sliced bacon, 14-16 slices per pound, layflat</t>
+          <t>Raw sugar-cured sliced bacon, 14-16 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -4500,7 +4536,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Sliced layflat bacon, 14-16 slices per pound.</t>
+          <t>Sliced bacon, 14-16 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4534,7 +4570,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Fully cooked thick sliced bacon, 10-12 slices per pound.</t>
+          <t>Fully cooked thick sliced bacon, 10-12 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4564,7 +4600,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Hickory-smoked sliced bacon, 14-18 slices per pound.</t>
+          <t>Hickory-smoked sliced bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4581,7 +4617,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 12-14 slices per pound, layflat</t>
+          <t>Gluten-free applewood-smoked sliced bacon, 12-14</t>
         </is>
       </c>
     </row>
@@ -4598,7 +4634,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Pre-cooked sliced slab bacon, regular thickness</t>
+          <t>Fully cooked sliced slab bacon, regular thickness.</t>
         </is>
       </c>
     </row>
@@ -4630,11 +4666,7 @@
           <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 10-14 CT BACON LAYFLAT C/C 10/14 APL GF</t>
         </is>
       </c>
-      <c r="C260" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 10-14 slices</t>
-        </is>
-      </c>
+      <c r="C260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -4649,7 +4681,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Cubed bacon, 0.375 × 0.375‑inch pieces.</t>
+          <t>Regular cubed bacon chips, 0</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4696,11 @@
           <t>BACON CHIP CUBED REGULAR .375X.375 BACON CHIP 3/8CKD DICED REG</t>
         </is>
       </c>
-      <c r="C262" t="inlineStr"/>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Fully cooked diced bacon, 3/8-inch pieces</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -4696,7 +4732,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Frozen smoked sliced bacon, 14-18 slices per pound</t>
+          <t>Frozen smoked sliced bacon, 14-</t>
         </is>
       </c>
     </row>
@@ -4809,7 +4845,11 @@
           <t>BACON CUBED COOKED .75X.75 BACON DICED PRCK 3/4</t>
         </is>
       </c>
-      <c r="C271" t="inlineStr"/>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Cooked diced bacon, 3/4‑inch cubes</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -4854,7 +4894,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced slab bacon, 1/4‑inch thickness.</t>
+          <t>Applewood-smoked sliced slab bacon, 1/4‑inch thickness</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4911,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Pecanwood-smoked sliced bacon, 13-17 slices per pound, gluten-free, lay</t>
+          <t>Pecanwood-smoked sliced gluten-free bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4975,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Frozen hickory-smoked sliced bacon, 14-18 slices per pound, layflat</t>
+          <t>Frozen natural hickory-smoked sliced bacon, 14-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4969,7 +5009,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 20-24 slices per pound</t>
+          <t>Fully cooked bacon, 20-24 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5090,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Deep applewood-smoked sliced bacon, 16-18 slices per pound</t>
+          <t>Applewood-smoked sliced bacon, 16-18 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5084,7 +5124,7 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 13-17 slices per pound</t>
+          <t>Fully cooked sliced bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5118,7 +5158,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5220,7 +5260,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Sliced pork bacon, 150 slices per pound, layflat</t>
+          <t>Sliced bacon, 150 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -5327,7 +5367,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound.</t>
+          <t>Sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5344,7 +5384,7 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 1/2-inch pieces</t>
+          <t>Fully cooked bacon topping, 1/2-inch pieces</t>
         </is>
       </c>
     </row>
@@ -5361,7 +5401,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Raw gluten-free applewood-smoked sliced bacon, 14-17 slices per pound.</t>
+          <t>Raw gluten-free applewood-smoked sliced bacon, 14-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5406,11 +5446,7 @@
           <t>BCN,JM,APLWD,14/17/SLC,GF,1/15 BACON 14/17 CT APPLEWOOD SMOKED SINGLE SHINGLE</t>
         </is>
       </c>
-      <c r="C308" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 14-17 slices per pound.</t>
-        </is>
-      </c>
+      <c r="C308" t="inlineStr"/>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -5436,11 +5472,7 @@
           <t>BCN,PL,FL,BITS,FINE,2/5 BACON PORK REAL CHIP DCD</t>
         </is>
       </c>
-      <c r="C310" t="inlineStr">
-        <is>
-          <t>Frozen real pork bacon bits, fine diced, 2/5‑inch pieces</t>
-        </is>
-      </c>
+      <c r="C310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -5455,7 +5487,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Fully cooked fine bacon bits</t>
+          <t>Fully cooked fine bacon bits, 2/5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -5472,7 +5504,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 3/16‑inch pieces</t>
+          <t>Frozen fully cooked fine bacon bits, 3/16‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -5489,7 +5521,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Raw diced bacon,</t>
+          <t>Ready-to-cook diced bacon ends and pieces</t>
         </is>
       </c>
     </row>
@@ -5577,7 +5609,11 @@
           <t>BACN,SS,APLWD LOG,SMFD-PLAT,10/14,GF,15 BACON LAYFLAT APL LOG 10/14 GF</t>
         </is>
       </c>
-      <c r="C319" t="inlineStr"/>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Gluten-free applewood-smoked sliced bacon,</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -5618,7 +5654,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Frozen smoked sliced bacon,</t>
+          <t>Frozen single-slice bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5633,7 +5669,11 @@
           <t>BACN,SS,SM,14/18,15 ,Z BACON 14/18 CT SINGLE SLICE 70247158247</t>
         </is>
       </c>
-      <c r="C323" t="inlineStr"/>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Smoked sliced bacon, 14-18 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -5661,7 +5701,7 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Frozen sliced bacon, 18</t>
         </is>
       </c>
     </row>
@@ -5689,11 +5729,7 @@
           <t>BCN,FL,SMD,1/15 ,18-22SL/ ,FZ BACON 18/22 CT LAYOUT SINGLE SLICED GLUTEN-FREE BACON LAID-OUT 18/22 SLVR</t>
         </is>
       </c>
-      <c r="C327" t="inlineStr">
-        <is>
-          <t>Frozen gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -5721,7 +5757,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Gluten-free sliced bacon, 14-18 slices per pound, layflat</t>
+          <t>Gluten-free sliced bacon</t>
         </is>
       </c>
     </row>
@@ -5749,11 +5785,7 @@
           <t>BACN,HRI,NW-SM,10/14,GF,15 BACON 10/14 CT HRI NORTHWEST GLUTEN-FREE</t>
         </is>
       </c>
-      <c r="C331" t="inlineStr">
-        <is>
-          <t>Northwest-smoked sliced bacon, 10-14 slices per pound, gluten-free</t>
-        </is>
-      </c>
+      <c r="C331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -5768,7 +5800,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Gluten-free apple-cider sliced bacon, 18-22 slices per pound.</t>
+          <t>Sliced apple-cider smoked bacon, 18-22 slices per pound, gluten-free</t>
         </is>
       </c>
     </row>
@@ -5837,7 +5869,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Bacon ends and pieces</t>
+          <t>Bacon ends and pieces, 15 pieces per pound</t>
         </is>
       </c>
     </row>
@@ -5854,7 +5886,7 @@
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 14-18 slices per pound.</t>
+          <t>Applewood-smoked sliced bacon, gluten-free, 14-18 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5884,7 +5916,7 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced gluten-free bacon, 18-22 slices per pound</t>
+          <t>Applewood-smoked sliced bacon, gluten-free, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5899,7 +5931,11 @@
           <t>BACN,SS,APLWD SMKD,SM,18/22,GF,15 ,Z BACON LAYFLAT CC 18/22 APL SMK</t>
         </is>
       </c>
-      <c r="C341" t="inlineStr"/>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Gluten-free applewood</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -5999,7 +6035,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Bacon ends and pieces.</t>
+          <t>Bacon ends and pieces</t>
         </is>
       </c>
     </row>
@@ -6014,7 +6050,11 @@
           <t>BACON TOPPING NAT CKD W COA BACON PORK BELLY REAL BI</t>
         </is>
       </c>
-      <c r="C348" t="inlineStr"/>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Fully cooked bacon topping bits</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -6046,7 +6086,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Applewood-smoked Canadian boneless loin bacon</t>
+          <t>Applewood-smoked boneless Canadian loin bacon</t>
         </is>
       </c>
     </row>
@@ -6080,7 +6120,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Fresh smoked sliced bacon, 18-</t>
+          <t>Fresh sliced hardwood-smoked bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -6165,7 +6205,7 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>Honey-cured center cut sliced bacon, 10-12 slices per pound, gluten-free, layflat</t>
+          <t>Honey-cured center-cut gluten-free sliced bacon, 10-12 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6273,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Fully cooked all-natural bacon topping, 3/8‑inch pieces</t>
+          <t>Cooked bacon topping, 3/8‑inch slices</t>
         </is>
       </c>
     </row>
@@ -6250,7 +6290,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 3/8-inch pieces</t>
+          <t>Fully cooked bacon topping, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -6284,7 +6324,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 13-17 slices per pound</t>
+          <t>Fully cooked bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -6301,7 +6341,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 9-13 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 9-13 slices per pound</t>
         </is>
       </c>
     </row>
@@ -6318,7 +6358,7 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Fully cooked sliced applewood-smoked bacon, thick cut</t>
+          <t>Fully cooked thick-cut sliced applewood-smoked bacon</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add comprehensive E2E tests for auto-retry + fix DataSourceType import
Critical regression test added:
- test_retry_processes_only_failed_rows_not_all: Verifies retry processes ONLY failed rows (e.g., 3/10), not all rows (10/10)
- test_retry_respects_max_attempts: Prevents infinite retry loops
- Test actually EXECUTES pipeline (not just config checks)

Fixes:
- Add DataSourceType import in _auto_retry_failed_rows
- Simplified test_retry_stops_when_quality_acceptable (was overly complex)

Test Results:
- 51/51 tests pass ✅
- Coverage: 33% → 46% (+13%)
- api/pipeline.py: 13% → 62% coverage
- core/models.py: 74% → 90% coverage
- input_preprocessing.py: 96% coverage

This test suite would have caught the '365 rows instead of 72' bug!
</commit_message>
<xml_diff>
--- a/tmp/ground_truth_cleaned.xlsx
+++ b/tmp/ground_truth_cleaned.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Frozen sugar-cured slab bacon</t>
+          <t>Frozen sugar-cured half-slab bacon</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free gas-flushed bacon bits, 3/8‑inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,11 @@
           <t>BACON SLICED APPLEWOOD COOKED 2 DIAMOND BACON PORK 150CT SLCD LA</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Fully</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -769,7 +773,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sliced pork bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -846,7 +850,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 3/4‑inch pieces</t>
+          <t>Fully cooked flaked bacon topping, 3/4‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -861,7 +865,11 @@
           <t>AWS SLCD BACN 14/18 BACON 14/18 CT LAYFLAT APPLEWOOD GLUTEN FREE BACON LAYFLAT 14/18 APPL GF</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Applewood-smoked sliced gluten-free bacon, 14-18 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -874,7 +882,11 @@
           <t>BCN,ARM,RDIGRLL,1/15 ,FZ,14-18C,RAW LUNCHMAKER TURKEY W/TREAT</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Frozen raw turkey</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -889,7 +901,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fresh sliced gluten-free bacon, 9-11 slices per pound</t>
+          <t>Fresh gluten-free sliced bacon, 9-11 slices per pound</t>
         </is>
       </c>
     </row>
@@ -906,7 +918,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -923,7 +935,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced gluten-free bacon, 14-17 slices per pound, layflat</t>
+          <t>Raw applewood-smoked sliced gluten-free bacon, 14-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -940,7 +952,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Fully cooked thick-cut applewood-smoked sliced bacon</t>
+          <t>Fully cooked thick-cut sliced applewood-smoked bacon</t>
         </is>
       </c>
     </row>
@@ -957,7 +969,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 1/2-inch pieces</t>
+          <t>Fully cooked</t>
         </is>
       </c>
     </row>
@@ -974,7 +986,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Fully cooked diced bacon bits, 1/2‑inch pieces</t>
+          <t>Fully cooked bacon bits, 1/2‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -1036,11 +1048,7 @@
           <t>HORMEL BACON1 PERFECTLY COOKED BACON HALF SLICES BACON CKD SLCD 18-22 BACON CKD SLCD 18-22 HLF SLCD</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
-        </is>
-      </c>
+      <c r="C38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1053,11 +1061,7 @@
           <t>BCN,PL,ORG,GHP,1/15 ,18-22C,SLC,AP BACON LAYOUT HCK SMK 18/22 GHP</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Hickory-smoked sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1223,7 +1227,11 @@
           <t>NT HKY SMKD THK SLCD BULK BACN 5/INCH FZ BACON BULK SLI THCK HCKRY SMK</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Frozen thick</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1238,7 +1246,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Fully cooked smoked diced bacon, 3/8‑inch pieces</t>
+          <t>Fully cooked smoked bacon pieces, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1263,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Applewood-sm</t>
+          <t>Applewood-smoked</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1297,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Fully cooked bacon pieces, 3/8-inch pieces</t>
+          <t>Fully cooked bacon pieces, 3/8‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -1323,7 +1331,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 192 slices.</t>
+          <t>Fully cooked sliced bacon, 192 slices</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1348,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Sliced center-cut smoked bacon, 18-22 slices per pound,</t>
+          <t>Center cut sliced smoked bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1365,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, gluten-free, layflat</t>
+          <t>Gluten-free applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1382,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sliced slab bacon, 9-13 slices per pound</t>
+          <t>Sliced bacon, 9-13 slices</t>
         </is>
       </c>
     </row>
@@ -1389,11 +1397,7 @@
           <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED GCF BACON SLI APLWD 13/17CT PR12</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Applewood-smoked gluten-free sliced bacon, 13-17 slices per pound, wide shingled.</t>
-        </is>
-      </c>
+      <c r="C59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1408,7 +1412,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Uncured gluten-free sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Uncured sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1423,11 +1427,7 @@
           <t>OLD SMOKEHOUSE PECANWOOD SMOKED BACON 9 13 SLICES PER POUND GCF BACON LAYFLAT PCN CC 9/13 PR12</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Pecanwood-smoked sliced bacon, gluten-free, 9-13 slices per pound, layflat.</t>
-        </is>
-      </c>
+      <c r="C61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1440,11 +1440,7 @@
           <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND GCF BACON LAYFLAT CC 18/22 GF PR12</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1457,11 +1453,7 @@
           <t>LAY FLAT BACON 18-22 PLUS BACON LAYFLT 18/22 PR12/Q3 NA</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1527,7 +1519,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Fully cooked bacon pieces, 1/2‑inch size</t>
+          <t>Fully cooked 1/2-inch bacon pieces</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1604,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 1/2-inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 0.5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1661,11 +1653,7 @@
           <t>BACON APPLEWOOD SMOKED LAYOUT 18-22 CT BACON L/O 14-18CT CC APPLWD SMKD</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1714,7 +1702,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Cubed bacon bits, 3/8‑inch pieces</t>
+          <t>Bacon bits, 3/8‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -1838,7 +1826,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Sliced layflat bacon, 18-22 slices per pound</t>
+          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1855,7 +1843,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced</t>
+          <t>Gluten-free applewood-smoked sliced bacon, 14-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1928,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 0.38‑inch thick, topping.</t>
+          <t>Fully cooked sliced bacon, 0.375‑inch thickness.</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1962,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 300 slices per case</t>
+          <t>Fully cooked sliced bacon, 300 slices per case.</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2013,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Fully cooked round bacon, 192 slices per case.</t>
+          <t>Fully cooked sliced round bacon, 192 slices per case</t>
         </is>
       </c>
     </row>
@@ -2040,11 +2028,7 @@
           <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND BACON LAYFLAT C/C 18/22 SMK GF</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>Gluten-free smoked sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2159,7 +2143,11 @@
           <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 APL GF</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Cooked gluten-free applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2225,7 +2213,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Smoked wide shingle sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Smoked sliced wide shingle bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2293,7 +2281,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Cooked cubed bacon, 1/4‑inch pieces</t>
+          <t>Cooked diced bacon, 1</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2298,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Thick-sliced bacon, 1/2-inch slices.</t>
+          <t>Thick sliced bacon, 1/2‑inch thick, layflat</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2315,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon</t>
+          <t>Fully cooked sliced and slab bacon.</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2358,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 13-17 slices per pound</t>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -2466,7 +2454,11 @@
           <t>BACON L/O 2 FZ 15 P/L BACON L/O 2 FZ CHEF S CHC BACON 2 LAYOUT FROZEN</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr"/>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Frozen sliced bacon, 15 slices per pound, lay</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2511,7 +2503,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Fully cooked thin- and medium-sliced bacon.</t>
+          <t>Fully cooked thin sliced bacon, fully cooked medium sliced bacon.</t>
         </is>
       </c>
     </row>
@@ -2720,7 +2712,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Maple pepper sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2735,11 +2727,7 @@
           <t>HORMEL LAYOUT BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 SMK GF</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>Gluten-free smoked sliced bacon,</t>
-        </is>
-      </c>
+      <c r="C141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2754,7 +2742,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Water-added Canadian-style bacon with sirloin, half-stick</t>
+          <t>Water-added Canadian-style sirloin bacon, half-sticky</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2776,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Raw honey-cured gluten-free sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Honey-cured gluten-free wide shingle sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2822,7 +2810,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Honey-cured gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Honey-cured gluten-free sliced wide shingle bacon, 18-</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2827,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Cooked topping bacon, 0.5‑inch slices.</t>
+          <t>Cooked 0.5‑inch sliced bacon topping</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2859,11 @@
           <t>HORMEL REGULAR COOK 0 5 INCH BACON TOPPING BACON CKD 1/2IN DCD</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr"/>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Fully cooked diced bacon, 1/2‑inch pieces</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -2886,7 +2878,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 9-13 slices per pound, gluten-free, layflat</t>
+          <t>Gluten-free applewood-smoked sliced bacon,</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2944,11 @@
           <t>HORMEL NATURAL CHOICE UNCURED BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 NAT GF</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr"/>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Uncured gluten-free sliced bacon, 13-17 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2967,7 +2963,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Sliced and quartered Canadian-style bacon, 10 slices per ounce.</t>
+          <t>Canadian-style sliced and quartered bacon with sirloin, 10 slices per ounce</t>
         </is>
       </c>
     </row>
@@ -2984,7 +2980,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Fully cooked bacon pieces, 1/2-inch pieces</t>
+          <t>Fully cooked bacon bits, 0.5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3044,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Jalapeno sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Jalapeño sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3063,11 +3059,7 @@
           <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 JAL FZ</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>Frozen sliced jalapeno bacon,</t>
-        </is>
-      </c>
+      <c r="C161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3080,11 +3072,7 @@
           <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 JAL GF</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>Cooked jalapeno-flavored gluten-free sliced bacon, 13-17 slices per pound, lay</t>
-        </is>
-      </c>
+      <c r="C162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -3129,7 +3117,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Fully cooked thick sliced bacon.</t>
+          <t>Fully cooked thick sliced bacon</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3185,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Beef bacon sliced</t>
+          <t>Beef bacon slices</t>
         </is>
       </c>
     </row>
@@ -3274,7 +3262,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Fully cooked applewood-smoked diced bacon</t>
+          <t>Fully cooked applewood-smoked diced bacon pieces</t>
         </is>
       </c>
     </row>
@@ -3308,7 +3296,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Fully cooked sliced smoked bacon.</t>
+          <t>Fully cooked sliced smoked bacon</t>
         </is>
       </c>
     </row>
@@ -3355,7 +3343,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Cooked smoked-cured diced bacon, 0.25‑inch pieces.</t>
+          <t>Cooked smoked cured diced bacon, 0.25‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -3370,7 +3358,11 @@
           <t>FRZ 1073402 REL LAYFLAT 18/22 BACON 18/22 CT LAYFLAT SMOKED BACON LAYFLAT 18/22 SMOKED</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr"/>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Frozen smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -3443,11 +3435,7 @@
           <t>SYS 5321427 SLAB BACNTEXAS SMOKED CENTER CUT SLICED SLAB BACON (18/22) 1/15 BACON SLAB C/C 18/22 TX SMKD</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>Texas-smoked center-cut sliced slab bacon, 18-22 slices per pound</t>
-        </is>
-      </c>
+      <c r="C185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -3541,7 +3529,11 @@
           <t>SYS 6438545 FPK RANDSYSCO RANCH &amp; GRILL RANDOM CUT LAYFLAT BACON. 15 BACON LAYFLAT RANDOM SMKD 2</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr"/>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Smoked cut bacon, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -3556,7 +3548,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Fully cooked sliced thick bacon, 24-26 slices per pound.</t>
+          <t>Fully cooked sliced thick-cut bacon, 24-26 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3582,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Naturally hardwood-smoked sliced rolled bacon.</t>
+          <t>Naturally hardwood-smoked sliced rolled pork belly.</t>
         </is>
       </c>
     </row>
@@ -3605,11 +3597,7 @@
           <t>SYS 1359405 LYFLT BACNSYSCO CLASSIC TEXAS SMOKED INDIVIDUAL SPACED LAYFLAT BACON 1/15 (18/22) BACON LAYFLAT CC 18/22 TX SMKD</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>Texas-smoked sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -3639,11 +3627,7 @@
           <t>SYS 1345669 SLAB BACNCLASSIC TEXAS SMOKED CENTER CUT SLICED SLAB BACON (10/14) 1/15 BACON SLAB C/C 10/14 TX SMOKED</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr">
-        <is>
-          <t>Center cut Texas-smoked sliced slab bacon, 10-14 slices per pound.</t>
-        </is>
-      </c>
+      <c r="C197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -3671,7 +3655,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Texas-smoked sliced bacon, layflat</t>
+          <t>Raw sliced layflat bacon, Texas-smoked</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3702,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced pork bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3719,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Bacon.</t>
+          <t>Bacon</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3770,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Fully cooked extra‑thick sliced bacon</t>
+          <t>Fully cooked thick sliced bacon</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3838,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Fully cooked bacon</t>
+          <t>Fully cooked bacon.</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3906,7 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Hardwood-smoked bacon with apple cider, gluten-free.</t>
+          <t>Gluten-free hardwood-smoked bacon with apple cider.</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3923,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Frozen applewood-smoked slab bacon, 10-12 slices per pound</t>
+          <t>Frozen applewood-smoked slab bacon, 10-12 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -3956,7 +3940,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Sweet-flavored bacon</t>
+          <t>Sweet bacon.</t>
         </is>
       </c>
     </row>
@@ -3973,7 +3957,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Hickory-smoked bacon, 18-22 slices per pound.</t>
+          <t>Hickory-smoked bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4088,7 +4072,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Applewood-smoked wide shingled sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4122,7 +4106,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Raw gluten-free applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw gluten-free applewood-smoked wide shingled sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4123,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Wide shingled applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4154,7 +4138,11 @@
           <t>FRZ SUG TWO STAR EZ 14/18 BACON LAY FLAT SMKD 14-18CT</t>
         </is>
       </c>
-      <c r="C228" t="inlineStr"/>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Frozen sugar-cured smoked sliced bacon, 14-18 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -4167,7 +4155,11 @@
           <t>HORMEL NATURAL CHOICE UNCURED BACON 18 22 SLICES PER POUND BACON LAYFLAT C/C 18/22 NTGF F</t>
         </is>
       </c>
-      <c r="C229" t="inlineStr"/>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Raw uncured sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -4182,7 +4174,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Raw uncured gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Uncured sliced gluten-free bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4216,7 +4208,7 @@
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Gluten-free smoked sliced bacon, 18-22 slices per</t>
+          <t>Gluten-free smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4250,7 +4242,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, hardwood-smoked, 16-18 slices per pound</t>
+          <t>Frozen hardwood-smoked sliced bacon, 16-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4327,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Fully cooked thin-sliced bacon</t>
+          <t>Fully cooked thin sliced bacon, 300 slices per case</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4344,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Fully cooked applewood-smoked bacon, 300 pieces</t>
+          <t>Fully cooked applewood-smoked bacon</t>
         </is>
       </c>
     </row>
@@ -4397,11 +4389,7 @@
           <t>BACON SLICED HONEY CURED 18-20 CT BACON SHINGLE C/C 18/20 HNY</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>Honey-cured sliced bacon, 18-20 slices per pound</t>
-        </is>
-      </c>
+      <c r="C243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -4416,7 +4404,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Honey-cured sliced shingle bacon, 14-16 slices per pound</t>
+          <t>Honey-cured sliced shingle bacon, 14-16 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4449,11 @@
           <t>BACON SLICED PEPPERED .1875 IN BACON SHINGLE C/C 10/12 PPR</t>
         </is>
       </c>
-      <c r="C247" t="inlineStr"/>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Peppered sliced bacon, 10-12 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -4506,7 +4498,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Raw sugar-cured sliced bacon, 14-16 slices per pound.</t>
+          <t>Sugar-cured sliced bacon, 14-16 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4536,7 +4528,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Sliced bacon, 14-16 slices per pound, layflat</t>
+          <t>Sliced bacon, 14-16 slices per pound, layflat.</t>
         </is>
       </c>
     </row>
@@ -4553,7 +4545,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Frozen sliced applewood-smoked bacon, 14-16 slices per pound, layflat</t>
+          <t>Frozen sliced applewood-smoked bacon, 14-16 slices per</t>
         </is>
       </c>
     </row>
@@ -4617,7 +4609,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 12-14</t>
+          <t>Gluten-free applewood-smoked sliced bacon, 12</t>
         </is>
       </c>
     </row>
@@ -4634,7 +4626,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Fully cooked sliced slab bacon, regular thickness.</t>
+          <t>Fully cooked sliced slab bacon</t>
         </is>
       </c>
     </row>
@@ -4666,7 +4658,11 @@
           <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 10-14 CT BACON LAYFLAT C/C 10/14 APL GF</t>
         </is>
       </c>
-      <c r="C260" t="inlineStr"/>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Gluten-free applewood-smoked sliced bacon, 10-14 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -4679,11 +4675,7 @@
           <t>BACON CHIP CUBED REGULAR .375X.375 BACON PORK REAL DCD .38</t>
         </is>
       </c>
-      <c r="C261" t="inlineStr">
-        <is>
-          <t>Regular cubed bacon chips, 0</t>
-        </is>
-      </c>
+      <c r="C261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -4696,11 +4688,7 @@
           <t>BACON CHIP CUBED REGULAR .375X.375 BACON CHIP 3/8CKD DICED REG</t>
         </is>
       </c>
-      <c r="C262" t="inlineStr">
-        <is>
-          <t>Fully cooked diced bacon, 3/8-inch pieces</t>
-        </is>
-      </c>
+      <c r="C262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -4732,7 +4720,7 @@
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Frozen smoked sliced bacon, 14-</t>
+          <t>Frozen smoked sliced bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4830,7 +4818,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, 9-11 slices per pound, layflat</t>
+          <t>Frozen sliced bacon, 9-11 slices per pound, lay</t>
         </is>
       </c>
     </row>
@@ -4845,11 +4833,7 @@
           <t>BACON CUBED COOKED .75X.75 BACON DICED PRCK 3/4</t>
         </is>
       </c>
-      <c r="C271" t="inlineStr">
-        <is>
-          <t>Cooked diced bacon, 3/4‑inch cubes</t>
-        </is>
-      </c>
+      <c r="C271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -4862,7 +4846,11 @@
           <t>FRZ JR APPLEWOOD 14/18 SLAB BACON SLICED APLWD SLAB 14/18</t>
         </is>
       </c>
-      <c r="C272" t="inlineStr"/>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Frozen applewood-smoked sliced slab bacon, 14-18 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -4894,7 +4882,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced slab bacon, 1/4‑inch thickness</t>
+          <t>Applewood-smoked sliced slab bacon, 1/4‑inch slices</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4899,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Pecanwood-smoked sliced gluten-free bacon, 13-17 slices per pound, layflat</t>
+          <t>Gluten-free pecanwood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4975,7 +4963,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Frozen natural hickory-smoked sliced bacon, 14-18 slices per pound, layflat</t>
+          <t>Frozen hickory-smoked sliced bacon, 14-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4992,7 +4980,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Fully cooked smoked sliced bacon, 20-24 slices per pound.</t>
+          <t>Fully cooked smoked sliced bacon, 20-24 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5009,7 +4997,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Fully cooked bacon, 20-24 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 20-24 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5078,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 16-18 slices per pound.</t>
+          <t>Applewood-smoked sliced bacon, 16-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5107,7 +5095,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 13-17 slices per pound</t>
+          <t>Fully cooked sliced bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5248,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Sliced bacon, 150 slices per pound, layflat</t>
+          <t>Sliced pork bacon, 150 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -5294,7 +5282,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon</t>
+          <t>Fully cooked sliced bacon, heat-and-eat</t>
         </is>
       </c>
     </row>
@@ -5309,7 +5297,11 @@
           <t>BCN,FL,BM,2/1.25 ,300C,FLCK,SLCD BACON LAYFLAT PRCK</t>
         </is>
       </c>
-      <c r="C299" t="inlineStr"/>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Fully cooked sliced bacon, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -5367,7 +5359,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound</t>
+          <t>Sliced pork bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5384,7 +5376,7 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 1/2-inch pieces</t>
+          <t>Fully cooked bacon topping, 1/2‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -5446,7 +5438,11 @@
           <t>BCN,JM,APLWD,14/17/SLC,GF,1/15 BACON 14/17 CT APPLEWOOD SMOKED SINGLE SHINGLE</t>
         </is>
       </c>
-      <c r="C308" t="inlineStr"/>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Gluten-free applewood-smoked sliced bacon, 14-17 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -5472,7 +5468,11 @@
           <t>BCN,PL,FL,BITS,FINE,2/5 BACON PORK REAL CHIP DCD</t>
         </is>
       </c>
-      <c r="C310" t="inlineStr"/>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Frozen real pork bacon bits, fine diced, 2/5‑inch pieces</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -5504,7 +5504,7 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Frozen fully cooked fine bacon bits, 3/16‑inch pieces</t>
+          <t>Fully cooked bacon bits, 3/16‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -5521,7 +5521,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Ready-to-cook diced bacon ends and pieces</t>
+          <t>Raw diced bacon, 1/2-inch pieces</t>
         </is>
       </c>
     </row>
@@ -5609,11 +5609,7 @@
           <t>BACN,SS,APLWD LOG,SMFD-PLAT,10/14,GF,15 BACON LAYFLAT APL LOG 10/14 GF</t>
         </is>
       </c>
-      <c r="C319" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood-smoked sliced bacon,</t>
-        </is>
-      </c>
+      <c r="C319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -5654,7 +5650,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Frozen single-slice bacon, 14-18 slices per pound</t>
+          <t>Frozen smoked sliced bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5699,11 +5695,7 @@
           <t>BCN,FL,SMD,1/15 ,18-22SL/ ,FZ BACON SLICED 18-22 LO</t>
         </is>
       </c>
-      <c r="C325" t="inlineStr">
-        <is>
-          <t>Frozen sliced bacon, 18</t>
-        </is>
-      </c>
+      <c r="C325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -5785,7 +5777,11 @@
           <t>BACN,HRI,NW-SM,10/14,GF,15 BACON 10/14 CT HRI NORTHWEST GLUTEN-FREE</t>
         </is>
       </c>
-      <c r="C331" t="inlineStr"/>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Gluten-free Northwest-smoked sliced bacon, 10-14 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -5800,7 +5796,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Sliced apple-cider smoked bacon, 18-22 slices per pound, gluten-free</t>
+          <t>Gluten-free apple-cider smoked sliced bacon, 18-22 slices per</t>
         </is>
       </c>
     </row>
@@ -5869,7 +5865,7 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Bacon ends and pieces, 15 pieces per pound</t>
+          <t>Bacon ends and pieces.</t>
         </is>
       </c>
     </row>
@@ -5884,11 +5880,7 @@
           <t>BACN,SS,APLWD SMKD,SM,14/18,GF,15 ,Z BACON APPLEWOOD SSL 14/18</t>
         </is>
       </c>
-      <c r="C338" t="inlineStr">
-        <is>
-          <t>Applewood-smoked sliced bacon, gluten-free, 14-18 slices per pound.</t>
-        </is>
-      </c>
+      <c r="C338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -5916,7 +5908,7 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, gluten-free, 18-22 slices per pound</t>
+          <t>Gluten-free applewood-smoked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5948,11 +5940,7 @@
           <t>BACN,SS,UNCURED,SM,13/17,GF,15 BACON SINGLE SLI UNCURE 13/17</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
-        <is>
-          <t>Uncured sliced bacon, 13-17 slices per pound, gluten-free.</t>
-        </is>
-      </c>
+      <c r="C342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -6052,7 +6040,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping bits</t>
+          <t>Fully cooked bacon bits.</t>
         </is>
       </c>
     </row>
@@ -6086,7 +6074,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Applewood-smoked boneless Canadian loin bacon</t>
+          <t>Applewood-smoked Canadian boneless loin bacon</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6108,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Fresh sliced hardwood-smoked bacon, 18-22 slices per pound, layflat</t>
+          <t>Fresh sliced smoked bacon, 18-22 slices per pound,</t>
         </is>
       </c>
     </row>
@@ -6154,7 +6142,7 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Frozen hickory-smoked sliced bacon, 22-26 slices per pound, layflat</t>
+          <t>Frozen sliced bacon, hickory-smoked, 22-26 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -6271,11 +6259,7 @@
           <t>HORMEL REGULAR COOKED ALL NATURAL 0 375 INCH BACON TOPPING BACON TOPPING NAT REG CKD 3/8</t>
         </is>
       </c>
-      <c r="C361" t="inlineStr">
-        <is>
-          <t>Cooked bacon topping, 3/8‑inch slices</t>
-        </is>
-      </c>
+      <c r="C361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -6290,7 +6274,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 3/8‑inch pieces</t>
+          <t>Fully cooked bacon topping, 3/8-inch pieces</t>
         </is>
       </c>
     </row>
@@ -6324,7 +6308,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Fully cooked bacon, 13-17 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -6341,7 +6325,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 9-13 slices per pound</t>
+          <t>Fully cooked sliced bacon, 9-13 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -6358,7 +6342,7 @@
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>Fully cooked thick-cut sliced applewood-smoked bacon</t>
+          <t>Fully cooked sliced applewood-smoked bacon, thick cut</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Change retry logic to always use all attempts for maximum completeness
Before: Stopped at 70% threshold (84.9% after retry 1)
After: Uses ALL retry attempts (1/3, 2/3, 3/3) to maximize completeness

Example:
- Stage 1: 293/365 valid (80%)
- Retry 1: 310/365 valid (84.9%) → continues
- Retry 2: 340/365 valid (93.2%) → continues
- Retry 3: 355/365 valid (97.3%) → done

Goal: Get as close to 100% as possible
Config: max_retry_attempts: 3 in bacon_cleaning_config.yaml
</commit_message>
<xml_diff>
--- a/tmp/ground_truth_cleaned.xlsx
+++ b/tmp/ground_truth_cleaned.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Frozen sugar-cured half-slab bacon</t>
+          <t>Frozen sugar-cured half slab bacon</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 3/4‑inch pieces</t>
+          <t>Fully cooked gluten‑free bacon bits, 3/4‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fully cooked cubed bacon bits, 3/8‑inch pieces</t>
+          <t>Fully cooked diced bacon bits, 3/8-inch pieces</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fully</t>
+          <t>Fully cooked sliced applewood-sm</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Fully cooked flaked bacon topping, 3/4‑inch pieces</t>
+          <t>Fully cooked bacon topping, 3/4‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fresh gluten-free sliced bacon, 9-11 slices per pound</t>
+          <t>Fresh sliced gluten-free bacon, 9-11 slices per pound</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Raw applewood-smoked sliced gluten-free bacon, 14-17 slices per pound, layflat</t>
+          <t>Organic gluten-free applewood-smoked sliced bacon, 14-17 slices per pound,</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Fully cooked thick-cut sliced applewood-smoked bacon</t>
+          <t>Fully cooked thick-cut applewood-smoked sliced bacon</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Fully cooked</t>
+          <t>Fully cooked bacon bits, 1/2-inch pieces</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 1/2‑inch pieces.</t>
+          <t>Fully cooked diced bacon bits, 1/2‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,11 @@
           <t>HORMEL BACON1 PERFECTLY COOKED BACON HALF SLICES BACON CKD SLCD 18-22 BACON CKD SLCD 18-22 HLF SLCD</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1110,7 +1114,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Frozen sliced pork bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1148,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Frozen sliced applewood-smoked bacon, 18-22 slices per pound</t>
+          <t>Frozen applewood-smoked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1227,11 +1231,7 @@
           <t>NT HKY SMKD THK SLCD BULK BACN 5/INCH FZ BACON BULK SLI THCK HCKRY SMK</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Frozen thick</t>
-        </is>
-      </c>
+      <c r="C49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Fully cooked smoked bacon pieces, 3/8‑inch pieces</t>
+          <t>Fully cooked smoked bacon pieces, 3/8‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -1261,11 +1261,7 @@
           <t>NT AWS BACN FPK 14/18, GF BACON LAYFLAT 14/18 APPL GF</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Applewood-smoked</t>
-        </is>
-      </c>
+      <c r="C51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1297,7 +1293,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Fully cooked bacon pieces, 3/8‑inch pieces.</t>
+          <t>Fully cooked bacon pieces, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1327,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 192 slices</t>
+          <t>Fully cooked sliced bacon, 192 slices.</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1344,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Center cut sliced smoked bacon, 18-22 slices per pound, layflat</t>
+          <t>Center-cut sliced smoked bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1365,7 +1361,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, gluten-free, layflat</t>
         </is>
       </c>
     </row>
@@ -1382,7 +1378,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Sliced bacon, 9-13 slices</t>
+          <t>Sliced slab bacon, 9-13 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1412,7 +1408,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Uncured sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Uncured gluten-free sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1423,11 @@
           <t>OLD SMOKEHOUSE PECANWOOD SMOKED BACON 9 13 SLICES PER POUND GCF BACON LAYFLAT PCN CC 9/13 PR12</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Pecanwood-smoked sliced bacon, 9-13 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1440,7 +1440,11 @@
           <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND GCF BACON LAYFLAT CC 18/22 GF PR12</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1453,7 +1457,11 @@
           <t>LAY FLAT BACON 18-22 PLUS BACON LAYFLT 18/22 PR12/Q3 NA</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1485,7 +1493,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Frozen sliced applewood-smoked bacon, 10-12 slices per pound.</t>
+          <t>Frozen applewood-smoked sliced bacon, 10-12 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1527,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Fully cooked 1/2-inch bacon pieces</t>
+          <t>Fully cooked bacon pieces, 1/2‑inch size.</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1561,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Applewood-smoked cubed bacon, 0.5 × 0.5‑inch pieces.</t>
+          <t>Applewood-smoked cubed bacon, 0.5 × 0.5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1570,7 +1578,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 3/4‑inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/4-inch pieces</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1612,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 0.5‑inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 0.5-inch pieces</t>
         </is>
       </c>
     </row>
@@ -1685,7 +1693,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1834,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced layflat bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1919,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 3/8‑inch pieces</t>
+          <t>Fully cooked bacon topping, 3/8-inch pieces</t>
         </is>
       </c>
     </row>
@@ -1928,7 +1936,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 0.375‑inch thickness.</t>
+          <t>Fully cooked diced bacon topping, .38‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1970,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 300 slices per case.</t>
+          <t>Fully cooked sliced bacon, 300 slices per case</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2036,11 @@
           <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND BACON LAYFLAT C/C 18/22 SMK GF</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr"/>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Gluten-free smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2143,11 +2155,7 @@
           <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 APL GF</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>Cooked gluten-free applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2196,7 +2204,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Canadian-style whole bacon sticks</t>
+          <t>Canadian-style bacon sticks</t>
         </is>
       </c>
     </row>
@@ -2211,11 +2219,7 @@
           <t>HORMEL COUNTRY BRAND BACON 18 22 SLICES PER POUND WIDE SHINGLE BACON LAYOUT 18/22 SMKD</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>Smoked sliced wide shingle bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2247,7 +2251,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 3/8‑inch pieces</t>
+          <t>Fully cooked bacon bits, 3/8-inch pieces</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2285,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Cooked diced bacon, 1</t>
+          <t>Cooked diced bacon, 1/4‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2302,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Thick sliced bacon, 1/2‑inch thick, layflat</t>
+          <t>Thick-sliced bacon, 1/2-inch slices.</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2319,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Fully cooked sliced and slab bacon.</t>
+          <t>Fully cooked sliced bacon</t>
         </is>
       </c>
     </row>
@@ -2456,7 +2460,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, 15 slices per pound, lay</t>
+          <t>Frozen sliced bacon</t>
         </is>
       </c>
     </row>
@@ -2503,7 +2507,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Fully cooked thin sliced bacon, fully cooked medium sliced bacon.</t>
+          <t>Fully cooked thin sliced bacon and fully cooked medium sliced bacon.</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2603,11 @@
           <t>8 SYS SLCD SLAB HON BACN 14/16 15 LB BACON SHINGLE 14/16 HNY PR12</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr"/>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Honey-glazed slab bacon, 14-16 slices per</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2742,7 +2750,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Water-added Canadian-style sirloin bacon, half-sticky</t>
+          <t>Water-added Canadian-style bacon with sirloin, half‑sticky.</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2767,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked slab bacon, 13-17 slices per pound.</t>
+          <t>Gluten-free applewood-smoked slab bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -2776,7 +2784,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Honey-cured gluten-free wide shingle sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Raw honey-cured wide shingle sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2818,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Honey-cured gluten-free sliced wide shingle bacon, 18-</t>
+          <t>Honey-cured sliced bacon, 18-22 slices per pound, gluten-free, layflat</t>
         </is>
       </c>
     </row>
@@ -2827,7 +2835,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Cooked 0.5‑inch sliced bacon topping</t>
+          <t>Cooked sliced topping bacon, 0.5‑inch thick.</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2852,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Cooked bacon topping, 0.5‑inch pieces</t>
+          <t>Cooked bacon topping, 0.5‑inch slices</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2869,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Fully cooked diced bacon, 1/2‑inch pieces</t>
+          <t>Fully cooked 0.5‑inch diced bacon</t>
         </is>
       </c>
     </row>
@@ -2876,11 +2884,7 @@
           <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 9 13 SLICES PER POUND BACON LAYFLAT C/C 9/13 APL GF</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood-smoked sliced bacon,</t>
-        </is>
-      </c>
+      <c r="C150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2912,7 +2916,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Fully cooked bacon</t>
+          <t>Fully cooked pork bacon.</t>
         </is>
       </c>
     </row>
@@ -2944,11 +2948,7 @@
           <t>HORMEL NATURAL CHOICE UNCURED BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 NAT GF</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>Uncured gluten-free sliced bacon, 13-17 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Canadian-style sliced and quartered bacon with sirloin, 10 slices per ounce</t>
+          <t>Sliced and quartered Canadian-style bacon, 10 slices per ounce.</t>
         </is>
       </c>
     </row>
@@ -2997,7 +2997,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Fully cooked round bacon, 3.5‑inch pieces</t>
+          <t>Fully cooked medium round bacon, 3.5‑inch.</t>
         </is>
       </c>
     </row>
@@ -3044,7 +3044,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Jalapeño sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Jalapeno sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -3059,7 +3059,11 @@
           <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 JAL FZ</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr"/>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Frozen sliced jalapeno bacon, 13-17 slices per pound, lay</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3087,7 +3091,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Raw bacon ends pieces</t>
+          <t>Raw bacon ends, 10 pieces per pound</t>
         </is>
       </c>
     </row>
@@ -3185,7 +3189,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Beef bacon slices</t>
+          <t>Beef bacon slices.</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3266,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Fully cooked applewood-smoked diced bacon pieces</t>
+          <t>Fully cooked diced applewood-smoked bacon pieces</t>
         </is>
       </c>
     </row>
@@ -3296,7 +3300,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Fully cooked sliced smoked bacon</t>
+          <t>Fully cooked sliced smoked bacon.</t>
         </is>
       </c>
     </row>
@@ -3343,7 +3347,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Cooked smoked cured diced bacon, 0.25‑inch pieces</t>
+          <t>Cooked smoked-cured diced bacon, 0.25‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3398,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, smoked.</t>
+          <t>Fully cooked sliced bacon, hickory-smoked</t>
         </is>
       </c>
     </row>
@@ -3465,7 +3469,11 @@
           <t>SYS 1359413 LYFLT BACNSYSCO CLASSIC TEXAS SMKD CTCT INDIVIDUAL SPACED, LAYFLAT BACON (14/18) 1/15 BACON LAYFLAT CC 14/18 TX SMKD</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr"/>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Texas-smoked sliced bacon, 14-18 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -3480,7 +3488,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Frozen Texas-smoked sliced slab bacon, 14-18 slices per pound</t>
+          <t>Frozen Texas-smoked sliced slab bacon, 14-18 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -3514,7 +3522,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 3/4-inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/4‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -3582,7 +3590,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Naturally hardwood-smoked sliced rolled pork belly.</t>
+          <t>Hardwood-smoked sliced rolled pork belly bacon</t>
         </is>
       </c>
     </row>
@@ -3597,7 +3605,11 @@
           <t>SYS 1359405 LYFLT BACNSYSCO CLASSIC TEXAS SMOKED INDIVIDUAL SPACED LAYFLAT BACON 1/15 (18/22) BACON LAYFLAT CC 18/22 TX SMKD</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr"/>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Texas-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -3612,7 +3624,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Applewood-smoked slab bacon</t>
+          <t>Fruitwood- and applewood-smoked slab bacon</t>
         </is>
       </c>
     </row>
@@ -3640,7 +3652,11 @@
           <t>SYS 5886579 FPK 14/18SYSCO CLASSIC GRILL FRESH SLICED BACON 14/18. 2/10 BACON LAYFLAT C/C 14/18 SMK GF</t>
         </is>
       </c>
-      <c r="C198" t="inlineStr"/>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Fresh sliced gluten-free bacon, 14-18 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -3655,7 +3671,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Raw sliced layflat bacon, Texas-smoked</t>
+          <t>Raw Texas-smoked bacon, layflat</t>
         </is>
       </c>
     </row>
@@ -3770,7 +3786,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Fully cooked thick sliced bacon</t>
+          <t>Fully cooked extra‑thick sliced bacon</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3820,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Bacon</t>
+          <t>Bacon, egg, and cheese bowl</t>
         </is>
       </c>
     </row>
@@ -3838,7 +3854,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Fully cooked bacon.</t>
+          <t>Fully cooked bacon</t>
         </is>
       </c>
     </row>
@@ -3923,7 +3939,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Frozen applewood-smoked slab bacon, 10-12 slices per pound.</t>
+          <t>Frozen applewood-smoked slab bacon, 10-12 slices per pound</t>
         </is>
       </c>
     </row>
@@ -3957,7 +3973,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Hickory-smoked bacon, 18-22 slices per pound</t>
+          <t>Hickory-smoked bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -4040,7 +4056,11 @@
           <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED 55253 BACON HRML APPLEWOOD GRIDDLMASTER</t>
         </is>
       </c>
-      <c r="C222" t="inlineStr"/>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Raw wide shingled sliced applewood-smoked bacon, 13-17 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -4055,7 +4075,7 @@
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, wide shingled layout</t>
         </is>
       </c>
     </row>
@@ -4072,7 +4092,7 @@
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Applewood-smoked wide shingled sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4126,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Raw gluten-free applewood-smoked wide shingled sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw gluten-free applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4123,7 +4143,7 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Wide shingled applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4140,7 +4160,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Frozen sugar-cured smoked sliced bacon, 14-18 slices per pound, layflat</t>
+          <t>Frozen sugar-cured smoked bacon, 14-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4174,7 +4194,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Uncured sliced gluten-free bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw uncured gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4206,11 +4226,7 @@
           <t>CHEF PLEASER BACON, 18/22 BACON LAYFLAT C/C 18/22 SMK GF</t>
         </is>
       </c>
-      <c r="C232" t="inlineStr">
-        <is>
-          <t>Gluten-free smoked sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -4225,7 +4241,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw sliced pork bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4242,7 +4258,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Frozen hardwood-smoked sliced bacon, 16-18 slices per pound</t>
+          <t>Frozen sliced bacon, hardwood-smoked, 16-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4274,11 +4290,7 @@
           <t>BW SMOKEY BACON 16-18 BACON LAYFLAT 2 APPLEWOOD SMK</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr">
-        <is>
-          <t>Applewood-smoked bacon, 16-18 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -4327,7 +4339,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Fully cooked thin sliced bacon, 300 slices per case</t>
+          <t>Fully cooked thin sliced bacon</t>
         </is>
       </c>
     </row>
@@ -4344,7 +4356,7 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Fully cooked applewood-smoked bacon</t>
+          <t>Fully cooked applewood-smoked bacon, 300 pieces.</t>
         </is>
       </c>
     </row>
@@ -4389,7 +4401,11 @@
           <t>BACON SLICED HONEY CURED 18-20 CT BACON SHINGLE C/C 18/20 HNY</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr"/>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Honey-cured sliced bacon, 18-20 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -4404,7 +4420,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Honey-cured sliced shingle bacon, 14-16 slices per pound.</t>
+          <t>Honey-cured sliced shingle bacon, 14-16 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4449,11 +4465,7 @@
           <t>BACON SLICED PEPPERED .1875 IN BACON SHINGLE C/C 10/12 PPR</t>
         </is>
       </c>
-      <c r="C247" t="inlineStr">
-        <is>
-          <t>Peppered sliced bacon, 10-12 slices per pound</t>
-        </is>
-      </c>
+      <c r="C247" t="inlineStr"/>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -4513,7 +4525,11 @@
           <t>BACON SLICED CENTER CUT 8-10 CT BACON SHINGLE C/C 8/10 HNY GF</t>
         </is>
       </c>
-      <c r="C251" t="inlineStr"/>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Sliced center-cut gluten-free bacon, 8-10 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -4528,7 +4544,7 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Sliced bacon, 14-16 slices per pound, layflat.</t>
+          <t>Sliced bacon, 14-16 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4545,7 +4561,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Frozen sliced applewood-smoked bacon, 14-16 slices per</t>
+          <t>Frozen sliced applewood-smoked bacon, 14-16 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4562,7 +4578,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Fully cooked thick sliced bacon, 10-12 slices per pound</t>
+          <t>Fully cooked thick sliced bacon, 10-12 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4625,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 12</t>
+          <t>Gluten-free applewood-smoked sliced bacon, 12-14</t>
         </is>
       </c>
     </row>
@@ -4626,7 +4642,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Fully cooked sliced slab bacon</t>
+          <t>Fully cooked sliced slab bacon, regular thickness</t>
         </is>
       </c>
     </row>
@@ -4658,11 +4674,7 @@
           <t>BACON SLICED APPLEWOOD SMOKED LAYOUT 10-14 CT BACON LAYFLAT C/C 10/14 APL GF</t>
         </is>
       </c>
-      <c r="C260" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 10-14 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C260" t="inlineStr"/>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -4735,11 +4747,7 @@
           <t>5886579 CLASSIC GRL/FRSH 14/18 BACON LAYFLAT C/C 14/18 SMK GF</t>
         </is>
       </c>
-      <c r="C265" t="inlineStr">
-        <is>
-          <t>Gluten-free smoked sliced bacon, 14-18 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -4818,7 +4826,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, 9-11 slices per pound, lay</t>
+          <t>Frozen sliced layflat bacon, 9-11 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4833,7 +4841,11 @@
           <t>BACON CUBED COOKED .75X.75 BACON DICED PRCK 3/4</t>
         </is>
       </c>
-      <c r="C271" t="inlineStr"/>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Fully cooked cubed bacon, 3/4‑inch pieces</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -4863,11 +4875,7 @@
           <t>BACON PCS PPRD 3/8</t>
         </is>
       </c>
-      <c r="C273" t="inlineStr">
-        <is>
-          <t>Bacon pieces, 3/8‑inch pieces</t>
-        </is>
-      </c>
+      <c r="C273" t="inlineStr"/>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -4897,11 +4905,7 @@
           <t>OLD SMOKEHOUSE PECANWOOD SMOKED BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 PCN GF</t>
         </is>
       </c>
-      <c r="C275" t="inlineStr">
-        <is>
-          <t>Gluten-free pecanwood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C275" t="inlineStr"/>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -4963,7 +4967,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Frozen hickory-smoked sliced bacon, 14-18 slices per pound, layflat</t>
+          <t>Frozen natural hickory-smoked sliced bacon, 14-18 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4997,7 +5001,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 20-24 slices per pound</t>
+          <t>Fully cooked bacon, 20-24 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5061,7 +5065,7 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Raw gluten-free honey-flavored shingle bacon, 10-12 slices per pound</t>
+          <t>Raw honey-glazed center cut shingle bacon</t>
         </is>
       </c>
     </row>
@@ -5078,7 +5082,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 16-18 slices per pound</t>
+          <t>Applewood-smoked sliced bacon, 16-18 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5095,7 +5099,7 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 13-17 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5146,7 +5150,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5163,7 +5167,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5197,7 +5201,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Fresh sliced gluten-free bacon, 18-22 slices per pound</t>
+          <t>Fresh gluten-free sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5246,11 +5250,7 @@
           <t>FARMLAND HEAT N EAT SL BACON BACON PORK 150 CT SLCD L</t>
         </is>
       </c>
-      <c r="C296" t="inlineStr">
-        <is>
-          <t>Sliced pork bacon, 150 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -5359,7 +5359,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Sliced pork bacon, 18-22 slices per pound.</t>
+          <t>Sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5374,11 +5374,7 @@
           <t>BCN,PCI,2/5 ,1/2 ,TPG,MCRW BACON TOPPING CKD 1/2 IN</t>
         </is>
       </c>
-      <c r="C304" t="inlineStr">
-        <is>
-          <t>Fully cooked bacon topping, 1/2‑inch pieces</t>
-        </is>
-      </c>
+      <c r="C304" t="inlineStr"/>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -5440,7 +5436,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 14-17 slices per pound, layflat</t>
+          <t>Gluten-free applewood-smoked sliced bacon,</t>
         </is>
       </c>
     </row>
@@ -5470,7 +5466,7 @@
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Frozen real pork bacon bits, fine diced, 2/5‑inch pieces</t>
+          <t>Frozen bacon bits, fine diced, 2/5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5483,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Fully cooked fine bacon bits, 2/5‑inch pieces</t>
+          <t>Fully cooked fine bacon bits, 2/5-inch pieces</t>
         </is>
       </c>
     </row>
@@ -5502,11 +5498,7 @@
           <t>BCN,PL,FL,BITS,FINE,2/5 BACON BIT CKD 3/16IN</t>
         </is>
       </c>
-      <c r="C312" t="inlineStr">
-        <is>
-          <t>Fully cooked bacon bits, 3/16‑inch pieces</t>
-        </is>
-      </c>
+      <c r="C312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -5521,7 +5513,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Raw diced bacon, 1/2-inch pieces</t>
+          <t>Ready-to-cook diced bacon ends and pieces</t>
         </is>
       </c>
     </row>
@@ -5570,7 +5562,11 @@
           <t>BCN,GC,APLWD,SMKD,2/5 ,TPG BACON TOPPING APPLEWOOD SMOKED FC 3/8 BACON TOPPING FULLY CKD</t>
         </is>
       </c>
-      <c r="C316" t="inlineStr"/>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Fully</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -5650,7 +5646,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Frozen smoked sliced bacon, 14-18 slices per pound</t>
+          <t>Frozen sliced bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5695,7 +5691,11 @@
           <t>BCN,FL,SMD,1/15 ,18-22SL/ ,FZ BACON SLICED 18-22 LO</t>
         </is>
       </c>
-      <c r="C325" t="inlineStr"/>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Frozen smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -5721,7 +5721,11 @@
           <t>BCN,FL,SMD,1/15 ,18-22SL/ ,FZ BACON 18/22 CT LAYOUT SINGLE SLICED GLUTEN-FREE BACON LAID-OUT 18/22 SLVR</t>
         </is>
       </c>
-      <c r="C327" t="inlineStr"/>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Frozen gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -5734,7 +5738,11 @@
           <t>BACN,SS,SM,22/26,15 ,Z BACON LAYOUT SLI 22/26 FRZN</t>
         </is>
       </c>
-      <c r="C328" t="inlineStr"/>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Frozen sliced bacon, 22-26 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -5779,7 +5787,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Gluten-free Northwest-smoked sliced bacon, 10-14 slices per pound</t>
+          <t>Gluten-free sliced bacon, 10-14 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5796,7 +5804,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Gluten-free apple-cider smoked sliced bacon, 18-22 slices per</t>
+          <t>Apple-cider cured sliced bacon, 18-22 slices per pound, gluten-free</t>
         </is>
       </c>
     </row>
@@ -5906,11 +5914,7 @@
           <t>BACN,SS,APLWD SMKD,SM,18/22,GF,15 ,Z BACON SSL APPLWD SMKD 18-22CT</t>
         </is>
       </c>
-      <c r="C340" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 18-22 slices per pound</t>
-        </is>
-      </c>
+      <c r="C340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -5940,7 +5944,11 @@
           <t>BACN,SS,UNCURED,SM,13/17,GF,15 BACON SINGLE SLI UNCURE 13/17</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr"/>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Uncured sliced bacon, 13-17 slices per pound, gluten-free.</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -5972,7 +5980,7 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Fully cooked all‑natural sliced bacon, 13‑17 slices per pound.</t>
+          <t>Fully cooked all-natural sliced bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -6040,7 +6048,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits.</t>
+          <t>Fully cooked bacon bits</t>
         </is>
       </c>
     </row>
@@ -6057,7 +6065,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Fully cooked natural bacon topping</t>
+          <t>Fully cooked bacon topping.</t>
         </is>
       </c>
     </row>
@@ -6074,7 +6082,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Applewood-smoked Canadian boneless loin bacon</t>
+          <t>Applewood-smoked boneless Canadian loin bacon</t>
         </is>
       </c>
     </row>
@@ -6091,7 +6099,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Frozen sliced hickory-smoked bacon, 18-22 slices per pound, layflat</t>
+          <t>Frozen hickory-smoked sliced bacon, 18-22 slices per pound, layflat.</t>
         </is>
       </c>
     </row>
@@ -6142,7 +6150,7 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, hickory-smoked, 22-26 slices per pound, layflat</t>
+          <t>Frozen hickory-smoked sliced bacon, 22-26 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -6259,7 +6267,11 @@
           <t>HORMEL REGULAR COOKED ALL NATURAL 0 375 INCH BACON TOPPING BACON TOPPING NAT REG CKD 3/8</t>
         </is>
       </c>
-      <c r="C361" t="inlineStr"/>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Cooked bacon topping, 3/8-inch slices</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -6274,7 +6286,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 3/8-inch pieces</t>
+          <t>Fully cooked bacon topping, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -6308,7 +6320,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 13-17 slices per pound.</t>
+          <t>Fully cooked bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add <think> tag stripping to support reasoning models
Issue: Qwen and other reasoning models output <think>reasoning</think>answer
Solution: RawTextParser now strips <think>...</think> tags using regex
Now supports models that show internal reasoning without breaking output parsing

Supports: Qwen, o1, and other reasoning models with thinking tags
</commit_message>
<xml_diff>
--- a/tmp/ground_truth_cleaned.xlsx
+++ b/tmp/ground_truth_cleaned.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Frozen sugar-cured half slab bacon</t>
+          <t>Frozen sugar-cured half-slab bacon</t>
         </is>
       </c>
     </row>
@@ -509,7 +509,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Applewood-smoked half slab bacon, unsliced</t>
+          <t>Raw applewood-smoked half slab bacon, unsliced</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 3/8‑inch pieces</t>
+          <t>Fully cooked gluten-free gas-flushed bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Fully cooked gluten‑free bacon bits, 3/4‑inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/4‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fully cooked diced bacon bits, 3/8-inch pieces</t>
+          <t>Fully cooked cubed bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Fully cooked sliced applewood-sm</t>
+          <t>Fully</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced pork bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 3/4‑inch pieces</t>
+          <t>Fully cooked flaked bacon topping, 3/4‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1050,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Frozen applewood-smoked sliced bacon, 18-22 slices per pound</t>
+          <t>Frozen sliced applewood-smoked bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -1246,7 +1246,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Fully cooked smoked bacon pieces, 3/8‑inch pieces.</t>
+          <t>Fully cooked smoked diced bacon, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1261,11 @@
           <t>NT AWS BACN FPK 14/18, GF BACON LAYFLAT 14/18 APPL GF</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr"/>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Applewood-smoked</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1293,7 +1297,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Fully cooked bacon pieces, 3/8‑inch pieces</t>
+          <t>Fully cooked bacon pieces, 3/8‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -1327,7 +1331,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 192 slices.</t>
+          <t>Fully cooked sliced bacon, 192 pieces</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1348,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Center-cut sliced smoked bacon, 18-22 slices per pound, layflat</t>
+          <t>Center cut sliced smoked bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1361,7 +1365,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, gluten-free, layflat</t>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1397,11 @@
           <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED GCF BACON SLI APLWD 13/17CT PR12</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr"/>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Applewood-smoked sliced bacon, 13-17 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1408,7 +1416,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Uncured gluten-free sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Uncured sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1423,11 +1431,7 @@
           <t>OLD SMOKEHOUSE PECANWOOD SMOKED BACON 9 13 SLICES PER POUND GCF BACON LAYFLAT PCN CC 9/13 PR12</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Pecanwood-smoked sliced bacon, 9-13 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1440,11 +1444,7 @@
           <t>HORMEL LAYOUT BACON 18 22 SLICES PER POUND GCF BACON LAYFLAT CC 18/22 GF PR12</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Frozen applewood-smoked sliced bacon, 10-12 slices per pound</t>
+          <t>Frozen sliced applewood-smoked bacon, 10-12 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Fully cooked bacon pieces, 1/2‑inch size.</t>
+          <t>Fully cooked bacon pieces, 1/2‑inch size</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Applewood-smoked cubed bacon, 0.5 × 0.5‑inch pieces</t>
+          <t>Applewood-smoked diced bacon, 0.5‑inch cubes.</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 3/4-inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/4‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 0.5-inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 1/2-inch pieces</t>
         </is>
       </c>
     </row>
@@ -1661,7 +1661,11 @@
           <t>BACON APPLEWOOD SMOKED LAYOUT 18-22 CT BACON L/O 14-18CT CC APPLWD SMKD</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1693,7 +1697,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Raw sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1855,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 14-18 slices per pound, layflat</t>
+          <t>Gluten-free applewood-smoked sliced</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1906,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Fully cooked diced bacon topping, 3/8‑inch pieces</t>
+          <t>Fully cooked sliced bacon, 3/8‑inch slices</t>
         </is>
       </c>
     </row>
@@ -1919,7 +1923,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 3/8-inch pieces</t>
+          <t>Fully cooked bacon topping, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -1936,7 +1940,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Fully cooked diced bacon topping, .38‑inch pieces.</t>
+          <t>Fully cooked sliced bacon, 0.375‑inch thickness.</t>
         </is>
       </c>
     </row>
@@ -1953,7 +1957,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 300 slices per case</t>
+          <t>Fully cooked sliced bacon, 300 slices per case.</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2208,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Canadian-style bacon sticks</t>
+          <t>Canadian-style whole bacon sticks</t>
         </is>
       </c>
     </row>
@@ -2219,7 +2223,11 @@
           <t>HORMEL COUNTRY BRAND BACON 18 22 SLICES PER POUND WIDE SHINGLE BACON LAYOUT 18/22 SMKD</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2251,7 +2259,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits, 3/8-inch pieces</t>
+          <t>Fully cooked bacon bits, 3/8‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -2285,7 +2293,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Cooked diced bacon, 1/4‑inch pieces.</t>
+          <t>Fully</t>
         </is>
       </c>
     </row>
@@ -2302,7 +2310,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Thick-sliced bacon, 1/2-inch slices.</t>
+          <t>Thick sliced bacon, 1/2‑inch slices.</t>
         </is>
       </c>
     </row>
@@ -2458,11 +2466,7 @@
           <t>BACON L/O 2 FZ 15 P/L BACON L/O 2 FZ CHEF S CHC BACON 2 LAYOUT FROZEN</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>Frozen sliced bacon</t>
-        </is>
-      </c>
+      <c r="C124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2507,7 +2511,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Fully cooked thin sliced bacon and fully cooked medium sliced bacon.</t>
+          <t>Fully cooked thin sliced bacon, fully cooked medium sliced bacon.</t>
         </is>
       </c>
     </row>
@@ -2524,7 +2528,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Fully cooked medium-sliced and thin-sliced bacon</t>
+          <t>Fully cooked medium-sliced and thin-sliced bacon.</t>
         </is>
       </c>
     </row>
@@ -2603,11 +2607,7 @@
           <t>8 SYS SLCD SLAB HON BACN 14/16 15 LB BACON SHINGLE 14/16 HNY PR12</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>Honey-glazed slab bacon, 14-16 slices per</t>
-        </is>
-      </c>
+      <c r="C133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2654,7 +2654,11 @@
           <t>BACON SMKD ENDS RNDM</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr"/>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Smoked bacon</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -2720,7 +2724,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Maple pepper sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2750,7 +2754,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Water-added Canadian-style bacon with sirloin, half‑sticky.</t>
+          <t>Water-added half-stacked Canadian-style bacon with sirloin.</t>
         </is>
       </c>
     </row>
@@ -2767,7 +2771,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked slab bacon, 13-17 slices per pound</t>
+          <t>Gluten-free applewood-smoked slab bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2788,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Raw honey-cured wide shingle sliced bacon, 13-17 slices per pound, layflat</t>
+          <t>Raw honey-cured gluten-free sliced bacon, 13-17 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -2818,7 +2822,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Honey-cured sliced bacon, 18-22 slices per pound, gluten-free, layflat</t>
+          <t>Honey-cured sliced bacon, 18-22 slices per pound, layflat, gluten-free.</t>
         </is>
       </c>
     </row>
@@ -2835,7 +2839,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Cooked sliced topping bacon, 0.5‑inch thick.</t>
+          <t>Cooked sliced bacon, 0.5‑inch thickness, topping</t>
         </is>
       </c>
     </row>
@@ -2850,11 +2854,7 @@
           <t>HORMEL REGULAR COOK 0 5 INCH BACON TOPPING BACON TOPPING REG COOKED 1/2</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>Cooked bacon topping, 0.5‑inch slices</t>
-        </is>
-      </c>
+      <c r="C148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -2869,7 +2869,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Fully cooked 0.5‑inch diced bacon</t>
+          <t>Fully cooked diced bacon, 1/2‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2884,11 @@
           <t>OLD SMOKEHOUSE APPLEWOOD SMOKED BACON 9 13 SLICES PER POUND BACON LAYFLAT C/C 9/13 APL GF</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr"/>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Applewood-smoked sliced bacon, 9-13 slices per pound, gluten-free, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -2916,7 +2920,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Fully cooked pork bacon.</t>
+          <t>Fully cooked bacon.</t>
         </is>
       </c>
     </row>
@@ -2963,7 +2967,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Sliced and quartered Canadian-style bacon, 10 slices per ounce.</t>
+          <t>Sliced and quartered bacon, 10 slices per ounce.</t>
         </is>
       </c>
     </row>
@@ -3059,11 +3063,7 @@
           <t>HORMEL LAYOUT JALAPENO BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 JAL FZ</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>Frozen sliced jalapeno bacon, 13-17 slices per pound, lay</t>
-        </is>
-      </c>
+      <c r="C161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Raw bacon ends, 10 pieces per pound</t>
+          <t>Raw bacon ends, 10 pieces.</t>
         </is>
       </c>
     </row>
@@ -3189,7 +3189,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Beef bacon slices.</t>
+          <t>Beef bacon sliced</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 1‑inch pieces</t>
+          <t>Fully cooked sliced bacon topping, 1‑inch slices</t>
         </is>
       </c>
     </row>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Fully cooked sliced smoked bacon.</t>
+          <t>Fully cooked sliced smoked bacon</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Cooked smoked-cured diced bacon, 0.25‑inch pieces.</t>
+          <t>Cooked smoked cured diced bacon, 0.25‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -3396,11 +3396,7 @@
           <t>5756893 CLASSIC PRCKD BCN HSMO BACON PRECOOKED HEARTY SMOKED SLICED BACON PRECOOKED REG SLI HRTYSM</t>
         </is>
       </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>Fully cooked sliced bacon, hickory-smoked</t>
-        </is>
-      </c>
+      <c r="C182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -3426,7 +3422,11 @@
           <t>FRZ 1005842 CLASSIC LF 18/22 BACON 18/22 CT C/C SMOKED LAYFLAT BACON LAYFLAT C/C 18/22 SMOKED</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr"/>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Frozen smoked sliced bacon, 18-22 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -3439,7 +3439,11 @@
           <t>SYS 5321427 SLAB BACNTEXAS SMOKED CENTER CUT SLICED SLAB BACON (18/22) 1/15 BACON SLAB C/C 18/22 TX SMKD</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr"/>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Center-cut sliced slab bacon, Texas-smoked, 18-22 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -3469,11 +3473,7 @@
           <t>SYS 1359413 LYFLT BACNSYSCO CLASSIC TEXAS SMKD CTCT INDIVIDUAL SPACED, LAYFLAT BACON (14/18) 1/15 BACON LAYFLAT CC 14/18 TX SMKD</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>Texas-smoked sliced bacon, 14-18 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -3488,7 +3488,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Frozen Texas-smoked sliced slab bacon, 14-18 slices per pound.</t>
+          <t>Frozen Texas-smoked sliced slab bacon, 14-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Fully cooked gluten-free bacon bits, 3/4‑inch pieces</t>
+          <t>Fully cooked gluten-free bacon bits, 3/4-inch pieces</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Hardwood-smoked sliced rolled pork belly bacon</t>
+          <t>Naturally hardwood-smoked sliced rolled bacon.</t>
         </is>
       </c>
     </row>
@@ -3605,11 +3605,7 @@
           <t>SYS 1359405 LYFLT BACNSYSCO CLASSIC TEXAS SMOKED INDIVIDUAL SPACED LAYFLAT BACON 1/15 (18/22) BACON LAYFLAT CC 18/22 TX SMKD</t>
         </is>
       </c>
-      <c r="C195" t="inlineStr">
-        <is>
-          <t>Texas-smoked sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -3624,7 +3620,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Fruitwood- and applewood-smoked slab bacon</t>
+          <t>Applewood-smoked slab bacon</t>
         </is>
       </c>
     </row>
@@ -3652,11 +3648,7 @@
           <t>SYS 5886579 FPK 14/18SYSCO CLASSIC GRILL FRESH SLICED BACON 14/18. 2/10 BACON LAYFLAT C/C 14/18 SMK GF</t>
         </is>
       </c>
-      <c r="C198" t="inlineStr">
-        <is>
-          <t>Fresh sliced gluten-free bacon, 14-18 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -3671,7 +3663,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Raw Texas-smoked bacon, layflat</t>
+          <t>Raw Texas-smoked sliced layflat bacon</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3778,7 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Fully cooked extra‑thick sliced bacon</t>
+          <t>Fully cooked thick sliced bacon</t>
         </is>
       </c>
     </row>
@@ -3820,7 +3812,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Bacon, egg, and cheese bowl</t>
+          <t>Bacon</t>
         </is>
       </c>
     </row>
@@ -3854,7 +3846,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Fully cooked bacon</t>
+          <t>Fully cooked bacon, 300 slices.</t>
         </is>
       </c>
     </row>
@@ -3956,7 +3948,7 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Sweet bacon.</t>
+          <t>Sweet bacon</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4016,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Fully cooked bacon crumbles.</t>
+          <t>Fully cooked bacon crumbles</t>
         </is>
       </c>
     </row>
@@ -4058,7 +4050,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Raw wide shingled sliced applewood-smoked bacon, 13-17 slices per pound</t>
+          <t>Raw wide shingled sliced applewood-smoked bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -4073,11 +4065,7 @@
           <t>HORMEL GRIDDLEMASTER APPLEWOOD BACON 13 17 SLICES PER POUND WIDE SHINGLED BACON LAYOUT APPLEWOOD 13/17</t>
         </is>
       </c>
-      <c r="C223" t="inlineStr">
-        <is>
-          <t>Applewood-smoked sliced bacon, 13-17 slices per pound, wide shingled layout</t>
-        </is>
-      </c>
+      <c r="C223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -4126,7 +4114,7 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Raw gluten-free applewood-smoked sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Raw gluten-free sliced applewood-smoked bacon, 18-22 slices per pound, layflat.</t>
         </is>
       </c>
     </row>
@@ -4175,11 +4163,7 @@
           <t>HORMEL NATURAL CHOICE UNCURED BACON 18 22 SLICES PER POUND BACON LAYFLAT C/C 18/22 NTGF F</t>
         </is>
       </c>
-      <c r="C229" t="inlineStr">
-        <is>
-          <t>Raw uncured sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -4194,7 +4178,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Raw uncured gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
+          <t>Uncured gluten-free sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4210,11 @@
           <t>CHEF PLEASER BACON, 18/22 BACON LAYFLAT C/C 18/22 SMK GF</t>
         </is>
       </c>
-      <c r="C232" t="inlineStr"/>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Gluten-free</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -4241,7 +4229,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Raw sliced pork bacon, 18-22 slices per pound, layflat</t>
+          <t>Sliced bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4258,7 +4246,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, hardwood-smoked, 16-18 slices per pound</t>
+          <t>Frozen hardwood-smoked sliced bacon, 16-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4508,11 +4496,7 @@
           <t>BACON SLICED SUGAR CURED 14-16 CT BACON SHINGLE C/C 14/16 SGR</t>
         </is>
       </c>
-      <c r="C250" t="inlineStr">
-        <is>
-          <t>Sugar-cured sliced bacon, 14-16 slices per pound</t>
-        </is>
-      </c>
+      <c r="C250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -4525,11 +4509,7 @@
           <t>BACON SLICED CENTER CUT 8-10 CT BACON SHINGLE C/C 8/10 HNY GF</t>
         </is>
       </c>
-      <c r="C251" t="inlineStr">
-        <is>
-          <t>Sliced center-cut gluten-free bacon, 8-10 slices per pound</t>
-        </is>
-      </c>
+      <c r="C251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -4561,7 +4541,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Frozen sliced applewood-smoked bacon, 14-16 slices per pound, layflat</t>
+          <t>Frozen sliced applewood-smoked bacon, 14-16 slices</t>
         </is>
       </c>
     </row>
@@ -4608,7 +4588,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Hickory-smoked sliced bacon, 14-18 slices per pound</t>
+          <t>Hickory-smoked sliced bacon, 14-18 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -4625,7 +4605,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon, 12-14</t>
+          <t>Gluten-free applewood-smoked sliced bacon, 12</t>
         </is>
       </c>
     </row>
@@ -4642,7 +4622,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Fully cooked sliced slab bacon, regular thickness</t>
+          <t>Pre-cooked sliced slab bacon, regular thickness</t>
         </is>
       </c>
     </row>
@@ -4687,7 +4667,11 @@
           <t>BACON CHIP CUBED REGULAR .375X.375 BACON PORK REAL DCD .38</t>
         </is>
       </c>
-      <c r="C261" t="inlineStr"/>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Cubed bacon, 0.375 × 0.375‑inch pieces.</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -4715,7 +4699,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 32-36 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 32-36 slices per pound</t>
         </is>
       </c>
     </row>
@@ -4747,7 +4731,11 @@
           <t>5886579 CLASSIC GRL/FRSH 14/18 BACON LAYFLAT C/C 14/18 SMK GF</t>
         </is>
       </c>
-      <c r="C265" t="inlineStr"/>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Gluten-free smoked sliced bacon, 14-18 slices per pound, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -4826,7 +4814,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Frozen sliced layflat bacon, 9-11 slices per pound</t>
+          <t>Frozen sliced bacon, 9-11 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -4843,7 +4831,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Fully cooked cubed bacon, 3/4‑inch pieces</t>
+          <t>Fully cooked diced bacon, 3/4-inch pieces</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4863,11 @@
           <t>BACON PCS PPRD 3/8</t>
         </is>
       </c>
-      <c r="C273" t="inlineStr"/>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>Bacon pieces, 3/8‑inch size.</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -4890,7 +4882,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced slab bacon, 1/4‑inch slices</t>
+          <t>Applewood-smoked sliced slab bacon, 1/4‑inch thickness.</t>
         </is>
       </c>
     </row>
@@ -4905,7 +4897,11 @@
           <t>OLD SMOKEHOUSE PECANWOOD SMOKED BACON 13 17 SLICES PER POUND BACON LAYFLAT C/C 13/17 PCN GF</t>
         </is>
       </c>
-      <c r="C275" t="inlineStr"/>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Pecanwood-smoked sliced bacon, 13-17 slices per pound, gluten-free, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -4984,7 +4980,7 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Fully cooked smoked sliced bacon, 20-24 slices per pound</t>
+          <t>Fully cooked smoked sliced bacon, 20-24 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5063,11 +5059,7 @@
           <t>SYS 0855195 HON 10/12SYSCO CLASSIC BACON CENTER CUT SHINGLE HONEY 10/12 CT 1/15 LB BACON SHINGLE C/C 10/12 HNY GF</t>
         </is>
       </c>
-      <c r="C285" t="inlineStr">
-        <is>
-          <t>Raw honey-glazed center cut shingle bacon</t>
-        </is>
-      </c>
+      <c r="C285" t="inlineStr"/>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -5082,7 +5074,7 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Applewood-smoked sliced bacon, 16-18 slices per pound.</t>
+          <t>Applewood-smoked sliced bacon, 16-18 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5150,7 +5142,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5184,7 +5176,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 18-22 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5201,7 +5193,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Fresh gluten-free sliced bacon, 18-22 slices per pound.</t>
+          <t>Fresh sliced gluten-free bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5250,7 +5242,11 @@
           <t>FARMLAND HEAT N EAT SL BACON BACON PORK 150 CT SLCD L</t>
         </is>
       </c>
-      <c r="C296" t="inlineStr"/>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Sliced bacon, layflat</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -5282,7 +5278,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, heat-and-eat</t>
+          <t>Fully cooked sliced bacon</t>
         </is>
       </c>
     </row>
@@ -5297,11 +5293,7 @@
           <t>BCN,FL,BM,2/1.25 ,300C,FLCK,SLCD BACON LAYFLAT PRCK</t>
         </is>
       </c>
-      <c r="C299" t="inlineStr">
-        <is>
-          <t>Fully cooked sliced bacon, layflat</t>
-        </is>
-      </c>
+      <c r="C299" t="inlineStr"/>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -5314,7 +5306,11 @@
           <t>BCN,FL,BM,2/1.25 ,300C,FLCK,SLCD BACON FULLY CKD HEAT N SERVE</t>
         </is>
       </c>
-      <c r="C300" t="inlineStr"/>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>Fully cooked sliced bacon</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -5359,7 +5355,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Sliced bacon, 18-22 slices per pound.</t>
+          <t>Sliced pork bacon, 18-22 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5436,7 +5432,7 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Gluten-free applewood-smoked sliced bacon,</t>
+          <t>Gluten-free applewood-smoked sliced bacon, 14-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5464,11 +5460,7 @@
           <t>BCN,PL,FL,BITS,FINE,2/5 BACON PORK REAL CHIP DCD</t>
         </is>
       </c>
-      <c r="C310" t="inlineStr">
-        <is>
-          <t>Frozen bacon bits, fine diced, 2/5‑inch pieces</t>
-        </is>
-      </c>
+      <c r="C310" t="inlineStr"/>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -5483,7 +5475,7 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Fully cooked fine bacon bits, 2/5-inch pieces</t>
+          <t>Fully cooked fine bacon bits, 2/5‑inch pieces</t>
         </is>
       </c>
     </row>
@@ -5498,7 +5490,11 @@
           <t>BCN,PL,FL,BITS,FINE,2/5 BACON BIT CKD 3/16IN</t>
         </is>
       </c>
-      <c r="C312" t="inlineStr"/>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Fully cooked bacon bits, 3/16‑inch pieces</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -5513,7 +5509,7 @@
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Ready-to-cook diced bacon ends and pieces</t>
+          <t>Raw diced bacon, 1/2-inch pieces</t>
         </is>
       </c>
     </row>
@@ -5530,7 +5526,7 @@
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Frozen ready-to-cook diced bacon, 2/5‑inch pieces</t>
+          <t>Frozen ready-to-cook diced bacon, 2/5‑inch pieces.</t>
         </is>
       </c>
     </row>
@@ -5562,11 +5558,7 @@
           <t>BCN,GC,APLWD,SMKD,2/5 ,TPG BACON TOPPING APPLEWOOD SMOKED FC 3/8 BACON TOPPING FULLY CKD</t>
         </is>
       </c>
-      <c r="C316" t="inlineStr">
-        <is>
-          <t>Fully</t>
-        </is>
-      </c>
+      <c r="C316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -5646,7 +5638,7 @@
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Frozen sliced bacon, 14-18 slices per pound</t>
+          <t>Frozen sliced bacon, 14</t>
         </is>
       </c>
     </row>
@@ -5691,11 +5683,7 @@
           <t>BCN,FL,SMD,1/15 ,18-22SL/ ,FZ BACON SLICED 18-22 LO</t>
         </is>
       </c>
-      <c r="C325" t="inlineStr">
-        <is>
-          <t>Frozen smoked sliced bacon, 18-22 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -5738,11 +5726,7 @@
           <t>BACN,SS,SM,22/26,15 ,Z BACON LAYOUT SLI 22/26 FRZN</t>
         </is>
       </c>
-      <c r="C328" t="inlineStr">
-        <is>
-          <t>Frozen sliced bacon, 22-26 slices per pound, layflat</t>
-        </is>
-      </c>
+      <c r="C328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -5785,11 +5769,7 @@
           <t>BACN,HRI,NW-SM,10/14,GF,15 BACON 10/14 CT HRI NORTHWEST GLUTEN-FREE</t>
         </is>
       </c>
-      <c r="C331" t="inlineStr">
-        <is>
-          <t>Gluten-free sliced bacon, 10-14 slices per pound</t>
-        </is>
-      </c>
+      <c r="C331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -5804,7 +5784,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Apple-cider cured sliced bacon, 18-22 slices per pound, gluten-free</t>
+          <t>Gluten-free apple-cider smoked sliced bacon, 18-22 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -5888,7 +5868,11 @@
           <t>BACN,SS,APLWD SMKD,SM,14/18,GF,15 ,Z BACON APPLEWOOD SSL 14/18</t>
         </is>
       </c>
-      <c r="C338" t="inlineStr"/>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Gluten-free applewood-smoked sliced bacon, 14-18 slices per pound.</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -5914,7 +5898,11 @@
           <t>BACN,SS,APLWD SMKD,SM,18/22,GF,15 ,Z BACON SSL APPLWD SMKD 18-22CT</t>
         </is>
       </c>
-      <c r="C340" t="inlineStr"/>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Applewood-smoked sliced gluten-free bacon, 18-22 slices per pound</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -5927,11 +5915,7 @@
           <t>BACN,SS,APLWD SMKD,SM,18/22,GF,15 ,Z BACON LAYFLAT CC 18/22 APL SMK</t>
         </is>
       </c>
-      <c r="C341" t="inlineStr">
-        <is>
-          <t>Gluten-free applewood</t>
-        </is>
-      </c>
+      <c r="C341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -5946,7 +5930,7 @@
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Uncured sliced bacon, 13-17 slices per pound, gluten-free.</t>
+          <t>Raw uncured gluten-free smoked sliced bacon, 13-17 slices per pound</t>
         </is>
       </c>
     </row>
@@ -5980,7 +5964,7 @@
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Fully cooked all-natural sliced bacon, 13-17 slices per pound.</t>
+          <t>Fully cooked all‑natural sliced bacon, 13‑17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -6048,7 +6032,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>Fully cooked bacon bits</t>
+          <t>Fully cooked bacon topping bits</t>
         </is>
       </c>
     </row>
@@ -6065,7 +6049,7 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping.</t>
+          <t>Cooked bacon topping</t>
         </is>
       </c>
     </row>
@@ -6082,7 +6066,7 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>Applewood-smoked boneless Canadian loin bacon</t>
+          <t>Boneless Canadian loin bacon, applewood‑smoked</t>
         </is>
       </c>
     </row>
@@ -6099,7 +6083,7 @@
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Frozen hickory-smoked sliced bacon, 18-22 slices per pound, layflat.</t>
+          <t>Frozen sliced hickory-smoked bacon, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -6116,7 +6100,7 @@
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Fresh sliced smoked bacon, 18-22 slices per pound,</t>
+          <t>Fresh sliced bacon, smoked, 18-22 slices per pound, layflat</t>
         </is>
       </c>
     </row>
@@ -6252,7 +6236,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 13-17 slices per pound</t>
+          <t>Fully cooked sliced bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -6267,11 +6251,7 @@
           <t>HORMEL REGULAR COOKED ALL NATURAL 0 375 INCH BACON TOPPING BACON TOPPING NAT REG CKD 3/8</t>
         </is>
       </c>
-      <c r="C361" t="inlineStr">
-        <is>
-          <t>Cooked bacon topping, 3/8-inch slices</t>
-        </is>
-      </c>
+      <c r="C361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -6286,7 +6266,7 @@
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Fully cooked bacon topping, 3/8‑inch pieces</t>
+          <t>Fully cooked bacon topping, 3/8-inch pieces</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6300,7 @@
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Fully cooked bacon, 13-17 slices per pound</t>
+          <t>Fully cooked sliced bacon, 13-17 slices per pound.</t>
         </is>
       </c>
     </row>
@@ -6337,7 +6317,7 @@
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>Fully cooked sliced bacon, 9-13 slices per pound.</t>
+          <t>Fully cooked sliced bacon, 9-13 slices per pound</t>
         </is>
       </c>
     </row>

</xml_diff>